<commit_message>
daily auto-refresh 2026-09-16 13:01
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L343"/>
+  <dimension ref="A1:L345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,12 +434,12 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Turmeric Curcumin</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Lemon Ginger</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5251,10 +5251,10 @@
         <v>2</v>
       </c>
       <c r="D121" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E121" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -5291,10 +5291,10 @@
         <v>1</v>
       </c>
       <c r="D122" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E122" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F122" t="n">
         <v>0</v>
@@ -5531,10 +5531,10 @@
         <v>34</v>
       </c>
       <c r="D128" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E128" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F128" t="n">
         <v>0</v>
@@ -5571,10 +5571,10 @@
         <v>9</v>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E129" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F129" t="n">
         <v>0</v>
@@ -5611,10 +5611,10 @@
         <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E130" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F130" t="n">
         <v>0</v>
@@ -5691,10 +5691,10 @@
         <v>2</v>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E132" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F132" t="n">
         <v>0</v>
@@ -6051,10 +6051,10 @@
         <v>13</v>
       </c>
       <c r="D141" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E141" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F141" t="n">
         <v>0</v>
@@ -6091,10 +6091,10 @@
         <v>3</v>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F142" t="n">
         <v>0</v>
@@ -6131,10 +6131,10 @@
         <v>7</v>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E143" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F143" t="n">
         <v>0</v>
@@ -6171,10 +6171,10 @@
         <v>7</v>
       </c>
       <c r="D144" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E144" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F144" t="n">
         <v>0</v>
@@ -6211,10 +6211,10 @@
         <v>2</v>
       </c>
       <c r="D145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F145" t="n">
         <v>0</v>
@@ -6251,10 +6251,10 @@
         <v>1</v>
       </c>
       <c r="D146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E146" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F146" t="n">
         <v>0</v>
@@ -6331,10 +6331,10 @@
         <v>8</v>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E148" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -6371,10 +6371,10 @@
         <v>4</v>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E149" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F149" t="n">
         <v>0</v>
@@ -6451,10 +6451,10 @@
         <v>0</v>
       </c>
       <c r="D151" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E151" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>
@@ -6491,10 +6491,10 @@
         <v>0</v>
       </c>
       <c r="D152" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E152" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F152" t="n">
         <v>0</v>
@@ -6531,10 +6531,10 @@
         <v>0</v>
       </c>
       <c r="D153" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E153" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F153" t="n">
         <v>0</v>
@@ -6571,10 +6571,10 @@
         <v>0</v>
       </c>
       <c r="D154" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="E154" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F154" t="n">
         <v>0</v>
@@ -6611,10 +6611,10 @@
         <v>1</v>
       </c>
       <c r="D155" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E155" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F155" t="n">
         <v>0</v>
@@ -6651,10 +6651,10 @@
         <v>0</v>
       </c>
       <c r="D156" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E156" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
@@ -6731,10 +6731,10 @@
         <v>0</v>
       </c>
       <c r="D158" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E158" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F158" t="n">
         <v>0</v>
@@ -6771,10 +6771,10 @@
         <v>2</v>
       </c>
       <c r="D159" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E159" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -6811,10 +6811,10 @@
         <v>1</v>
       </c>
       <c r="D160" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E160" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F160" t="n">
         <v>0</v>
@@ -6851,10 +6851,10 @@
         <v>5</v>
       </c>
       <c r="D161" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E161" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
@@ -6891,10 +6891,10 @@
         <v>5</v>
       </c>
       <c r="D162" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E162" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F162" t="n">
         <v>0</v>
@@ -6931,10 +6931,10 @@
         <v>8</v>
       </c>
       <c r="D163" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E163" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F163" t="n">
         <v>0</v>
@@ -6971,10 +6971,10 @@
         <v>2</v>
       </c>
       <c r="D164" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E164" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F164" t="n">
         <v>0</v>
@@ -7011,10 +7011,10 @@
         <v>5</v>
       </c>
       <c r="D165" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E165" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F165" t="n">
         <v>0</v>
@@ -7051,10 +7051,10 @@
         <v>3</v>
       </c>
       <c r="D166" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E166" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -7091,10 +7091,10 @@
         <v>5</v>
       </c>
       <c r="D167" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E167" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F167" t="n">
         <v>0</v>
@@ -7131,10 +7131,10 @@
         <v>1</v>
       </c>
       <c r="D168" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E168" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F168" t="n">
         <v>0</v>
@@ -7171,10 +7171,10 @@
         <v>1</v>
       </c>
       <c r="D169" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E169" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F169" t="n">
         <v>0</v>
@@ -7211,10 +7211,10 @@
         <v>2</v>
       </c>
       <c r="D170" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E170" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F170" t="n">
         <v>0</v>
@@ -7251,10 +7251,10 @@
         <v>0</v>
       </c>
       <c r="D171" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E171" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F171" t="n">
         <v>0</v>
@@ -7291,10 +7291,10 @@
         <v>3</v>
       </c>
       <c r="D172" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="E172" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="F172" t="n">
         <v>0</v>
@@ -7331,10 +7331,10 @@
         <v>3</v>
       </c>
       <c r="D173" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E173" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -7371,10 +7371,10 @@
         <v>4</v>
       </c>
       <c r="D174" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E174" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F174" t="n">
         <v>0</v>
@@ -7451,10 +7451,10 @@
         <v>2</v>
       </c>
       <c r="D176" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F176" t="n">
         <v>0</v>
@@ -7571,10 +7571,10 @@
         <v>2</v>
       </c>
       <c r="D179" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E179" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F179" t="n">
         <v>0</v>
@@ -7851,10 +7851,10 @@
         <v>2</v>
       </c>
       <c r="D186" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E186" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F186" t="n">
         <v>0</v>
@@ -7891,10 +7891,10 @@
         <v>0</v>
       </c>
       <c r="D187" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E187" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F187" t="n">
         <v>0</v>
@@ -8011,10 +8011,10 @@
         <v>2</v>
       </c>
       <c r="D190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E190" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F190" t="n">
         <v>0</v>
@@ -8051,10 +8051,10 @@
         <v>3</v>
       </c>
       <c r="D191" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E191" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F191" t="n">
         <v>0</v>
@@ -8131,10 +8131,10 @@
         <v>0</v>
       </c>
       <c r="D193" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E193" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F193" t="n">
         <v>0</v>
@@ -8251,10 +8251,10 @@
         <v>0</v>
       </c>
       <c r="D196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E196" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
@@ -8371,10 +8371,10 @@
         <v>0</v>
       </c>
       <c r="D199" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E199" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F199" t="n">
         <v>0</v>
@@ -8491,10 +8491,10 @@
         <v>0</v>
       </c>
       <c r="D202" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E202" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F202" t="n">
         <v>0</v>
@@ -8531,10 +8531,10 @@
         <v>1</v>
       </c>
       <c r="D203" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E203" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F203" t="n">
         <v>0</v>
@@ -8651,10 +8651,10 @@
         <v>0</v>
       </c>
       <c r="D206" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E206" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F206" t="n">
         <v>0</v>
@@ -8891,10 +8891,10 @@
         <v>0</v>
       </c>
       <c r="D212" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E212" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F212" t="n">
         <v>0</v>
@@ -9091,10 +9091,10 @@
         <v>0</v>
       </c>
       <c r="D217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E217" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F217" t="n">
         <v>0</v>
@@ -9811,10 +9811,10 @@
         <v>56</v>
       </c>
       <c r="D235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E235" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F235" t="n">
         <v>0</v>
@@ -9851,10 +9851,10 @@
         <v>172</v>
       </c>
       <c r="D236" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E236" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F236" t="n">
         <v>0</v>
@@ -9931,10 +9931,10 @@
         <v>66</v>
       </c>
       <c r="D238" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E238" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F238" t="n">
         <v>0</v>
@@ -10011,10 +10011,10 @@
         <v>66</v>
       </c>
       <c r="D240" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E240" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F240" t="n">
         <v>0</v>
@@ -10051,10 +10051,10 @@
         <v>36</v>
       </c>
       <c r="D241" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E241" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F241" t="n">
         <v>0</v>
@@ -10091,10 +10091,10 @@
         <v>36</v>
       </c>
       <c r="D242" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E242" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F242" t="n">
         <v>0</v>
@@ -10131,10 +10131,10 @@
         <v>18</v>
       </c>
       <c r="D243" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E243" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F243" t="n">
         <v>0</v>
@@ -10171,10 +10171,10 @@
         <v>21</v>
       </c>
       <c r="D244" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E244" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F244" t="n">
         <v>0</v>
@@ -10211,10 +10211,10 @@
         <v>0</v>
       </c>
       <c r="D245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E245" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F245" t="n">
         <v>0</v>
@@ -10251,10 +10251,10 @@
         <v>111</v>
       </c>
       <c r="D246" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E246" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F246" t="n">
         <v>0</v>
@@ -10291,10 +10291,10 @@
         <v>23</v>
       </c>
       <c r="D247" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E247" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F247" t="n">
         <v>0</v>
@@ -10331,10 +10331,10 @@
         <v>2</v>
       </c>
       <c r="D248" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E248" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F248" t="n">
         <v>0</v>
@@ -10371,10 +10371,10 @@
         <v>12</v>
       </c>
       <c r="D249" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E249" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F249" t="n">
         <v>0</v>
@@ -10411,10 +10411,10 @@
         <v>11</v>
       </c>
       <c r="D250" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E250" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F250" t="n">
         <v>0</v>
@@ -10571,10 +10571,10 @@
         <v>21</v>
       </c>
       <c r="D254" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E254" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F254" t="n">
         <v>0</v>
@@ -10611,10 +10611,10 @@
         <v>11</v>
       </c>
       <c r="D255" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E255" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F255" t="n">
         <v>0</v>
@@ -10651,10 +10651,10 @@
         <v>16</v>
       </c>
       <c r="D256" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E256" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F256" t="n">
         <v>0</v>
@@ -10691,10 +10691,10 @@
         <v>15</v>
       </c>
       <c r="D257" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E257" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F257" t="n">
         <v>0</v>
@@ -10811,10 +10811,10 @@
         <v>19</v>
       </c>
       <c r="D260" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E260" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F260" t="n">
         <v>0</v>
@@ -10851,10 +10851,10 @@
         <v>0</v>
       </c>
       <c r="D261" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E261" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F261" t="n">
         <v>0</v>
@@ -10891,10 +10891,10 @@
         <v>0</v>
       </c>
       <c r="D262" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E262" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F262" t="n">
         <v>0</v>
@@ -10931,10 +10931,10 @@
         <v>0</v>
       </c>
       <c r="D263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E263" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F263" t="n">
         <v>0</v>
@@ -10971,10 +10971,10 @@
         <v>0</v>
       </c>
       <c r="D264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E264" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F264" t="n">
         <v>0</v>
@@ -11051,10 +11051,10 @@
         <v>0</v>
       </c>
       <c r="D266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F266" t="n">
         <v>0</v>
@@ -11091,10 +11091,10 @@
         <v>0</v>
       </c>
       <c r="D267" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E267" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F267" t="n">
         <v>0</v>
@@ -11131,10 +11131,10 @@
         <v>0</v>
       </c>
       <c r="D268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F268" t="n">
         <v>0</v>
@@ -11171,10 +11171,10 @@
         <v>0</v>
       </c>
       <c r="D269" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E269" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F269" t="n">
         <v>0</v>
@@ -11211,10 +11211,10 @@
         <v>0</v>
       </c>
       <c r="D270" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E270" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F270" t="n">
         <v>0</v>
@@ -11251,10 +11251,10 @@
         <v>0</v>
       </c>
       <c r="D271" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E271" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F271" t="n">
         <v>0</v>
@@ -11291,10 +11291,10 @@
         <v>0</v>
       </c>
       <c r="D272" t="n">
+        <v>0</v>
+      </c>
+      <c r="E272" t="n">
         <v>24</v>
-      </c>
-      <c r="E272" t="n">
-        <v>0</v>
       </c>
       <c r="F272" t="n">
         <v>0</v>
@@ -11331,10 +11331,10 @@
         <v>0</v>
       </c>
       <c r="D273" t="n">
+        <v>0</v>
+      </c>
+      <c r="E273" t="n">
         <v>30</v>
-      </c>
-      <c r="E273" t="n">
-        <v>0</v>
       </c>
       <c r="F273" t="n">
         <v>0</v>
@@ -11371,10 +11371,10 @@
         <v>0</v>
       </c>
       <c r="D274" t="n">
+        <v>9</v>
+      </c>
+      <c r="E274" t="n">
         <v>41</v>
-      </c>
-      <c r="E274" t="n">
-        <v>9</v>
       </c>
       <c r="F274" t="n">
         <v>0</v>
@@ -11411,10 +11411,10 @@
         <v>0</v>
       </c>
       <c r="D275" t="n">
+        <v>1</v>
+      </c>
+      <c r="E275" t="n">
         <v>18</v>
-      </c>
-      <c r="E275" t="n">
-        <v>1</v>
       </c>
       <c r="F275" t="n">
         <v>0</v>
@@ -11451,10 +11451,10 @@
         <v>0</v>
       </c>
       <c r="D276" t="n">
+        <v>0</v>
+      </c>
+      <c r="E276" t="n">
         <v>24</v>
-      </c>
-      <c r="E276" t="n">
-        <v>0</v>
       </c>
       <c r="F276" t="n">
         <v>0</v>
@@ -11491,10 +11491,10 @@
         <v>0</v>
       </c>
       <c r="D277" t="n">
+        <v>0</v>
+      </c>
+      <c r="E277" t="n">
         <v>27</v>
-      </c>
-      <c r="E277" t="n">
-        <v>0</v>
       </c>
       <c r="F277" t="n">
         <v>0</v>
@@ -11531,10 +11531,10 @@
         <v>0</v>
       </c>
       <c r="D278" t="n">
+        <v>0</v>
+      </c>
+      <c r="E278" t="n">
         <v>36</v>
-      </c>
-      <c r="E278" t="n">
-        <v>0</v>
       </c>
       <c r="F278" t="n">
         <v>0</v>
@@ -11571,10 +11571,10 @@
         <v>0</v>
       </c>
       <c r="D279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E279" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F279" t="n">
         <v>0</v>
@@ -11611,10 +11611,10 @@
         <v>0</v>
       </c>
       <c r="D280" t="n">
+        <v>8</v>
+      </c>
+      <c r="E280" t="n">
         <v>9</v>
-      </c>
-      <c r="E280" t="n">
-        <v>8</v>
       </c>
       <c r="F280" t="n">
         <v>0</v>
@@ -11651,10 +11651,10 @@
         <v>0</v>
       </c>
       <c r="D281" t="n">
+        <v>0</v>
+      </c>
+      <c r="E281" t="n">
         <v>30</v>
-      </c>
-      <c r="E281" t="n">
-        <v>0</v>
       </c>
       <c r="F281" t="n">
         <v>0</v>
@@ -11691,10 +11691,10 @@
         <v>0</v>
       </c>
       <c r="D282" t="n">
+        <v>7</v>
+      </c>
+      <c r="E282" t="n">
         <v>29</v>
-      </c>
-      <c r="E282" t="n">
-        <v>7</v>
       </c>
       <c r="F282" t="n">
         <v>0</v>
@@ -11731,10 +11731,10 @@
         <v>0</v>
       </c>
       <c r="D283" t="n">
+        <v>0</v>
+      </c>
+      <c r="E283" t="n">
         <v>11</v>
-      </c>
-      <c r="E283" t="n">
-        <v>0</v>
       </c>
       <c r="F283" t="n">
         <v>0</v>
@@ -11771,10 +11771,10 @@
         <v>0</v>
       </c>
       <c r="D284" t="n">
+        <v>6</v>
+      </c>
+      <c r="E284" t="n">
         <v>15</v>
-      </c>
-      <c r="E284" t="n">
-        <v>6</v>
       </c>
       <c r="F284" t="n">
         <v>0</v>
@@ -11811,10 +11811,10 @@
         <v>0</v>
       </c>
       <c r="D285" t="n">
+        <v>8</v>
+      </c>
+      <c r="E285" t="n">
         <v>18</v>
-      </c>
-      <c r="E285" t="n">
-        <v>8</v>
       </c>
       <c r="F285" t="n">
         <v>0</v>
@@ -11851,10 +11851,10 @@
         <v>0</v>
       </c>
       <c r="D286" t="n">
+        <v>6</v>
+      </c>
+      <c r="E286" t="n">
         <v>19</v>
-      </c>
-      <c r="E286" t="n">
-        <v>6</v>
       </c>
       <c r="F286" t="n">
         <v>0</v>
@@ -11891,10 +11891,10 @@
         <v>0</v>
       </c>
       <c r="D287" t="n">
+        <v>2</v>
+      </c>
+      <c r="E287" t="n">
         <v>19</v>
-      </c>
-      <c r="E287" t="n">
-        <v>2</v>
       </c>
       <c r="F287" t="n">
         <v>0</v>
@@ -11931,10 +11931,10 @@
         <v>0</v>
       </c>
       <c r="D288" t="n">
+        <v>5</v>
+      </c>
+      <c r="E288" t="n">
         <v>15</v>
-      </c>
-      <c r="E288" t="n">
-        <v>5</v>
       </c>
       <c r="F288" t="n">
         <v>0</v>
@@ -11971,10 +11971,10 @@
         <v>0</v>
       </c>
       <c r="D289" t="n">
+        <v>4</v>
+      </c>
+      <c r="E289" t="n">
         <v>13</v>
-      </c>
-      <c r="E289" t="n">
-        <v>4</v>
       </c>
       <c r="F289" t="n">
         <v>0</v>
@@ -12011,10 +12011,10 @@
         <v>0</v>
       </c>
       <c r="D290" t="n">
+        <v>0</v>
+      </c>
+      <c r="E290" t="n">
         <v>19</v>
-      </c>
-      <c r="E290" t="n">
-        <v>0</v>
       </c>
       <c r="F290" t="n">
         <v>0</v>
@@ -12051,10 +12051,10 @@
         <v>0</v>
       </c>
       <c r="D291" t="n">
+        <v>2</v>
+      </c>
+      <c r="E291" t="n">
         <v>20</v>
-      </c>
-      <c r="E291" t="n">
-        <v>2</v>
       </c>
       <c r="F291" t="n">
         <v>0</v>
@@ -12091,10 +12091,10 @@
         <v>0</v>
       </c>
       <c r="D292" t="n">
+        <v>2</v>
+      </c>
+      <c r="E292" t="n">
         <v>17</v>
-      </c>
-      <c r="E292" t="n">
-        <v>2</v>
       </c>
       <c r="F292" t="n">
         <v>0</v>
@@ -12131,10 +12131,10 @@
         <v>0</v>
       </c>
       <c r="D293" t="n">
+        <v>0</v>
+      </c>
+      <c r="E293" t="n">
         <v>20</v>
-      </c>
-      <c r="E293" t="n">
-        <v>0</v>
       </c>
       <c r="F293" t="n">
         <v>0</v>
@@ -12171,10 +12171,10 @@
         <v>0</v>
       </c>
       <c r="D294" t="n">
+        <v>0</v>
+      </c>
+      <c r="E294" t="n">
         <v>12</v>
-      </c>
-      <c r="E294" t="n">
-        <v>0</v>
       </c>
       <c r="F294" t="n">
         <v>0</v>
@@ -12211,10 +12211,10 @@
         <v>0</v>
       </c>
       <c r="D295" t="n">
+        <v>13</v>
+      </c>
+      <c r="E295" t="n">
         <v>26</v>
-      </c>
-      <c r="E295" t="n">
-        <v>13</v>
       </c>
       <c r="F295" t="n">
         <v>0</v>
@@ -12251,10 +12251,10 @@
         <v>0</v>
       </c>
       <c r="D296" t="n">
+        <v>4</v>
+      </c>
+      <c r="E296" t="n">
         <v>23</v>
-      </c>
-      <c r="E296" t="n">
-        <v>4</v>
       </c>
       <c r="F296" t="n">
         <v>0</v>
@@ -12291,10 +12291,10 @@
         <v>0</v>
       </c>
       <c r="D297" t="n">
+        <v>2</v>
+      </c>
+      <c r="E297" t="n">
         <v>24</v>
-      </c>
-      <c r="E297" t="n">
-        <v>2</v>
       </c>
       <c r="F297" t="n">
         <v>0</v>
@@ -12331,10 +12331,10 @@
         <v>0</v>
       </c>
       <c r="D298" t="n">
+        <v>0</v>
+      </c>
+      <c r="E298" t="n">
         <v>17</v>
-      </c>
-      <c r="E298" t="n">
-        <v>0</v>
       </c>
       <c r="F298" t="n">
         <v>0</v>
@@ -12371,10 +12371,10 @@
         <v>0</v>
       </c>
       <c r="D299" t="n">
+        <v>0</v>
+      </c>
+      <c r="E299" t="n">
         <v>38</v>
-      </c>
-      <c r="E299" t="n">
-        <v>0</v>
       </c>
       <c r="F299" t="n">
         <v>0</v>
@@ -12411,10 +12411,10 @@
         <v>0</v>
       </c>
       <c r="D300" t="n">
+        <v>0</v>
+      </c>
+      <c r="E300" t="n">
         <v>17</v>
-      </c>
-      <c r="E300" t="n">
-        <v>0</v>
       </c>
       <c r="F300" t="n">
         <v>0</v>
@@ -12451,10 +12451,10 @@
         <v>0</v>
       </c>
       <c r="D301" t="n">
+        <v>0</v>
+      </c>
+      <c r="E301" t="n">
         <v>26</v>
-      </c>
-      <c r="E301" t="n">
-        <v>0</v>
       </c>
       <c r="F301" t="n">
         <v>0</v>
@@ -12491,10 +12491,10 @@
         <v>0</v>
       </c>
       <c r="D302" t="n">
+        <v>0</v>
+      </c>
+      <c r="E302" t="n">
         <v>22</v>
-      </c>
-      <c r="E302" t="n">
-        <v>0</v>
       </c>
       <c r="F302" t="n">
         <v>0</v>
@@ -12531,10 +12531,10 @@
         <v>16</v>
       </c>
       <c r="D303" t="n">
+        <v>20</v>
+      </c>
+      <c r="E303" t="n">
         <v>15</v>
-      </c>
-      <c r="E303" t="n">
-        <v>20</v>
       </c>
       <c r="F303" t="n">
         <v>0</v>
@@ -12571,10 +12571,10 @@
         <v>5</v>
       </c>
       <c r="D304" t="n">
+        <v>1</v>
+      </c>
+      <c r="E304" t="n">
         <v>21</v>
-      </c>
-      <c r="E304" t="n">
-        <v>1</v>
       </c>
       <c r="F304" t="n">
         <v>0</v>
@@ -12611,10 +12611,10 @@
         <v>24</v>
       </c>
       <c r="D305" t="n">
+        <v>2</v>
+      </c>
+      <c r="E305" t="n">
         <v>22</v>
-      </c>
-      <c r="E305" t="n">
-        <v>2</v>
       </c>
       <c r="F305" t="n">
         <v>1</v>
@@ -12651,10 +12651,10 @@
         <v>27</v>
       </c>
       <c r="D306" t="n">
+        <v>3</v>
+      </c>
+      <c r="E306" t="n">
         <v>6</v>
-      </c>
-      <c r="E306" t="n">
-        <v>3</v>
       </c>
       <c r="F306" t="n">
         <v>6</v>
@@ -12811,10 +12811,10 @@
         <v>28</v>
       </c>
       <c r="D310" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E310" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F310" t="n">
         <v>13</v>
@@ -13051,10 +13051,10 @@
         <v>25</v>
       </c>
       <c r="D316" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E316" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F316" t="n">
         <v>25</v>
@@ -13211,10 +13211,10 @@
         <v>10</v>
       </c>
       <c r="D320" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E320" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F320" t="n">
         <v>4</v>
@@ -13371,10 +13371,10 @@
         <v>11</v>
       </c>
       <c r="D324" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E324" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F324" t="n">
         <v>4</v>
@@ -13411,10 +13411,10 @@
         <v>8</v>
       </c>
       <c r="D325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E325" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F325" t="n">
         <v>7</v>
@@ -13451,10 +13451,10 @@
         <v>19</v>
       </c>
       <c r="D326" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E326" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F326" t="n">
         <v>10</v>
@@ -13931,10 +13931,10 @@
         <v>32</v>
       </c>
       <c r="D338" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E338" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F338" t="n">
         <v>0</v>
@@ -14051,10 +14051,10 @@
         <v>10</v>
       </c>
       <c r="D341" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F341" t="n">
         <v>0</v>
@@ -14156,6 +14156,86 @@
       </c>
       <c r="L343" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>27</v>
+      </c>
+      <c r="C344" t="n">
+        <v>26</v>
+      </c>
+      <c r="D344" t="n">
+        <v>4</v>
+      </c>
+      <c r="E344" t="n">
+        <v>0</v>
+      </c>
+      <c r="F344" t="n">
+        <v>0</v>
+      </c>
+      <c r="G344" t="n">
+        <v>2</v>
+      </c>
+      <c r="H344" t="n">
+        <v>0</v>
+      </c>
+      <c r="I344" t="n">
+        <v>0</v>
+      </c>
+      <c r="J344" t="n">
+        <v>0</v>
+      </c>
+      <c r="K344" t="n">
+        <v>2</v>
+      </c>
+      <c r="L344" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>28</v>
+      </c>
+      <c r="C345" t="n">
+        <v>29</v>
+      </c>
+      <c r="D345" t="n">
+        <v>4</v>
+      </c>
+      <c r="E345" t="n">
+        <v>0</v>
+      </c>
+      <c r="F345" t="n">
+        <v>0</v>
+      </c>
+      <c r="G345" t="n">
+        <v>9</v>
+      </c>
+      <c r="H345" t="n">
+        <v>0</v>
+      </c>
+      <c r="I345" t="n">
+        <v>0</v>
+      </c>
+      <c r="J345" t="n">
+        <v>0</v>
+      </c>
+      <c r="K345" t="n">
+        <v>3</v>
+      </c>
+      <c r="L345" t="n">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-22 11:00
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L350"/>
+  <dimension ref="A1:L351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,12 +464,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>GUTSHIFT</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Other</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -11509,10 +11509,10 @@
         <v>0</v>
       </c>
       <c r="J277" t="n">
+        <v>0</v>
+      </c>
+      <c r="K277" t="n">
         <v>3</v>
-      </c>
-      <c r="K277" t="n">
-        <v>0</v>
       </c>
       <c r="L277" t="n">
         <v>103</v>
@@ -11589,10 +11589,10 @@
         <v>0</v>
       </c>
       <c r="J279" t="n">
+        <v>0</v>
+      </c>
+      <c r="K279" t="n">
         <v>2</v>
-      </c>
-      <c r="K279" t="n">
-        <v>0</v>
       </c>
       <c r="L279" t="n">
         <v>5</v>
@@ -11629,10 +11629,10 @@
         <v>0</v>
       </c>
       <c r="J280" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L280" t="n">
         <v>146</v>
@@ -11709,10 +11709,10 @@
         <v>1</v>
       </c>
       <c r="J282" t="n">
+        <v>0</v>
+      </c>
+      <c r="K282" t="n">
         <v>2</v>
-      </c>
-      <c r="K282" t="n">
-        <v>0</v>
       </c>
       <c r="L282" t="n">
         <v>104</v>
@@ -11749,10 +11749,10 @@
         <v>0</v>
       </c>
       <c r="J283" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L283" t="n">
         <v>104</v>
@@ -11789,10 +11789,10 @@
         <v>0</v>
       </c>
       <c r="J284" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L284" t="n">
         <v>101</v>
@@ -11829,10 +11829,10 @@
         <v>0</v>
       </c>
       <c r="J285" t="n">
+        <v>0</v>
+      </c>
+      <c r="K285" t="n">
         <v>5</v>
-      </c>
-      <c r="K285" t="n">
-        <v>0</v>
       </c>
       <c r="L285" t="n">
         <v>122</v>
@@ -11869,10 +11869,10 @@
         <v>0</v>
       </c>
       <c r="J286" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L286" t="n">
         <v>297</v>
@@ -11909,10 +11909,10 @@
         <v>0</v>
       </c>
       <c r="J287" t="n">
+        <v>0</v>
+      </c>
+      <c r="K287" t="n">
         <v>3</v>
-      </c>
-      <c r="K287" t="n">
-        <v>0</v>
       </c>
       <c r="L287" t="n">
         <v>30</v>
@@ -11949,10 +11949,10 @@
         <v>0</v>
       </c>
       <c r="J288" t="n">
+        <v>0</v>
+      </c>
+      <c r="K288" t="n">
         <v>2</v>
-      </c>
-      <c r="K288" t="n">
-        <v>0</v>
       </c>
       <c r="L288" t="n">
         <v>38</v>
@@ -11989,10 +11989,10 @@
         <v>0</v>
       </c>
       <c r="J289" t="n">
+        <v>0</v>
+      </c>
+      <c r="K289" t="n">
         <v>3</v>
-      </c>
-      <c r="K289" t="n">
-        <v>0</v>
       </c>
       <c r="L289" t="n">
         <v>110</v>
@@ -12029,10 +12029,10 @@
         <v>0</v>
       </c>
       <c r="J290" t="n">
+        <v>0</v>
+      </c>
+      <c r="K290" t="n">
         <v>2</v>
-      </c>
-      <c r="K290" t="n">
-        <v>0</v>
       </c>
       <c r="L290" t="n">
         <v>311</v>
@@ -12069,10 +12069,10 @@
         <v>0</v>
       </c>
       <c r="J291" t="n">
+        <v>0</v>
+      </c>
+      <c r="K291" t="n">
         <v>3</v>
-      </c>
-      <c r="K291" t="n">
-        <v>0</v>
       </c>
       <c r="L291" t="n">
         <v>129</v>
@@ -12109,10 +12109,10 @@
         <v>0</v>
       </c>
       <c r="J292" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K292" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L292" t="n">
         <v>26</v>
@@ -13629,10 +13629,10 @@
         <v>0</v>
       </c>
       <c r="J330" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K330" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L330" t="n">
         <v>71</v>
@@ -13669,10 +13669,10 @@
         <v>0</v>
       </c>
       <c r="J331" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K331" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L331" t="n">
         <v>149</v>
@@ -13949,10 +13949,10 @@
         <v>0</v>
       </c>
       <c r="J338" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K338" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L338" t="n">
         <v>54</v>
@@ -14069,10 +14069,10 @@
         <v>0</v>
       </c>
       <c r="J341" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L341" t="n">
         <v>15</v>
@@ -14189,10 +14189,10 @@
         <v>0</v>
       </c>
       <c r="J344" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K344" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L344" t="n">
         <v>61</v>
@@ -14229,10 +14229,10 @@
         <v>0</v>
       </c>
       <c r="J345" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K345" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L345" t="n">
         <v>73</v>
@@ -14269,10 +14269,10 @@
         <v>0</v>
       </c>
       <c r="J346" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K346" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L346" t="n">
         <v>56</v>
@@ -14309,10 +14309,10 @@
         <v>0</v>
       </c>
       <c r="J347" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K347" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L347" t="n">
         <v>26</v>
@@ -14349,10 +14349,10 @@
         <v>0</v>
       </c>
       <c r="J348" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K348" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L348" t="n">
         <v>60</v>
@@ -14389,10 +14389,10 @@
         <v>0</v>
       </c>
       <c r="J349" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K349" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L349" t="n">
         <v>31</v>
@@ -14429,13 +14429,53 @@
         <v>0</v>
       </c>
       <c r="J350" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K350" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L350" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B351" t="n">
+        <v>18</v>
+      </c>
+      <c r="C351" t="n">
+        <v>19</v>
+      </c>
+      <c r="D351" t="n">
+        <v>9</v>
+      </c>
+      <c r="E351" t="n">
+        <v>0</v>
+      </c>
+      <c r="F351" t="n">
+        <v>0</v>
+      </c>
+      <c r="G351" t="n">
+        <v>8</v>
+      </c>
+      <c r="H351" t="n">
+        <v>5</v>
+      </c>
+      <c r="I351" t="n">
+        <v>0</v>
+      </c>
+      <c r="J351" t="n">
+        <v>2</v>
+      </c>
+      <c r="K351" t="n">
+        <v>0</v>
+      </c>
+      <c r="L351" t="n">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-23 13:00
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L351"/>
+  <dimension ref="A1:M352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Matcha</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Total units</t>
         </is>
       </c>
@@ -515,6 +520,9 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
         <v>14</v>
       </c>
     </row>
@@ -555,6 +563,9 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
         <v>34</v>
       </c>
     </row>
@@ -595,6 +606,9 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -635,6 +649,9 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
         <v>4</v>
       </c>
     </row>
@@ -675,6 +692,9 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -715,6 +735,9 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -755,6 +778,9 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
         <v>5</v>
       </c>
     </row>
@@ -795,6 +821,9 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -835,6 +864,9 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
         <v>5</v>
       </c>
     </row>
@@ -875,6 +907,9 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
         <v>4</v>
       </c>
     </row>
@@ -915,6 +950,9 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
         <v>3</v>
       </c>
     </row>
@@ -955,6 +993,9 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -995,6 +1036,9 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1035,6 +1079,9 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1075,6 +1122,9 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1115,6 +1165,9 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1155,6 +1208,9 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1195,6 +1251,9 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1235,6 +1294,9 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1275,6 +1337,9 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1315,6 +1380,9 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1355,6 +1423,9 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1395,6 +1466,9 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1435,6 +1509,9 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1475,6 +1552,9 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1515,6 +1595,9 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1555,6 +1638,9 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
         <v>28</v>
       </c>
     </row>
@@ -1595,6 +1681,9 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
         <v>26</v>
       </c>
     </row>
@@ -1635,6 +1724,9 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1675,6 +1767,9 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
         <v>29</v>
       </c>
     </row>
@@ -1715,6 +1810,9 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
         <v>29</v>
       </c>
     </row>
@@ -1755,6 +1853,9 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1795,6 +1896,9 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1835,6 +1939,9 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1875,6 +1982,9 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1915,6 +2025,9 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1955,6 +2068,9 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1995,6 +2111,9 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2035,6 +2154,9 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2075,6 +2197,9 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2115,6 +2240,9 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="n">
         <v>34</v>
       </c>
     </row>
@@ -2155,6 +2283,9 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2195,6 +2326,9 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2235,6 +2369,9 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2275,6 +2412,9 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2315,6 +2455,9 @@
         <v>0</v>
       </c>
       <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2355,6 +2498,9 @@
         <v>0</v>
       </c>
       <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2395,6 +2541,9 @@
         <v>0</v>
       </c>
       <c r="L49" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2435,6 +2584,9 @@
         <v>0</v>
       </c>
       <c r="L50" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2475,6 +2627,9 @@
         <v>0</v>
       </c>
       <c r="L51" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2515,6 +2670,9 @@
         <v>0</v>
       </c>
       <c r="L52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2555,6 +2713,9 @@
         <v>0</v>
       </c>
       <c r="L53" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2595,6 +2756,9 @@
         <v>0</v>
       </c>
       <c r="L54" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2635,6 +2799,9 @@
         <v>0</v>
       </c>
       <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2675,6 +2842,9 @@
         <v>0</v>
       </c>
       <c r="L56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2715,6 +2885,9 @@
         <v>0</v>
       </c>
       <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="n">
         <v>49</v>
       </c>
     </row>
@@ -2755,6 +2928,9 @@
         <v>0</v>
       </c>
       <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2795,6 +2971,9 @@
         <v>0</v>
       </c>
       <c r="L59" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2835,6 +3014,9 @@
         <v>0</v>
       </c>
       <c r="L60" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2875,6 +3057,9 @@
         <v>0</v>
       </c>
       <c r="L61" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2915,6 +3100,9 @@
         <v>0</v>
       </c>
       <c r="L62" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2955,6 +3143,9 @@
         <v>0</v>
       </c>
       <c r="L63" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2995,6 +3186,9 @@
         <v>0</v>
       </c>
       <c r="L64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3035,6 +3229,9 @@
         <v>0</v>
       </c>
       <c r="L65" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" t="n">
         <v>70</v>
       </c>
     </row>
@@ -3075,6 +3272,9 @@
         <v>0</v>
       </c>
       <c r="L66" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" t="n">
         <v>26</v>
       </c>
     </row>
@@ -3115,6 +3315,9 @@
         <v>0</v>
       </c>
       <c r="L67" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" t="n">
         <v>44</v>
       </c>
     </row>
@@ -3155,6 +3358,9 @@
         <v>0</v>
       </c>
       <c r="L68" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3195,6 +3401,9 @@
         <v>0</v>
       </c>
       <c r="L69" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" t="n">
         <v>39</v>
       </c>
     </row>
@@ -3235,6 +3444,9 @@
         <v>0</v>
       </c>
       <c r="L70" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" t="n">
         <v>27</v>
       </c>
     </row>
@@ -3275,6 +3487,9 @@
         <v>0</v>
       </c>
       <c r="L71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3315,6 +3530,9 @@
         <v>0</v>
       </c>
       <c r="L72" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3355,6 +3573,9 @@
         <v>0</v>
       </c>
       <c r="L73" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3395,6 +3616,9 @@
         <v>0</v>
       </c>
       <c r="L74" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" t="n">
         <v>41</v>
       </c>
     </row>
@@ -3435,6 +3659,9 @@
         <v>0</v>
       </c>
       <c r="L75" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3475,6 +3702,9 @@
         <v>0</v>
       </c>
       <c r="L76" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" t="n">
         <v>38</v>
       </c>
     </row>
@@ -3515,6 +3745,9 @@
         <v>0</v>
       </c>
       <c r="L77" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3555,6 +3788,9 @@
         <v>0</v>
       </c>
       <c r="L78" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3595,6 +3831,9 @@
         <v>0</v>
       </c>
       <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3635,6 +3874,9 @@
         <v>0</v>
       </c>
       <c r="L80" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" t="n">
         <v>35</v>
       </c>
     </row>
@@ -3675,6 +3917,9 @@
         <v>0</v>
       </c>
       <c r="L81" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" t="n">
         <v>35</v>
       </c>
     </row>
@@ -3715,6 +3960,9 @@
         <v>0</v>
       </c>
       <c r="L82" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3755,6 +4003,9 @@
         <v>0</v>
       </c>
       <c r="L83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" t="n">
         <v>46</v>
       </c>
     </row>
@@ -3795,6 +4046,9 @@
         <v>0</v>
       </c>
       <c r="L84" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3835,6 +4089,9 @@
         <v>0</v>
       </c>
       <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3875,6 +4132,9 @@
         <v>0</v>
       </c>
       <c r="L86" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3915,6 +4175,9 @@
         <v>0</v>
       </c>
       <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
         <v>57</v>
       </c>
     </row>
@@ -3955,6 +4218,9 @@
         <v>0</v>
       </c>
       <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3995,6 +4261,9 @@
         <v>0</v>
       </c>
       <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4035,6 +4304,9 @@
         <v>0</v>
       </c>
       <c r="L90" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4075,6 +4347,9 @@
         <v>0</v>
       </c>
       <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
         <v>22</v>
       </c>
     </row>
@@ -4115,6 +4390,9 @@
         <v>0</v>
       </c>
       <c r="L92" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4155,6 +4433,9 @@
         <v>0</v>
       </c>
       <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="n">
         <v>16</v>
       </c>
     </row>
@@ -4195,6 +4476,9 @@
         <v>0</v>
       </c>
       <c r="L94" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4235,6 +4519,9 @@
         <v>0</v>
       </c>
       <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="n">
         <v>36</v>
       </c>
     </row>
@@ -4275,6 +4562,9 @@
         <v>0</v>
       </c>
       <c r="L96" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" t="n">
         <v>21</v>
       </c>
     </row>
@@ -4315,6 +4605,9 @@
         <v>0</v>
       </c>
       <c r="L97" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" t="n">
         <v>23</v>
       </c>
     </row>
@@ -4355,6 +4648,9 @@
         <v>0</v>
       </c>
       <c r="L98" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4395,6 +4691,9 @@
         <v>0</v>
       </c>
       <c r="L99" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4435,6 +4734,9 @@
         <v>0</v>
       </c>
       <c r="L100" t="n">
+        <v>0</v>
+      </c>
+      <c r="M100" t="n">
         <v>39</v>
       </c>
     </row>
@@ -4475,6 +4777,9 @@
         <v>0</v>
       </c>
       <c r="L101" t="n">
+        <v>0</v>
+      </c>
+      <c r="M101" t="n">
         <v>28</v>
       </c>
     </row>
@@ -4515,6 +4820,9 @@
         <v>0</v>
       </c>
       <c r="L102" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" t="n">
         <v>21</v>
       </c>
     </row>
@@ -4555,6 +4863,9 @@
         <v>0</v>
       </c>
       <c r="L103" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" t="n">
         <v>46</v>
       </c>
     </row>
@@ -4595,6 +4906,9 @@
         <v>0</v>
       </c>
       <c r="L104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4635,6 +4949,9 @@
         <v>0</v>
       </c>
       <c r="L105" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4675,6 +4992,9 @@
         <v>0</v>
       </c>
       <c r="L106" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4715,6 +5035,9 @@
         <v>0</v>
       </c>
       <c r="L107" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" t="n">
         <v>21</v>
       </c>
     </row>
@@ -4755,6 +5078,9 @@
         <v>0</v>
       </c>
       <c r="L108" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" t="n">
         <v>23</v>
       </c>
     </row>
@@ -4795,6 +5121,9 @@
         <v>0</v>
       </c>
       <c r="L109" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4835,6 +5164,9 @@
         <v>0</v>
       </c>
       <c r="L110" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" t="n">
         <v>42</v>
       </c>
     </row>
@@ -4875,6 +5207,9 @@
         <v>0</v>
       </c>
       <c r="L111" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4915,6 +5250,9 @@
         <v>0</v>
       </c>
       <c r="L112" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4955,6 +5293,9 @@
         <v>0</v>
       </c>
       <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="n">
         <v>53</v>
       </c>
     </row>
@@ -4995,6 +5336,9 @@
         <v>0</v>
       </c>
       <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
         <v>29</v>
       </c>
     </row>
@@ -5035,6 +5379,9 @@
         <v>0</v>
       </c>
       <c r="L115" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5075,6 +5422,9 @@
         <v>0</v>
       </c>
       <c r="L116" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5115,6 +5465,9 @@
         <v>0</v>
       </c>
       <c r="L117" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5155,6 +5508,9 @@
         <v>0</v>
       </c>
       <c r="L118" t="n">
+        <v>0</v>
+      </c>
+      <c r="M118" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5195,6 +5551,9 @@
         <v>0</v>
       </c>
       <c r="L119" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5235,6 +5594,9 @@
         <v>0</v>
       </c>
       <c r="L120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5275,6 +5637,9 @@
         <v>0</v>
       </c>
       <c r="L121" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" t="n">
         <v>34</v>
       </c>
     </row>
@@ -5315,6 +5680,9 @@
         <v>0</v>
       </c>
       <c r="L122" t="n">
+        <v>0</v>
+      </c>
+      <c r="M122" t="n">
         <v>5</v>
       </c>
     </row>
@@ -5355,6 +5723,9 @@
         <v>0</v>
       </c>
       <c r="L123" t="n">
+        <v>0</v>
+      </c>
+      <c r="M123" t="n">
         <v>40</v>
       </c>
     </row>
@@ -5395,6 +5766,9 @@
         <v>0</v>
       </c>
       <c r="L124" t="n">
+        <v>0</v>
+      </c>
+      <c r="M124" t="n">
         <v>46</v>
       </c>
     </row>
@@ -5435,6 +5809,9 @@
         <v>0</v>
       </c>
       <c r="L125" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" t="n">
         <v>33</v>
       </c>
     </row>
@@ -5475,6 +5852,9 @@
         <v>0</v>
       </c>
       <c r="L126" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" t="n">
         <v>26</v>
       </c>
     </row>
@@ -5515,6 +5895,9 @@
         <v>0</v>
       </c>
       <c r="L127" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" t="n">
         <v>31</v>
       </c>
     </row>
@@ -5555,6 +5938,9 @@
         <v>0</v>
       </c>
       <c r="L128" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" t="n">
         <v>142</v>
       </c>
     </row>
@@ -5595,6 +5981,9 @@
         <v>0</v>
       </c>
       <c r="L129" t="n">
+        <v>0</v>
+      </c>
+      <c r="M129" t="n">
         <v>41</v>
       </c>
     </row>
@@ -5635,6 +6024,9 @@
         <v>0</v>
       </c>
       <c r="L130" t="n">
+        <v>0</v>
+      </c>
+      <c r="M130" t="n">
         <v>34</v>
       </c>
     </row>
@@ -5675,6 +6067,9 @@
         <v>0</v>
       </c>
       <c r="L131" t="n">
+        <v>0</v>
+      </c>
+      <c r="M131" t="n">
         <v>24</v>
       </c>
     </row>
@@ -5715,6 +6110,9 @@
         <v>0</v>
       </c>
       <c r="L132" t="n">
+        <v>0</v>
+      </c>
+      <c r="M132" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5755,6 +6153,9 @@
         <v>0</v>
       </c>
       <c r="L133" t="n">
+        <v>0</v>
+      </c>
+      <c r="M133" t="n">
         <v>98</v>
       </c>
     </row>
@@ -5795,6 +6196,9 @@
         <v>0</v>
       </c>
       <c r="L134" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5835,6 +6239,9 @@
         <v>0</v>
       </c>
       <c r="L135" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" t="n">
         <v>29</v>
       </c>
     </row>
@@ -5875,6 +6282,9 @@
         <v>0</v>
       </c>
       <c r="L136" t="n">
+        <v>0</v>
+      </c>
+      <c r="M136" t="n">
         <v>24</v>
       </c>
     </row>
@@ -5915,6 +6325,9 @@
         <v>0</v>
       </c>
       <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
         <v>21</v>
       </c>
     </row>
@@ -5955,6 +6368,9 @@
         <v>0</v>
       </c>
       <c r="L138" t="n">
+        <v>0</v>
+      </c>
+      <c r="M138" t="n">
         <v>33</v>
       </c>
     </row>
@@ -5995,6 +6411,9 @@
         <v>0</v>
       </c>
       <c r="L139" t="n">
+        <v>0</v>
+      </c>
+      <c r="M139" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6035,6 +6454,9 @@
         <v>0</v>
       </c>
       <c r="L140" t="n">
+        <v>0</v>
+      </c>
+      <c r="M140" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6075,6 +6497,9 @@
         <v>0</v>
       </c>
       <c r="L141" t="n">
+        <v>0</v>
+      </c>
+      <c r="M141" t="n">
         <v>81</v>
       </c>
     </row>
@@ -6115,6 +6540,9 @@
         <v>0</v>
       </c>
       <c r="L142" t="n">
+        <v>0</v>
+      </c>
+      <c r="M142" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6155,6 +6583,9 @@
         <v>0</v>
       </c>
       <c r="L143" t="n">
+        <v>0</v>
+      </c>
+      <c r="M143" t="n">
         <v>32</v>
       </c>
     </row>
@@ -6195,6 +6626,9 @@
         <v>0</v>
       </c>
       <c r="L144" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" t="n">
         <v>60</v>
       </c>
     </row>
@@ -6235,6 +6669,9 @@
         <v>0</v>
       </c>
       <c r="L145" t="n">
+        <v>0</v>
+      </c>
+      <c r="M145" t="n">
         <v>28</v>
       </c>
     </row>
@@ -6275,6 +6712,9 @@
         <v>0</v>
       </c>
       <c r="L146" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6315,6 +6755,9 @@
         <v>0</v>
       </c>
       <c r="L147" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" t="n">
         <v>34</v>
       </c>
     </row>
@@ -6355,6 +6798,9 @@
         <v>0</v>
       </c>
       <c r="L148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M148" t="n">
         <v>45</v>
       </c>
     </row>
@@ -6395,6 +6841,9 @@
         <v>0</v>
       </c>
       <c r="L149" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" t="n">
         <v>45</v>
       </c>
     </row>
@@ -6435,6 +6884,9 @@
         <v>0</v>
       </c>
       <c r="L150" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" t="n">
         <v>35</v>
       </c>
     </row>
@@ -6475,6 +6927,9 @@
         <v>0</v>
       </c>
       <c r="L151" t="n">
+        <v>0</v>
+      </c>
+      <c r="M151" t="n">
         <v>29</v>
       </c>
     </row>
@@ -6515,6 +6970,9 @@
         <v>0</v>
       </c>
       <c r="L152" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" t="n">
         <v>50</v>
       </c>
     </row>
@@ -6555,6 +7013,9 @@
         <v>0</v>
       </c>
       <c r="L153" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" t="n">
         <v>47</v>
       </c>
     </row>
@@ -6595,6 +7056,9 @@
         <v>0</v>
       </c>
       <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
         <v>77</v>
       </c>
     </row>
@@ -6635,6 +7099,9 @@
         <v>0</v>
       </c>
       <c r="L155" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" t="n">
         <v>34</v>
       </c>
     </row>
@@ -6675,6 +7142,9 @@
         <v>0</v>
       </c>
       <c r="L156" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" t="n">
         <v>81</v>
       </c>
     </row>
@@ -6715,6 +7185,9 @@
         <v>0</v>
       </c>
       <c r="L157" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6755,6 +7228,9 @@
         <v>0</v>
       </c>
       <c r="L158" t="n">
+        <v>0</v>
+      </c>
+      <c r="M158" t="n">
         <v>47</v>
       </c>
     </row>
@@ -6795,6 +7271,9 @@
         <v>0</v>
       </c>
       <c r="L159" t="n">
+        <v>0</v>
+      </c>
+      <c r="M159" t="n">
         <v>42</v>
       </c>
     </row>
@@ -6835,6 +7314,9 @@
         <v>0</v>
       </c>
       <c r="L160" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" t="n">
         <v>30</v>
       </c>
     </row>
@@ -6875,6 +7357,9 @@
         <v>0</v>
       </c>
       <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="n">
         <v>59</v>
       </c>
     </row>
@@ -6915,6 +7400,9 @@
         <v>0</v>
       </c>
       <c r="L162" t="n">
+        <v>0</v>
+      </c>
+      <c r="M162" t="n">
         <v>113</v>
       </c>
     </row>
@@ -6955,6 +7443,9 @@
         <v>0</v>
       </c>
       <c r="L163" t="n">
+        <v>0</v>
+      </c>
+      <c r="M163" t="n">
         <v>44</v>
       </c>
     </row>
@@ -6995,6 +7486,9 @@
         <v>0</v>
       </c>
       <c r="L164" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" t="n">
         <v>52</v>
       </c>
     </row>
@@ -7035,6 +7529,9 @@
         <v>0</v>
       </c>
       <c r="L165" t="n">
+        <v>0</v>
+      </c>
+      <c r="M165" t="n">
         <v>55</v>
       </c>
     </row>
@@ -7075,6 +7572,9 @@
         <v>0</v>
       </c>
       <c r="L166" t="n">
+        <v>0</v>
+      </c>
+      <c r="M166" t="n">
         <v>42</v>
       </c>
     </row>
@@ -7115,6 +7615,9 @@
         <v>0</v>
       </c>
       <c r="L167" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" t="n">
         <v>37</v>
       </c>
     </row>
@@ -7155,6 +7658,9 @@
         <v>0</v>
       </c>
       <c r="L168" t="n">
+        <v>0</v>
+      </c>
+      <c r="M168" t="n">
         <v>27</v>
       </c>
     </row>
@@ -7195,6 +7701,9 @@
         <v>0</v>
       </c>
       <c r="L169" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" t="n">
         <v>39</v>
       </c>
     </row>
@@ -7235,6 +7744,9 @@
         <v>0</v>
       </c>
       <c r="L170" t="n">
+        <v>0</v>
+      </c>
+      <c r="M170" t="n">
         <v>34</v>
       </c>
     </row>
@@ -7275,6 +7787,9 @@
         <v>0</v>
       </c>
       <c r="L171" t="n">
+        <v>0</v>
+      </c>
+      <c r="M171" t="n">
         <v>32</v>
       </c>
     </row>
@@ -7315,6 +7830,9 @@
         <v>0</v>
       </c>
       <c r="L172" t="n">
+        <v>0</v>
+      </c>
+      <c r="M172" t="n">
         <v>137</v>
       </c>
     </row>
@@ -7355,6 +7873,9 @@
         <v>0</v>
       </c>
       <c r="L173" t="n">
+        <v>0</v>
+      </c>
+      <c r="M173" t="n">
         <v>40</v>
       </c>
     </row>
@@ -7395,6 +7916,9 @@
         <v>0</v>
       </c>
       <c r="L174" t="n">
+        <v>0</v>
+      </c>
+      <c r="M174" t="n">
         <v>119</v>
       </c>
     </row>
@@ -7435,6 +7959,9 @@
         <v>0</v>
       </c>
       <c r="L175" t="n">
+        <v>0</v>
+      </c>
+      <c r="M175" t="n">
         <v>40</v>
       </c>
     </row>
@@ -7475,6 +8002,9 @@
         <v>0</v>
       </c>
       <c r="L176" t="n">
+        <v>0</v>
+      </c>
+      <c r="M176" t="n">
         <v>70</v>
       </c>
     </row>
@@ -7515,6 +8045,9 @@
         <v>0</v>
       </c>
       <c r="L177" t="n">
+        <v>0</v>
+      </c>
+      <c r="M177" t="n">
         <v>73</v>
       </c>
     </row>
@@ -7555,6 +8088,9 @@
         <v>0</v>
       </c>
       <c r="L178" t="n">
+        <v>0</v>
+      </c>
+      <c r="M178" t="n">
         <v>50</v>
       </c>
     </row>
@@ -7595,6 +8131,9 @@
         <v>0</v>
       </c>
       <c r="L179" t="n">
+        <v>0</v>
+      </c>
+      <c r="M179" t="n">
         <v>71</v>
       </c>
     </row>
@@ -7635,6 +8174,9 @@
         <v>0</v>
       </c>
       <c r="L180" t="n">
+        <v>0</v>
+      </c>
+      <c r="M180" t="n">
         <v>126</v>
       </c>
     </row>
@@ -7675,6 +8217,9 @@
         <v>0</v>
       </c>
       <c r="L181" t="n">
+        <v>0</v>
+      </c>
+      <c r="M181" t="n">
         <v>115</v>
       </c>
     </row>
@@ -7715,6 +8260,9 @@
         <v>0</v>
       </c>
       <c r="L182" t="n">
+        <v>0</v>
+      </c>
+      <c r="M182" t="n">
         <v>38</v>
       </c>
     </row>
@@ -7755,6 +8303,9 @@
         <v>0</v>
       </c>
       <c r="L183" t="n">
+        <v>0</v>
+      </c>
+      <c r="M183" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7795,6 +8346,9 @@
         <v>0</v>
       </c>
       <c r="L184" t="n">
+        <v>0</v>
+      </c>
+      <c r="M184" t="n">
         <v>138</v>
       </c>
     </row>
@@ -7835,6 +8389,9 @@
         <v>0</v>
       </c>
       <c r="L185" t="n">
+        <v>0</v>
+      </c>
+      <c r="M185" t="n">
         <v>129</v>
       </c>
     </row>
@@ -7875,6 +8432,9 @@
         <v>0</v>
       </c>
       <c r="L186" t="n">
+        <v>0</v>
+      </c>
+      <c r="M186" t="n">
         <v>50</v>
       </c>
     </row>
@@ -7915,6 +8475,9 @@
         <v>0</v>
       </c>
       <c r="L187" t="n">
+        <v>0</v>
+      </c>
+      <c r="M187" t="n">
         <v>68</v>
       </c>
     </row>
@@ -7955,6 +8518,9 @@
         <v>0</v>
       </c>
       <c r="L188" t="n">
+        <v>0</v>
+      </c>
+      <c r="M188" t="n">
         <v>33</v>
       </c>
     </row>
@@ -7995,6 +8561,9 @@
         <v>0</v>
       </c>
       <c r="L189" t="n">
+        <v>0</v>
+      </c>
+      <c r="M189" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8035,6 +8604,9 @@
         <v>0</v>
       </c>
       <c r="L190" t="n">
+        <v>0</v>
+      </c>
+      <c r="M190" t="n">
         <v>133</v>
       </c>
     </row>
@@ -8075,6 +8647,9 @@
         <v>0</v>
       </c>
       <c r="L191" t="n">
+        <v>0</v>
+      </c>
+      <c r="M191" t="n">
         <v>125</v>
       </c>
     </row>
@@ -8115,6 +8690,9 @@
         <v>0</v>
       </c>
       <c r="L192" t="n">
+        <v>0</v>
+      </c>
+      <c r="M192" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8155,6 +8733,9 @@
         <v>0</v>
       </c>
       <c r="L193" t="n">
+        <v>0</v>
+      </c>
+      <c r="M193" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8195,6 +8776,9 @@
         <v>0</v>
       </c>
       <c r="L194" t="n">
+        <v>0</v>
+      </c>
+      <c r="M194" t="n">
         <v>58</v>
       </c>
     </row>
@@ -8235,6 +8819,9 @@
         <v>0</v>
       </c>
       <c r="L195" t="n">
+        <v>0</v>
+      </c>
+      <c r="M195" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8275,6 +8862,9 @@
         <v>0</v>
       </c>
       <c r="L196" t="n">
+        <v>0</v>
+      </c>
+      <c r="M196" t="n">
         <v>104</v>
       </c>
     </row>
@@ -8315,6 +8905,9 @@
         <v>0</v>
       </c>
       <c r="L197" t="n">
+        <v>0</v>
+      </c>
+      <c r="M197" t="n">
         <v>63</v>
       </c>
     </row>
@@ -8355,6 +8948,9 @@
         <v>0</v>
       </c>
       <c r="L198" t="n">
+        <v>0</v>
+      </c>
+      <c r="M198" t="n">
         <v>62</v>
       </c>
     </row>
@@ -8395,6 +8991,9 @@
         <v>0</v>
       </c>
       <c r="L199" t="n">
+        <v>0</v>
+      </c>
+      <c r="M199" t="n">
         <v>58</v>
       </c>
     </row>
@@ -8435,6 +9034,9 @@
         <v>0</v>
       </c>
       <c r="L200" t="n">
+        <v>0</v>
+      </c>
+      <c r="M200" t="n">
         <v>45</v>
       </c>
     </row>
@@ -8475,6 +9077,9 @@
         <v>0</v>
       </c>
       <c r="L201" t="n">
+        <v>0</v>
+      </c>
+      <c r="M201" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8515,6 +9120,9 @@
         <v>0</v>
       </c>
       <c r="L202" t="n">
+        <v>0</v>
+      </c>
+      <c r="M202" t="n">
         <v>182</v>
       </c>
     </row>
@@ -8555,6 +9163,9 @@
         <v>0</v>
       </c>
       <c r="L203" t="n">
+        <v>0</v>
+      </c>
+      <c r="M203" t="n">
         <v>4</v>
       </c>
     </row>
@@ -8595,6 +9206,9 @@
         <v>0</v>
       </c>
       <c r="L204" t="n">
+        <v>0</v>
+      </c>
+      <c r="M204" t="n">
         <v>105</v>
       </c>
     </row>
@@ -8635,6 +9249,9 @@
         <v>0</v>
       </c>
       <c r="L205" t="n">
+        <v>0</v>
+      </c>
+      <c r="M205" t="n">
         <v>102</v>
       </c>
     </row>
@@ -8675,6 +9292,9 @@
         <v>0</v>
       </c>
       <c r="L206" t="n">
+        <v>0</v>
+      </c>
+      <c r="M206" t="n">
         <v>28</v>
       </c>
     </row>
@@ -8715,6 +9335,9 @@
         <v>0</v>
       </c>
       <c r="L207" t="n">
+        <v>0</v>
+      </c>
+      <c r="M207" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8755,6 +9378,9 @@
         <v>0</v>
       </c>
       <c r="L208" t="n">
+        <v>0</v>
+      </c>
+      <c r="M208" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8795,6 +9421,9 @@
         <v>0</v>
       </c>
       <c r="L209" t="n">
+        <v>0</v>
+      </c>
+      <c r="M209" t="n">
         <v>15</v>
       </c>
     </row>
@@ -8835,6 +9464,9 @@
         <v>0</v>
       </c>
       <c r="L210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M210" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8875,6 +9507,9 @@
         <v>0</v>
       </c>
       <c r="L211" t="n">
+        <v>0</v>
+      </c>
+      <c r="M211" t="n">
         <v>24</v>
       </c>
     </row>
@@ -8915,6 +9550,9 @@
         <v>0</v>
       </c>
       <c r="L212" t="n">
+        <v>0</v>
+      </c>
+      <c r="M212" t="n">
         <v>21</v>
       </c>
     </row>
@@ -8955,6 +9593,9 @@
         <v>0</v>
       </c>
       <c r="L213" t="n">
+        <v>0</v>
+      </c>
+      <c r="M213" t="n">
         <v>17</v>
       </c>
     </row>
@@ -8995,6 +9636,9 @@
         <v>0</v>
       </c>
       <c r="L214" t="n">
+        <v>0</v>
+      </c>
+      <c r="M214" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9035,6 +9679,9 @@
         <v>0</v>
       </c>
       <c r="L215" t="n">
+        <v>0</v>
+      </c>
+      <c r="M215" t="n">
         <v>22</v>
       </c>
     </row>
@@ -9075,6 +9722,9 @@
         <v>0</v>
       </c>
       <c r="L216" t="n">
+        <v>0</v>
+      </c>
+      <c r="M216" t="n">
         <v>27</v>
       </c>
     </row>
@@ -9115,6 +9765,9 @@
         <v>0</v>
       </c>
       <c r="L217" t="n">
+        <v>0</v>
+      </c>
+      <c r="M217" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9155,6 +9808,9 @@
         <v>0</v>
       </c>
       <c r="L218" t="n">
+        <v>0</v>
+      </c>
+      <c r="M218" t="n">
         <v>53</v>
       </c>
     </row>
@@ -9195,6 +9851,9 @@
         <v>0</v>
       </c>
       <c r="L219" t="n">
+        <v>0</v>
+      </c>
+      <c r="M219" t="n">
         <v>33</v>
       </c>
     </row>
@@ -9235,6 +9894,9 @@
         <v>0</v>
       </c>
       <c r="L220" t="n">
+        <v>0</v>
+      </c>
+      <c r="M220" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9275,6 +9937,9 @@
         <v>0</v>
       </c>
       <c r="L221" t="n">
+        <v>0</v>
+      </c>
+      <c r="M221" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9315,6 +9980,9 @@
         <v>0</v>
       </c>
       <c r="L222" t="n">
+        <v>0</v>
+      </c>
+      <c r="M222" t="n">
         <v>59</v>
       </c>
     </row>
@@ -9355,6 +10023,9 @@
         <v>0</v>
       </c>
       <c r="L223" t="n">
+        <v>0</v>
+      </c>
+      <c r="M223" t="n">
         <v>29</v>
       </c>
     </row>
@@ -9395,6 +10066,9 @@
         <v>0</v>
       </c>
       <c r="L224" t="n">
+        <v>0</v>
+      </c>
+      <c r="M224" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9435,6 +10109,9 @@
         <v>0</v>
       </c>
       <c r="L225" t="n">
+        <v>0</v>
+      </c>
+      <c r="M225" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9475,6 +10152,9 @@
         <v>0</v>
       </c>
       <c r="L226" t="n">
+        <v>0</v>
+      </c>
+      <c r="M226" t="n">
         <v>23</v>
       </c>
     </row>
@@ -9515,6 +10195,9 @@
         <v>0</v>
       </c>
       <c r="L227" t="n">
+        <v>0</v>
+      </c>
+      <c r="M227" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9555,6 +10238,9 @@
         <v>0</v>
       </c>
       <c r="L228" t="n">
+        <v>0</v>
+      </c>
+      <c r="M228" t="n">
         <v>48</v>
       </c>
     </row>
@@ -9595,6 +10281,9 @@
         <v>0</v>
       </c>
       <c r="L229" t="n">
+        <v>0</v>
+      </c>
+      <c r="M229" t="n">
         <v>39</v>
       </c>
     </row>
@@ -9635,6 +10324,9 @@
         <v>0</v>
       </c>
       <c r="L230" t="n">
+        <v>0</v>
+      </c>
+      <c r="M230" t="n">
         <v>41</v>
       </c>
     </row>
@@ -9675,6 +10367,9 @@
         <v>0</v>
       </c>
       <c r="L231" t="n">
+        <v>0</v>
+      </c>
+      <c r="M231" t="n">
         <v>65</v>
       </c>
     </row>
@@ -9715,6 +10410,9 @@
         <v>0</v>
       </c>
       <c r="L232" t="n">
+        <v>0</v>
+      </c>
+      <c r="M232" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9755,6 +10453,9 @@
         <v>0</v>
       </c>
       <c r="L233" t="n">
+        <v>0</v>
+      </c>
+      <c r="M233" t="n">
         <v>89</v>
       </c>
     </row>
@@ -9795,6 +10496,9 @@
         <v>0</v>
       </c>
       <c r="L234" t="n">
+        <v>0</v>
+      </c>
+      <c r="M234" t="n">
         <v>58</v>
       </c>
     </row>
@@ -9835,6 +10539,9 @@
         <v>0</v>
       </c>
       <c r="L235" t="n">
+        <v>0</v>
+      </c>
+      <c r="M235" t="n">
         <v>73</v>
       </c>
     </row>
@@ -9875,6 +10582,9 @@
         <v>0</v>
       </c>
       <c r="L236" t="n">
+        <v>0</v>
+      </c>
+      <c r="M236" t="n">
         <v>199</v>
       </c>
     </row>
@@ -9915,6 +10625,9 @@
         <v>0</v>
       </c>
       <c r="L237" t="n">
+        <v>0</v>
+      </c>
+      <c r="M237" t="n">
         <v>94</v>
       </c>
     </row>
@@ -9955,6 +10668,9 @@
         <v>0</v>
       </c>
       <c r="L238" t="n">
+        <v>0</v>
+      </c>
+      <c r="M238" t="n">
         <v>139</v>
       </c>
     </row>
@@ -9995,6 +10711,9 @@
         <v>0</v>
       </c>
       <c r="L239" t="n">
+        <v>0</v>
+      </c>
+      <c r="M239" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10035,6 +10754,9 @@
         <v>0</v>
       </c>
       <c r="L240" t="n">
+        <v>0</v>
+      </c>
+      <c r="M240" t="n">
         <v>168</v>
       </c>
     </row>
@@ -10075,6 +10797,9 @@
         <v>0</v>
       </c>
       <c r="L241" t="n">
+        <v>0</v>
+      </c>
+      <c r="M241" t="n">
         <v>71</v>
       </c>
     </row>
@@ -10115,6 +10840,9 @@
         <v>0</v>
       </c>
       <c r="L242" t="n">
+        <v>0</v>
+      </c>
+      <c r="M242" t="n">
         <v>77</v>
       </c>
     </row>
@@ -10155,6 +10883,9 @@
         <v>0</v>
       </c>
       <c r="L243" t="n">
+        <v>0</v>
+      </c>
+      <c r="M243" t="n">
         <v>46</v>
       </c>
     </row>
@@ -10195,6 +10926,9 @@
         <v>0</v>
       </c>
       <c r="L244" t="n">
+        <v>0</v>
+      </c>
+      <c r="M244" t="n">
         <v>42</v>
       </c>
     </row>
@@ -10235,6 +10969,9 @@
         <v>0</v>
       </c>
       <c r="L245" t="n">
+        <v>0</v>
+      </c>
+      <c r="M245" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10275,6 +11012,9 @@
         <v>0</v>
       </c>
       <c r="L246" t="n">
+        <v>0</v>
+      </c>
+      <c r="M246" t="n">
         <v>204</v>
       </c>
     </row>
@@ -10315,6 +11055,9 @@
         <v>0</v>
       </c>
       <c r="L247" t="n">
+        <v>0</v>
+      </c>
+      <c r="M247" t="n">
         <v>50</v>
       </c>
     </row>
@@ -10355,6 +11098,9 @@
         <v>0</v>
       </c>
       <c r="L248" t="n">
+        <v>0</v>
+      </c>
+      <c r="M248" t="n">
         <v>32</v>
       </c>
     </row>
@@ -10395,6 +11141,9 @@
         <v>0</v>
       </c>
       <c r="L249" t="n">
+        <v>0</v>
+      </c>
+      <c r="M249" t="n">
         <v>61</v>
       </c>
     </row>
@@ -10435,6 +11184,9 @@
         <v>0</v>
       </c>
       <c r="L250" t="n">
+        <v>0</v>
+      </c>
+      <c r="M250" t="n">
         <v>43</v>
       </c>
     </row>
@@ -10475,6 +11227,9 @@
         <v>0</v>
       </c>
       <c r="L251" t="n">
+        <v>0</v>
+      </c>
+      <c r="M251" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10515,6 +11270,9 @@
         <v>0</v>
       </c>
       <c r="L252" t="n">
+        <v>0</v>
+      </c>
+      <c r="M252" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10555,6 +11313,9 @@
         <v>0</v>
       </c>
       <c r="L253" t="n">
+        <v>0</v>
+      </c>
+      <c r="M253" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10595,6 +11356,9 @@
         <v>0</v>
       </c>
       <c r="L254" t="n">
+        <v>0</v>
+      </c>
+      <c r="M254" t="n">
         <v>60</v>
       </c>
     </row>
@@ -10635,6 +11399,9 @@
         <v>0</v>
       </c>
       <c r="L255" t="n">
+        <v>0</v>
+      </c>
+      <c r="M255" t="n">
         <v>152</v>
       </c>
     </row>
@@ -10675,6 +11442,9 @@
         <v>0</v>
       </c>
       <c r="L256" t="n">
+        <v>0</v>
+      </c>
+      <c r="M256" t="n">
         <v>236</v>
       </c>
     </row>
@@ -10715,6 +11485,9 @@
         <v>0</v>
       </c>
       <c r="L257" t="n">
+        <v>0</v>
+      </c>
+      <c r="M257" t="n">
         <v>72</v>
       </c>
     </row>
@@ -10755,6 +11528,9 @@
         <v>0</v>
       </c>
       <c r="L258" t="n">
+        <v>0</v>
+      </c>
+      <c r="M258" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10795,6 +11571,9 @@
         <v>0</v>
       </c>
       <c r="L259" t="n">
+        <v>0</v>
+      </c>
+      <c r="M259" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10835,6 +11614,9 @@
         <v>0</v>
       </c>
       <c r="L260" t="n">
+        <v>0</v>
+      </c>
+      <c r="M260" t="n">
         <v>295</v>
       </c>
     </row>
@@ -10875,6 +11657,9 @@
         <v>0</v>
       </c>
       <c r="L261" t="n">
+        <v>0</v>
+      </c>
+      <c r="M261" t="n">
         <v>1170</v>
       </c>
     </row>
@@ -10915,6 +11700,9 @@
         <v>0</v>
       </c>
       <c r="L262" t="n">
+        <v>0</v>
+      </c>
+      <c r="M262" t="n">
         <v>161</v>
       </c>
     </row>
@@ -10955,6 +11743,9 @@
         <v>0</v>
       </c>
       <c r="L263" t="n">
+        <v>0</v>
+      </c>
+      <c r="M263" t="n">
         <v>173</v>
       </c>
     </row>
@@ -10995,6 +11786,9 @@
         <v>0</v>
       </c>
       <c r="L264" t="n">
+        <v>0</v>
+      </c>
+      <c r="M264" t="n">
         <v>192</v>
       </c>
     </row>
@@ -11035,6 +11829,9 @@
         <v>0</v>
       </c>
       <c r="L265" t="n">
+        <v>0</v>
+      </c>
+      <c r="M265" t="n">
         <v>269</v>
       </c>
     </row>
@@ -11075,6 +11872,9 @@
         <v>0</v>
       </c>
       <c r="L266" t="n">
+        <v>0</v>
+      </c>
+      <c r="M266" t="n">
         <v>61</v>
       </c>
     </row>
@@ -11115,6 +11915,9 @@
         <v>0</v>
       </c>
       <c r="L267" t="n">
+        <v>0</v>
+      </c>
+      <c r="M267" t="n">
         <v>135</v>
       </c>
     </row>
@@ -11155,6 +11958,9 @@
         <v>0</v>
       </c>
       <c r="L268" t="n">
+        <v>0</v>
+      </c>
+      <c r="M268" t="n">
         <v>67</v>
       </c>
     </row>
@@ -11195,6 +12001,9 @@
         <v>0</v>
       </c>
       <c r="L269" t="n">
+        <v>0</v>
+      </c>
+      <c r="M269" t="n">
         <v>12</v>
       </c>
     </row>
@@ -11235,6 +12044,9 @@
         <v>0</v>
       </c>
       <c r="L270" t="n">
+        <v>0</v>
+      </c>
+      <c r="M270" t="n">
         <v>64</v>
       </c>
     </row>
@@ -11275,6 +12087,9 @@
         <v>0</v>
       </c>
       <c r="L271" t="n">
+        <v>0</v>
+      </c>
+      <c r="M271" t="n">
         <v>49</v>
       </c>
     </row>
@@ -11315,6 +12130,9 @@
         <v>0</v>
       </c>
       <c r="L272" t="n">
+        <v>0</v>
+      </c>
+      <c r="M272" t="n">
         <v>26</v>
       </c>
     </row>
@@ -11355,6 +12173,9 @@
         <v>0</v>
       </c>
       <c r="L273" t="n">
+        <v>0</v>
+      </c>
+      <c r="M273" t="n">
         <v>30</v>
       </c>
     </row>
@@ -11395,6 +12216,9 @@
         <v>0</v>
       </c>
       <c r="L274" t="n">
+        <v>0</v>
+      </c>
+      <c r="M274" t="n">
         <v>233</v>
       </c>
     </row>
@@ -11435,6 +12259,9 @@
         <v>0</v>
       </c>
       <c r="L275" t="n">
+        <v>0</v>
+      </c>
+      <c r="M275" t="n">
         <v>274</v>
       </c>
     </row>
@@ -11475,6 +12302,9 @@
         <v>0</v>
       </c>
       <c r="L276" t="n">
+        <v>0</v>
+      </c>
+      <c r="M276" t="n">
         <v>85</v>
       </c>
     </row>
@@ -11515,6 +12345,9 @@
         <v>3</v>
       </c>
       <c r="L277" t="n">
+        <v>0</v>
+      </c>
+      <c r="M277" t="n">
         <v>103</v>
       </c>
     </row>
@@ -11555,6 +12388,9 @@
         <v>0</v>
       </c>
       <c r="L278" t="n">
+        <v>0</v>
+      </c>
+      <c r="M278" t="n">
         <v>93</v>
       </c>
     </row>
@@ -11595,6 +12431,9 @@
         <v>2</v>
       </c>
       <c r="L279" t="n">
+        <v>0</v>
+      </c>
+      <c r="M279" t="n">
         <v>5</v>
       </c>
     </row>
@@ -11635,6 +12474,9 @@
         <v>1</v>
       </c>
       <c r="L280" t="n">
+        <v>0</v>
+      </c>
+      <c r="M280" t="n">
         <v>146</v>
       </c>
     </row>
@@ -11675,6 +12517,9 @@
         <v>0</v>
       </c>
       <c r="L281" t="n">
+        <v>0</v>
+      </c>
+      <c r="M281" t="n">
         <v>155</v>
       </c>
     </row>
@@ -11715,6 +12560,9 @@
         <v>2</v>
       </c>
       <c r="L282" t="n">
+        <v>0</v>
+      </c>
+      <c r="M282" t="n">
         <v>104</v>
       </c>
     </row>
@@ -11755,6 +12603,9 @@
         <v>1</v>
       </c>
       <c r="L283" t="n">
+        <v>0</v>
+      </c>
+      <c r="M283" t="n">
         <v>104</v>
       </c>
     </row>
@@ -11795,6 +12646,9 @@
         <v>1</v>
       </c>
       <c r="L284" t="n">
+        <v>0</v>
+      </c>
+      <c r="M284" t="n">
         <v>101</v>
       </c>
     </row>
@@ -11835,6 +12689,9 @@
         <v>5</v>
       </c>
       <c r="L285" t="n">
+        <v>0</v>
+      </c>
+      <c r="M285" t="n">
         <v>122</v>
       </c>
     </row>
@@ -11875,6 +12732,9 @@
         <v>1</v>
       </c>
       <c r="L286" t="n">
+        <v>0</v>
+      </c>
+      <c r="M286" t="n">
         <v>297</v>
       </c>
     </row>
@@ -11915,6 +12775,9 @@
         <v>3</v>
       </c>
       <c r="L287" t="n">
+        <v>0</v>
+      </c>
+      <c r="M287" t="n">
         <v>30</v>
       </c>
     </row>
@@ -11955,6 +12818,9 @@
         <v>2</v>
       </c>
       <c r="L288" t="n">
+        <v>0</v>
+      </c>
+      <c r="M288" t="n">
         <v>38</v>
       </c>
     </row>
@@ -11995,6 +12861,9 @@
         <v>3</v>
       </c>
       <c r="L289" t="n">
+        <v>0</v>
+      </c>
+      <c r="M289" t="n">
         <v>110</v>
       </c>
     </row>
@@ -12035,6 +12904,9 @@
         <v>2</v>
       </c>
       <c r="L290" t="n">
+        <v>0</v>
+      </c>
+      <c r="M290" t="n">
         <v>311</v>
       </c>
     </row>
@@ -12075,6 +12947,9 @@
         <v>3</v>
       </c>
       <c r="L291" t="n">
+        <v>0</v>
+      </c>
+      <c r="M291" t="n">
         <v>129</v>
       </c>
     </row>
@@ -12115,6 +12990,9 @@
         <v>1</v>
       </c>
       <c r="L292" t="n">
+        <v>0</v>
+      </c>
+      <c r="M292" t="n">
         <v>26</v>
       </c>
     </row>
@@ -12155,6 +13033,9 @@
         <v>0</v>
       </c>
       <c r="L293" t="n">
+        <v>0</v>
+      </c>
+      <c r="M293" t="n">
         <v>25</v>
       </c>
     </row>
@@ -12195,6 +13076,9 @@
         <v>0</v>
       </c>
       <c r="L294" t="n">
+        <v>0</v>
+      </c>
+      <c r="M294" t="n">
         <v>14</v>
       </c>
     </row>
@@ -12235,6 +13119,9 @@
         <v>0</v>
       </c>
       <c r="L295" t="n">
+        <v>0</v>
+      </c>
+      <c r="M295" t="n">
         <v>146</v>
       </c>
     </row>
@@ -12275,6 +13162,9 @@
         <v>0</v>
       </c>
       <c r="L296" t="n">
+        <v>0</v>
+      </c>
+      <c r="M296" t="n">
         <v>130</v>
       </c>
     </row>
@@ -12315,6 +13205,9 @@
         <v>0</v>
       </c>
       <c r="L297" t="n">
+        <v>0</v>
+      </c>
+      <c r="M297" t="n">
         <v>52</v>
       </c>
     </row>
@@ -12355,6 +13248,9 @@
         <v>0</v>
       </c>
       <c r="L298" t="n">
+        <v>0</v>
+      </c>
+      <c r="M298" t="n">
         <v>21</v>
       </c>
     </row>
@@ -12395,6 +13291,9 @@
         <v>0</v>
       </c>
       <c r="L299" t="n">
+        <v>0</v>
+      </c>
+      <c r="M299" t="n">
         <v>46</v>
       </c>
     </row>
@@ -12435,6 +13334,9 @@
         <v>0</v>
       </c>
       <c r="L300" t="n">
+        <v>0</v>
+      </c>
+      <c r="M300" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12475,6 +13377,9 @@
         <v>0</v>
       </c>
       <c r="L301" t="n">
+        <v>0</v>
+      </c>
+      <c r="M301" t="n">
         <v>26</v>
       </c>
     </row>
@@ -12515,6 +13420,9 @@
         <v>0</v>
       </c>
       <c r="L302" t="n">
+        <v>0</v>
+      </c>
+      <c r="M302" t="n">
         <v>28</v>
       </c>
     </row>
@@ -12555,6 +13463,9 @@
         <v>0</v>
       </c>
       <c r="L303" t="n">
+        <v>0</v>
+      </c>
+      <c r="M303" t="n">
         <v>227</v>
       </c>
     </row>
@@ -12595,6 +13506,9 @@
         <v>0</v>
       </c>
       <c r="L304" t="n">
+        <v>0</v>
+      </c>
+      <c r="M304" t="n">
         <v>49</v>
       </c>
     </row>
@@ -12635,6 +13549,9 @@
         <v>0</v>
       </c>
       <c r="L305" t="n">
+        <v>0</v>
+      </c>
+      <c r="M305" t="n">
         <v>74</v>
       </c>
     </row>
@@ -12675,6 +13592,9 @@
         <v>0</v>
       </c>
       <c r="L306" t="n">
+        <v>0</v>
+      </c>
+      <c r="M306" t="n">
         <v>104</v>
       </c>
     </row>
@@ -12715,6 +13635,9 @@
         <v>0</v>
       </c>
       <c r="L307" t="n">
+        <v>0</v>
+      </c>
+      <c r="M307" t="n">
         <v>14</v>
       </c>
     </row>
@@ -12755,6 +13678,9 @@
         <v>0</v>
       </c>
       <c r="L308" t="n">
+        <v>0</v>
+      </c>
+      <c r="M308" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12795,6 +13721,9 @@
         <v>0</v>
       </c>
       <c r="L309" t="n">
+        <v>0</v>
+      </c>
+      <c r="M309" t="n">
         <v>100</v>
       </c>
     </row>
@@ -12835,6 +13764,9 @@
         <v>0</v>
       </c>
       <c r="L310" t="n">
+        <v>0</v>
+      </c>
+      <c r="M310" t="n">
         <v>126</v>
       </c>
     </row>
@@ -12875,6 +13807,9 @@
         <v>0</v>
       </c>
       <c r="L311" t="n">
+        <v>0</v>
+      </c>
+      <c r="M311" t="n">
         <v>37</v>
       </c>
     </row>
@@ -12915,6 +13850,9 @@
         <v>0</v>
       </c>
       <c r="L312" t="n">
+        <v>0</v>
+      </c>
+      <c r="M312" t="n">
         <v>283</v>
       </c>
     </row>
@@ -12955,6 +13893,9 @@
         <v>0</v>
       </c>
       <c r="L313" t="n">
+        <v>0</v>
+      </c>
+      <c r="M313" t="n">
         <v>393</v>
       </c>
     </row>
@@ -12995,6 +13936,9 @@
         <v>0</v>
       </c>
       <c r="L314" t="n">
+        <v>0</v>
+      </c>
+      <c r="M314" t="n">
         <v>373</v>
       </c>
     </row>
@@ -13035,6 +13979,9 @@
         <v>0</v>
       </c>
       <c r="L315" t="n">
+        <v>0</v>
+      </c>
+      <c r="M315" t="n">
         <v>204</v>
       </c>
     </row>
@@ -13075,6 +14022,9 @@
         <v>0</v>
       </c>
       <c r="L316" t="n">
+        <v>0</v>
+      </c>
+      <c r="M316" t="n">
         <v>95</v>
       </c>
     </row>
@@ -13115,6 +14065,9 @@
         <v>0</v>
       </c>
       <c r="L317" t="n">
+        <v>0</v>
+      </c>
+      <c r="M317" t="n">
         <v>110</v>
       </c>
     </row>
@@ -13155,6 +14108,9 @@
         <v>0</v>
       </c>
       <c r="L318" t="n">
+        <v>0</v>
+      </c>
+      <c r="M318" t="n">
         <v>109</v>
       </c>
     </row>
@@ -13195,6 +14151,9 @@
         <v>0</v>
       </c>
       <c r="L319" t="n">
+        <v>0</v>
+      </c>
+      <c r="M319" t="n">
         <v>31</v>
       </c>
     </row>
@@ -13235,6 +14194,9 @@
         <v>0</v>
       </c>
       <c r="L320" t="n">
+        <v>0</v>
+      </c>
+      <c r="M320" t="n">
         <v>34</v>
       </c>
     </row>
@@ -13275,6 +14237,9 @@
         <v>0</v>
       </c>
       <c r="L321" t="n">
+        <v>0</v>
+      </c>
+      <c r="M321" t="n">
         <v>46</v>
       </c>
     </row>
@@ -13315,6 +14280,9 @@
         <v>0</v>
       </c>
       <c r="L322" t="n">
+        <v>0</v>
+      </c>
+      <c r="M322" t="n">
         <v>23</v>
       </c>
     </row>
@@ -13355,6 +14323,9 @@
         <v>0</v>
       </c>
       <c r="L323" t="n">
+        <v>0</v>
+      </c>
+      <c r="M323" t="n">
         <v>15</v>
       </c>
     </row>
@@ -13395,6 +14366,9 @@
         <v>0</v>
       </c>
       <c r="L324" t="n">
+        <v>0</v>
+      </c>
+      <c r="M324" t="n">
         <v>32</v>
       </c>
     </row>
@@ -13435,6 +14409,9 @@
         <v>0</v>
       </c>
       <c r="L325" t="n">
+        <v>0</v>
+      </c>
+      <c r="M325" t="n">
         <v>31</v>
       </c>
     </row>
@@ -13475,6 +14452,9 @@
         <v>0</v>
       </c>
       <c r="L326" t="n">
+        <v>0</v>
+      </c>
+      <c r="M326" t="n">
         <v>46</v>
       </c>
     </row>
@@ -13515,6 +14495,9 @@
         <v>0</v>
       </c>
       <c r="L327" t="n">
+        <v>0</v>
+      </c>
+      <c r="M327" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13555,6 +14538,9 @@
         <v>0</v>
       </c>
       <c r="L328" t="n">
+        <v>0</v>
+      </c>
+      <c r="M328" t="n">
         <v>23</v>
       </c>
     </row>
@@ -13595,6 +14581,9 @@
         <v>0</v>
       </c>
       <c r="L329" t="n">
+        <v>0</v>
+      </c>
+      <c r="M329" t="n">
         <v>19</v>
       </c>
     </row>
@@ -13635,6 +14624,9 @@
         <v>0</v>
       </c>
       <c r="L330" t="n">
+        <v>0</v>
+      </c>
+      <c r="M330" t="n">
         <v>71</v>
       </c>
     </row>
@@ -13675,6 +14667,9 @@
         <v>0</v>
       </c>
       <c r="L331" t="n">
+        <v>0</v>
+      </c>
+      <c r="M331" t="n">
         <v>149</v>
       </c>
     </row>
@@ -13715,6 +14710,9 @@
         <v>0</v>
       </c>
       <c r="L332" t="n">
+        <v>0</v>
+      </c>
+      <c r="M332" t="n">
         <v>53</v>
       </c>
     </row>
@@ -13755,6 +14753,9 @@
         <v>0</v>
       </c>
       <c r="L333" t="n">
+        <v>0</v>
+      </c>
+      <c r="M333" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13795,6 +14796,9 @@
         <v>0</v>
       </c>
       <c r="L334" t="n">
+        <v>0</v>
+      </c>
+      <c r="M334" t="n">
         <v>34</v>
       </c>
     </row>
@@ -13835,6 +14839,9 @@
         <v>0</v>
       </c>
       <c r="L335" t="n">
+        <v>0</v>
+      </c>
+      <c r="M335" t="n">
         <v>4</v>
       </c>
     </row>
@@ -13875,6 +14882,9 @@
         <v>0</v>
       </c>
       <c r="L336" t="n">
+        <v>0</v>
+      </c>
+      <c r="M336" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13915,6 +14925,9 @@
         <v>0</v>
       </c>
       <c r="L337" t="n">
+        <v>0</v>
+      </c>
+      <c r="M337" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13955,6 +14968,9 @@
         <v>0</v>
       </c>
       <c r="L338" t="n">
+        <v>0</v>
+      </c>
+      <c r="M338" t="n">
         <v>54</v>
       </c>
     </row>
@@ -13995,6 +15011,9 @@
         <v>0</v>
       </c>
       <c r="L339" t="n">
+        <v>0</v>
+      </c>
+      <c r="M339" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14035,6 +15054,9 @@
         <v>0</v>
       </c>
       <c r="L340" t="n">
+        <v>0</v>
+      </c>
+      <c r="M340" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14075,6 +15097,9 @@
         <v>0</v>
       </c>
       <c r="L341" t="n">
+        <v>0</v>
+      </c>
+      <c r="M341" t="n">
         <v>15</v>
       </c>
     </row>
@@ -14115,6 +15140,9 @@
         <v>0</v>
       </c>
       <c r="L342" t="n">
+        <v>0</v>
+      </c>
+      <c r="M342" t="n">
         <v>10</v>
       </c>
     </row>
@@ -14155,6 +15183,9 @@
         <v>0</v>
       </c>
       <c r="L343" t="n">
+        <v>0</v>
+      </c>
+      <c r="M343" t="n">
         <v>6</v>
       </c>
     </row>
@@ -14195,6 +15226,9 @@
         <v>0</v>
       </c>
       <c r="L344" t="n">
+        <v>0</v>
+      </c>
+      <c r="M344" t="n">
         <v>61</v>
       </c>
     </row>
@@ -14235,6 +15269,9 @@
         <v>0</v>
       </c>
       <c r="L345" t="n">
+        <v>0</v>
+      </c>
+      <c r="M345" t="n">
         <v>73</v>
       </c>
     </row>
@@ -14275,6 +15312,9 @@
         <v>0</v>
       </c>
       <c r="L346" t="n">
+        <v>0</v>
+      </c>
+      <c r="M346" t="n">
         <v>56</v>
       </c>
     </row>
@@ -14315,6 +15355,9 @@
         <v>0</v>
       </c>
       <c r="L347" t="n">
+        <v>0</v>
+      </c>
+      <c r="M347" t="n">
         <v>26</v>
       </c>
     </row>
@@ -14355,6 +15398,9 @@
         <v>0</v>
       </c>
       <c r="L348" t="n">
+        <v>0</v>
+      </c>
+      <c r="M348" t="n">
         <v>60</v>
       </c>
     </row>
@@ -14395,6 +15441,9 @@
         <v>0</v>
       </c>
       <c r="L349" t="n">
+        <v>0</v>
+      </c>
+      <c r="M349" t="n">
         <v>31</v>
       </c>
     </row>
@@ -14435,6 +15484,9 @@
         <v>0</v>
       </c>
       <c r="L350" t="n">
+        <v>0</v>
+      </c>
+      <c r="M350" t="n">
         <v>18</v>
       </c>
     </row>
@@ -14475,7 +15527,53 @@
         <v>0</v>
       </c>
       <c r="L351" t="n">
+        <v>0</v>
+      </c>
+      <c r="M351" t="n">
         <v>61</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B352" t="n">
+        <v>15</v>
+      </c>
+      <c r="C352" t="n">
+        <v>16</v>
+      </c>
+      <c r="D352" t="n">
+        <v>7</v>
+      </c>
+      <c r="E352" t="n">
+        <v>0</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0</v>
+      </c>
+      <c r="G352" t="n">
+        <v>12</v>
+      </c>
+      <c r="H352" t="n">
+        <v>5</v>
+      </c>
+      <c r="I352" t="n">
+        <v>0</v>
+      </c>
+      <c r="J352" t="n">
+        <v>0</v>
+      </c>
+      <c r="K352" t="n">
+        <v>0</v>
+      </c>
+      <c r="L352" t="n">
+        <v>2</v>
+      </c>
+      <c r="M352" t="n">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-24 13:02
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M352"/>
+  <dimension ref="A1:M353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15576,6 +15576,49 @@
         <v>57</v>
       </c>
     </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B353" t="n">
+        <v>13</v>
+      </c>
+      <c r="C353" t="n">
+        <v>22</v>
+      </c>
+      <c r="D353" t="n">
+        <v>2</v>
+      </c>
+      <c r="E353" t="n">
+        <v>0</v>
+      </c>
+      <c r="F353" t="n">
+        <v>0</v>
+      </c>
+      <c r="G353" t="n">
+        <v>5</v>
+      </c>
+      <c r="H353" t="n">
+        <v>8</v>
+      </c>
+      <c r="I353" t="n">
+        <v>0</v>
+      </c>
+      <c r="J353" t="n">
+        <v>3</v>
+      </c>
+      <c r="K353" t="n">
+        <v>0</v>
+      </c>
+      <c r="L353" t="n">
+        <v>0</v>
+      </c>
+      <c r="M353" t="n">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-29 13:01
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M354"/>
+  <dimension ref="A1:M358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,12 +449,12 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Hibiscus</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Spearmint</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Hibiscus</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -12201,10 +12201,10 @@
         <v>0</v>
       </c>
       <c r="G274" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" t="n">
         <v>2</v>
-      </c>
-      <c r="H274" t="n">
-        <v>0</v>
       </c>
       <c r="I274" t="n">
         <v>0</v>
@@ -12244,10 +12244,10 @@
         <v>0</v>
       </c>
       <c r="G275" t="n">
+        <v>5</v>
+      </c>
+      <c r="H275" t="n">
         <v>3</v>
-      </c>
-      <c r="H275" t="n">
-        <v>5</v>
       </c>
       <c r="I275" t="n">
         <v>0</v>
@@ -12330,10 +12330,10 @@
         <v>0</v>
       </c>
       <c r="G277" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H277" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -12373,10 +12373,10 @@
         <v>0</v>
       </c>
       <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="n">
         <v>2</v>
-      </c>
-      <c r="H278" t="n">
-        <v>0</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
@@ -12502,10 +12502,10 @@
         <v>0</v>
       </c>
       <c r="G281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H281" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I281" t="n">
         <v>0</v>
@@ -12545,10 +12545,10 @@
         <v>0</v>
       </c>
       <c r="G282" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H282" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I282" t="n">
         <v>1</v>
@@ -12588,10 +12588,10 @@
         <v>0</v>
       </c>
       <c r="G283" t="n">
+        <v>1</v>
+      </c>
+      <c r="H283" t="n">
         <v>2</v>
-      </c>
-      <c r="H283" t="n">
-        <v>1</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -12631,10 +12631,10 @@
         <v>0</v>
       </c>
       <c r="G284" t="n">
+        <v>7</v>
+      </c>
+      <c r="H284" t="n">
         <v>6</v>
-      </c>
-      <c r="H284" t="n">
-        <v>7</v>
       </c>
       <c r="I284" t="n">
         <v>0</v>
@@ -12717,10 +12717,10 @@
         <v>0</v>
       </c>
       <c r="G286" t="n">
+        <v>1</v>
+      </c>
+      <c r="H286" t="n">
         <v>3</v>
-      </c>
-      <c r="H286" t="n">
-        <v>1</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -12803,10 +12803,10 @@
         <v>0</v>
       </c>
       <c r="G288" t="n">
+        <v>1</v>
+      </c>
+      <c r="H288" t="n">
         <v>2</v>
-      </c>
-      <c r="H288" t="n">
-        <v>1</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -12846,10 +12846,10 @@
         <v>0</v>
       </c>
       <c r="G289" t="n">
+        <v>7</v>
+      </c>
+      <c r="H289" t="n">
         <v>5</v>
-      </c>
-      <c r="H289" t="n">
-        <v>7</v>
       </c>
       <c r="I289" t="n">
         <v>0</v>
@@ -12889,10 +12889,10 @@
         <v>0</v>
       </c>
       <c r="G290" t="n">
+        <v>6</v>
+      </c>
+      <c r="H290" t="n">
         <v>3</v>
-      </c>
-      <c r="H290" t="n">
-        <v>6</v>
       </c>
       <c r="I290" t="n">
         <v>0</v>
@@ -12975,10 +12975,10 @@
         <v>0</v>
       </c>
       <c r="G292" t="n">
+        <v>3</v>
+      </c>
+      <c r="H292" t="n">
         <v>2</v>
-      </c>
-      <c r="H292" t="n">
-        <v>3</v>
       </c>
       <c r="I292" t="n">
         <v>0</v>
@@ -13104,10 +13104,10 @@
         <v>0</v>
       </c>
       <c r="G295" t="n">
+        <v>10</v>
+      </c>
+      <c r="H295" t="n">
         <v>6</v>
-      </c>
-      <c r="H295" t="n">
-        <v>10</v>
       </c>
       <c r="I295" t="n">
         <v>0</v>
@@ -13147,10 +13147,10 @@
         <v>0</v>
       </c>
       <c r="G296" t="n">
+        <v>8</v>
+      </c>
+      <c r="H296" t="n">
         <v>9</v>
-      </c>
-      <c r="H296" t="n">
-        <v>8</v>
       </c>
       <c r="I296" t="n">
         <v>0</v>
@@ -13190,10 +13190,10 @@
         <v>0</v>
       </c>
       <c r="G297" t="n">
+        <v>2</v>
+      </c>
+      <c r="H297" t="n">
         <v>3</v>
-      </c>
-      <c r="H297" t="n">
-        <v>2</v>
       </c>
       <c r="I297" t="n">
         <v>0</v>
@@ -13233,10 +13233,10 @@
         <v>0</v>
       </c>
       <c r="G298" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H298" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I298" t="n">
         <v>0</v>
@@ -13276,10 +13276,10 @@
         <v>0</v>
       </c>
       <c r="G299" t="n">
+        <v>2</v>
+      </c>
+      <c r="H299" t="n">
         <v>3</v>
-      </c>
-      <c r="H299" t="n">
-        <v>2</v>
       </c>
       <c r="I299" t="n">
         <v>0</v>
@@ -13448,10 +13448,10 @@
         <v>0</v>
       </c>
       <c r="G303" t="n">
+        <v>41</v>
+      </c>
+      <c r="H303" t="n">
         <v>17</v>
-      </c>
-      <c r="H303" t="n">
-        <v>41</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -13491,10 +13491,10 @@
         <v>0</v>
       </c>
       <c r="G304" t="n">
+        <v>1</v>
+      </c>
+      <c r="H304" t="n">
         <v>2</v>
-      </c>
-      <c r="H304" t="n">
-        <v>1</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -13534,10 +13534,10 @@
         <v>1</v>
       </c>
       <c r="G305" t="n">
+        <v>4</v>
+      </c>
+      <c r="H305" t="n">
         <v>2</v>
-      </c>
-      <c r="H305" t="n">
-        <v>4</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -13577,10 +13577,10 @@
         <v>6</v>
       </c>
       <c r="G306" t="n">
+        <v>3</v>
+      </c>
+      <c r="H306" t="n">
         <v>16</v>
-      </c>
-      <c r="H306" t="n">
-        <v>3</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -13620,10 +13620,10 @@
         <v>1</v>
       </c>
       <c r="G307" t="n">
+        <v>0</v>
+      </c>
+      <c r="H307" t="n">
         <v>4</v>
-      </c>
-      <c r="H307" t="n">
-        <v>0</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -13663,10 +13663,10 @@
         <v>0</v>
       </c>
       <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="n">
         <v>3</v>
-      </c>
-      <c r="H308" t="n">
-        <v>0</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -13706,10 +13706,10 @@
         <v>25</v>
       </c>
       <c r="G309" t="n">
+        <v>15</v>
+      </c>
+      <c r="H309" t="n">
         <v>18</v>
-      </c>
-      <c r="H309" t="n">
-        <v>15</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -13749,10 +13749,10 @@
         <v>13</v>
       </c>
       <c r="G310" t="n">
+        <v>30</v>
+      </c>
+      <c r="H310" t="n">
         <v>18</v>
-      </c>
-      <c r="H310" t="n">
-        <v>30</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -13835,10 +13835,10 @@
         <v>83</v>
       </c>
       <c r="G312" t="n">
+        <v>4</v>
+      </c>
+      <c r="H312" t="n">
         <v>14</v>
-      </c>
-      <c r="H312" t="n">
-        <v>4</v>
       </c>
       <c r="I312" t="n">
         <v>0</v>
@@ -13878,10 +13878,10 @@
         <v>97</v>
       </c>
       <c r="G313" t="n">
+        <v>4</v>
+      </c>
+      <c r="H313" t="n">
         <v>16</v>
-      </c>
-      <c r="H313" t="n">
-        <v>4</v>
       </c>
       <c r="I313" t="n">
         <v>0</v>
@@ -13921,10 +13921,10 @@
         <v>102</v>
       </c>
       <c r="G314" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" t="n">
         <v>7</v>
-      </c>
-      <c r="H314" t="n">
-        <v>0</v>
       </c>
       <c r="I314" t="n">
         <v>0</v>
@@ -13964,10 +13964,10 @@
         <v>60</v>
       </c>
       <c r="G315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H315" t="n">
         <v>3</v>
-      </c>
-      <c r="H315" t="n">
-        <v>0</v>
       </c>
       <c r="I315" t="n">
         <v>0</v>
@@ -14007,10 +14007,10 @@
         <v>25</v>
       </c>
       <c r="G316" t="n">
+        <v>1</v>
+      </c>
+      <c r="H316" t="n">
         <v>5</v>
-      </c>
-      <c r="H316" t="n">
-        <v>1</v>
       </c>
       <c r="I316" t="n">
         <v>0</v>
@@ -14050,10 +14050,10 @@
         <v>21</v>
       </c>
       <c r="G317" t="n">
+        <v>3</v>
+      </c>
+      <c r="H317" t="n">
         <v>2</v>
-      </c>
-      <c r="H317" t="n">
-        <v>3</v>
       </c>
       <c r="I317" t="n">
         <v>0</v>
@@ -14093,10 +14093,10 @@
         <v>17</v>
       </c>
       <c r="G318" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H318" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I318" t="n">
         <v>0</v>
@@ -14136,10 +14136,10 @@
         <v>8</v>
       </c>
       <c r="G319" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I319" t="n">
         <v>0</v>
@@ -14179,10 +14179,10 @@
         <v>4</v>
       </c>
       <c r="G320" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I320" t="n">
         <v>0</v>
@@ -14222,10 +14222,10 @@
         <v>10</v>
       </c>
       <c r="G321" t="n">
+        <v>1</v>
+      </c>
+      <c r="H321" t="n">
         <v>2</v>
-      </c>
-      <c r="H321" t="n">
-        <v>1</v>
       </c>
       <c r="I321" t="n">
         <v>0</v>
@@ -14265,10 +14265,10 @@
         <v>5</v>
       </c>
       <c r="G322" t="n">
+        <v>0</v>
+      </c>
+      <c r="H322" t="n">
         <v>2</v>
-      </c>
-      <c r="H322" t="n">
-        <v>0</v>
       </c>
       <c r="I322" t="n">
         <v>0</v>
@@ -14437,10 +14437,10 @@
         <v>10</v>
       </c>
       <c r="G326" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H326" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I326" t="n">
         <v>0</v>
@@ -14480,10 +14480,10 @@
         <v>2</v>
       </c>
       <c r="G327" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I327" t="n">
         <v>0</v>
@@ -14609,10 +14609,10 @@
         <v>6</v>
       </c>
       <c r="G330" t="n">
+        <v>5</v>
+      </c>
+      <c r="H330" t="n">
         <v>2</v>
-      </c>
-      <c r="H330" t="n">
-        <v>5</v>
       </c>
       <c r="I330" t="n">
         <v>0</v>
@@ -14652,10 +14652,10 @@
         <v>1</v>
       </c>
       <c r="G331" t="n">
+        <v>1</v>
+      </c>
+      <c r="H331" t="n">
         <v>2</v>
-      </c>
-      <c r="H331" t="n">
-        <v>1</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -14695,10 +14695,10 @@
         <v>1</v>
       </c>
       <c r="G332" t="n">
+        <v>0</v>
+      </c>
+      <c r="H332" t="n">
         <v>2</v>
-      </c>
-      <c r="H332" t="n">
-        <v>0</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -14738,10 +14738,10 @@
         <v>0</v>
       </c>
       <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="n">
         <v>3</v>
-      </c>
-      <c r="H333" t="n">
-        <v>0</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -14781,10 +14781,10 @@
         <v>0</v>
       </c>
       <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="n">
         <v>5</v>
-      </c>
-      <c r="H334" t="n">
-        <v>0</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -14910,10 +14910,10 @@
         <v>0</v>
       </c>
       <c r="G337" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -14953,10 +14953,10 @@
         <v>0</v>
       </c>
       <c r="G338" t="n">
+        <v>0</v>
+      </c>
+      <c r="H338" t="n">
         <v>2</v>
-      </c>
-      <c r="H338" t="n">
-        <v>0</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -14996,10 +14996,10 @@
         <v>0</v>
       </c>
       <c r="G339" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -15168,10 +15168,10 @@
         <v>0</v>
       </c>
       <c r="G343" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -15211,10 +15211,10 @@
         <v>0</v>
       </c>
       <c r="G344" t="n">
+        <v>0</v>
+      </c>
+      <c r="H344" t="n">
         <v>2</v>
-      </c>
-      <c r="H344" t="n">
-        <v>0</v>
       </c>
       <c r="I344" t="n">
         <v>0</v>
@@ -15254,10 +15254,10 @@
         <v>0</v>
       </c>
       <c r="G345" t="n">
+        <v>0</v>
+      </c>
+      <c r="H345" t="n">
         <v>9</v>
-      </c>
-      <c r="H345" t="n">
-        <v>0</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -15297,10 +15297,10 @@
         <v>0</v>
       </c>
       <c r="G346" t="n">
+        <v>0</v>
+      </c>
+      <c r="H346" t="n">
         <v>3</v>
-      </c>
-      <c r="H346" t="n">
-        <v>0</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -15383,10 +15383,10 @@
         <v>0</v>
       </c>
       <c r="G348" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H348" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I348" t="n">
         <v>0</v>
@@ -15426,10 +15426,10 @@
         <v>0</v>
       </c>
       <c r="G349" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H349" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -15469,10 +15469,10 @@
         <v>0</v>
       </c>
       <c r="G350" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H350" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
@@ -15512,10 +15512,10 @@
         <v>0</v>
       </c>
       <c r="G351" t="n">
+        <v>5</v>
+      </c>
+      <c r="H351" t="n">
         <v>8</v>
-      </c>
-      <c r="H351" t="n">
-        <v>5</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -15555,10 +15555,10 @@
         <v>0</v>
       </c>
       <c r="G352" t="n">
+        <v>5</v>
+      </c>
+      <c r="H352" t="n">
         <v>12</v>
-      </c>
-      <c r="H352" t="n">
-        <v>5</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -15598,10 +15598,10 @@
         <v>0</v>
       </c>
       <c r="G353" t="n">
+        <v>8</v>
+      </c>
+      <c r="H353" t="n">
         <v>5</v>
-      </c>
-      <c r="H353" t="n">
-        <v>8</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -15660,6 +15660,178 @@
       </c>
       <c r="M354" t="n">
         <v>53</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B355" t="n">
+        <v>4</v>
+      </c>
+      <c r="C355" t="n">
+        <v>15</v>
+      </c>
+      <c r="D355" t="n">
+        <v>0</v>
+      </c>
+      <c r="E355" t="n">
+        <v>0</v>
+      </c>
+      <c r="F355" t="n">
+        <v>0</v>
+      </c>
+      <c r="G355" t="n">
+        <v>4</v>
+      </c>
+      <c r="H355" t="n">
+        <v>1</v>
+      </c>
+      <c r="I355" t="n">
+        <v>0</v>
+      </c>
+      <c r="J355" t="n">
+        <v>0</v>
+      </c>
+      <c r="K355" t="n">
+        <v>0</v>
+      </c>
+      <c r="L355" t="n">
+        <v>0</v>
+      </c>
+      <c r="M355" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B356" t="n">
+        <v>15</v>
+      </c>
+      <c r="C356" t="n">
+        <v>18</v>
+      </c>
+      <c r="D356" t="n">
+        <v>4</v>
+      </c>
+      <c r="E356" t="n">
+        <v>0</v>
+      </c>
+      <c r="F356" t="n">
+        <v>0</v>
+      </c>
+      <c r="G356" t="n">
+        <v>12</v>
+      </c>
+      <c r="H356" t="n">
+        <v>2</v>
+      </c>
+      <c r="I356" t="n">
+        <v>0</v>
+      </c>
+      <c r="J356" t="n">
+        <v>3</v>
+      </c>
+      <c r="K356" t="n">
+        <v>0</v>
+      </c>
+      <c r="L356" t="n">
+        <v>1</v>
+      </c>
+      <c r="M356" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B357" t="n">
+        <v>1</v>
+      </c>
+      <c r="C357" t="n">
+        <v>5</v>
+      </c>
+      <c r="D357" t="n">
+        <v>2</v>
+      </c>
+      <c r="E357" t="n">
+        <v>0</v>
+      </c>
+      <c r="F357" t="n">
+        <v>0</v>
+      </c>
+      <c r="G357" t="n">
+        <v>1</v>
+      </c>
+      <c r="H357" t="n">
+        <v>0</v>
+      </c>
+      <c r="I357" t="n">
+        <v>0</v>
+      </c>
+      <c r="J357" t="n">
+        <v>0</v>
+      </c>
+      <c r="K357" t="n">
+        <v>0</v>
+      </c>
+      <c r="L357" t="n">
+        <v>0</v>
+      </c>
+      <c r="M357" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B358" t="n">
+        <v>29</v>
+      </c>
+      <c r="C358" t="n">
+        <v>42</v>
+      </c>
+      <c r="D358" t="n">
+        <v>17</v>
+      </c>
+      <c r="E358" t="n">
+        <v>0</v>
+      </c>
+      <c r="F358" t="n">
+        <v>0</v>
+      </c>
+      <c r="G358" t="n">
+        <v>52</v>
+      </c>
+      <c r="H358" t="n">
+        <v>6</v>
+      </c>
+      <c r="I358" t="n">
+        <v>0</v>
+      </c>
+      <c r="J358" t="n">
+        <v>2</v>
+      </c>
+      <c r="K358" t="n">
+        <v>0</v>
+      </c>
+      <c r="L358" t="n">
+        <v>2</v>
+      </c>
+      <c r="M358" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-30 15:00
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M358"/>
+  <dimension ref="A1:M359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15834,6 +15834,49 @@
         <v>150</v>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B359" t="n">
+        <v>21</v>
+      </c>
+      <c r="C359" t="n">
+        <v>24</v>
+      </c>
+      <c r="D359" t="n">
+        <v>16</v>
+      </c>
+      <c r="E359" t="n">
+        <v>0</v>
+      </c>
+      <c r="F359" t="n">
+        <v>4</v>
+      </c>
+      <c r="G359" t="n">
+        <v>37</v>
+      </c>
+      <c r="H359" t="n">
+        <v>1</v>
+      </c>
+      <c r="I359" t="n">
+        <v>0</v>
+      </c>
+      <c r="J359" t="n">
+        <v>1</v>
+      </c>
+      <c r="K359" t="n">
+        <v>0</v>
+      </c>
+      <c r="L359" t="n">
+        <v>0</v>
+      </c>
+      <c r="M359" t="n">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-06 13:03
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M365"/>
+  <dimension ref="A1:M366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15927,23 +15927,23 @@
         </is>
       </c>
       <c r="B361" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C361" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="D361" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="E361" t="n">
         <v>0</v>
       </c>
       <c r="F361" t="n">
+        <v>13</v>
+      </c>
+      <c r="G361" t="n">
         <v>26</v>
       </c>
-      <c r="G361" t="n">
-        <v>52</v>
-      </c>
       <c r="H361" t="n">
         <v>0</v>
       </c>
@@ -15951,7 +15951,7 @@
         <v>0</v>
       </c>
       <c r="J361" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K361" t="n">
         <v>0</v>
@@ -15960,7 +15960,7 @@
         <v>0</v>
       </c>
       <c r="M361" t="n">
-        <v>184</v>
+        <v>92</v>
       </c>
     </row>
     <row r="362">
@@ -15970,10 +15970,10 @@
         </is>
       </c>
       <c r="B362" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C362" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D362" t="n">
         <v>0</v>
@@ -15982,7 +15982,7 @@
         <v>0</v>
       </c>
       <c r="F362" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -15994,7 +15994,7 @@
         <v>0</v>
       </c>
       <c r="J362" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K362" t="n">
         <v>0</v>
@@ -16003,7 +16003,7 @@
         <v>0</v>
       </c>
       <c r="M362" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="363">
@@ -16013,10 +16013,10 @@
         </is>
       </c>
       <c r="B363" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C363" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D363" t="n">
         <v>0</v>
@@ -16025,7 +16025,7 @@
         <v>0</v>
       </c>
       <c r="F363" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -16037,7 +16037,7 @@
         <v>0</v>
       </c>
       <c r="J363" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K363" t="n">
         <v>0</v>
@@ -16046,7 +16046,7 @@
         <v>0</v>
       </c>
       <c r="M363" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="364">
@@ -16056,22 +16056,22 @@
         </is>
       </c>
       <c r="B364" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C364" t="n">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="D364" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E364" t="n">
         <v>0</v>
       </c>
       <c r="F364" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G364" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H364" t="n">
         <v>0</v>
@@ -16080,16 +16080,16 @@
         <v>0</v>
       </c>
       <c r="J364" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K364" t="n">
         <v>0</v>
       </c>
       <c r="L364" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M364" t="n">
-        <v>118</v>
+        <v>59</v>
       </c>
     </row>
     <row r="365">
@@ -16099,22 +16099,22 @@
         </is>
       </c>
       <c r="B365" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C365" t="n">
+        <v>7</v>
+      </c>
+      <c r="D365" t="n">
+        <v>0</v>
+      </c>
+      <c r="E365" t="n">
+        <v>0</v>
+      </c>
+      <c r="F365" t="n">
         <v>2</v>
       </c>
-      <c r="D365" t="n">
-        <v>0</v>
-      </c>
-      <c r="E365" t="n">
-        <v>0</v>
-      </c>
-      <c r="F365" t="n">
-        <v>1</v>
-      </c>
       <c r="G365" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H365" t="n">
         <v>0</v>
@@ -16123,16 +16123,59 @@
         <v>0</v>
       </c>
       <c r="J365" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K365" t="n">
         <v>0</v>
       </c>
       <c r="L365" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M365" t="n">
-        <v>3</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B366" t="n">
+        <v>0</v>
+      </c>
+      <c r="C366" t="n">
+        <v>1</v>
+      </c>
+      <c r="D366" t="n">
+        <v>0</v>
+      </c>
+      <c r="E366" t="n">
+        <v>0</v>
+      </c>
+      <c r="F366" t="n">
+        <v>0</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0</v>
+      </c>
+      <c r="H366" t="n">
+        <v>0</v>
+      </c>
+      <c r="I366" t="n">
+        <v>0</v>
+      </c>
+      <c r="J366" t="n">
+        <v>0</v>
+      </c>
+      <c r="K366" t="n">
+        <v>0</v>
+      </c>
+      <c r="L366" t="n">
+        <v>0</v>
+      </c>
+      <c r="M366" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-07 11:05
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -14637,10 +14637,10 @@
         </is>
       </c>
       <c r="B331" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C331" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D331" t="n">
         <v>0</v>
@@ -14670,7 +14670,7 @@
         <v>0</v>
       </c>
       <c r="M331" t="n">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="332">
@@ -15844,7 +15844,7 @@
         <v>21</v>
       </c>
       <c r="C359" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D359" t="n">
         <v>16</v>
@@ -15874,7 +15874,7 @@
         <v>0</v>
       </c>
       <c r="M359" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="360">
@@ -16142,40 +16142,40 @@
         </is>
       </c>
       <c r="B366" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C366" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D366" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E366" t="n">
         <v>0</v>
       </c>
       <c r="F366" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G366" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H366" t="n">
         <v>0</v>
       </c>
       <c r="I366" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J366" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K366" t="n">
         <v>0</v>
       </c>
       <c r="L366" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M366" t="n">
-        <v>1</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-07 13:06
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M366"/>
+  <dimension ref="A1:M367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14468,7 +14468,7 @@
         <v>3</v>
       </c>
       <c r="C327" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D327" t="n">
         <v>0</v>
@@ -14498,7 +14498,7 @@
         <v>0</v>
       </c>
       <c r="M327" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="328">
@@ -14597,7 +14597,7 @@
         <v>26</v>
       </c>
       <c r="C330" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D330" t="n">
         <v>0</v>
@@ -14606,7 +14606,7 @@
         <v>0</v>
       </c>
       <c r="F330" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G330" t="n">
         <v>5</v>
@@ -14627,7 +14627,7 @@
         <v>0</v>
       </c>
       <c r="M330" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="331">
@@ -16176,6 +16176,49 @@
       </c>
       <c r="M366" t="n">
         <v>102</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B367" t="n">
+        <v>0</v>
+      </c>
+      <c r="C367" t="n">
+        <v>0</v>
+      </c>
+      <c r="D367" t="n">
+        <v>0</v>
+      </c>
+      <c r="E367" t="n">
+        <v>0</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0</v>
+      </c>
+      <c r="H367" t="n">
+        <v>0</v>
+      </c>
+      <c r="I367" t="n">
+        <v>0</v>
+      </c>
+      <c r="J367" t="n">
+        <v>1</v>
+      </c>
+      <c r="K367" t="n">
+        <v>0</v>
+      </c>
+      <c r="L367" t="n">
+        <v>0</v>
+      </c>
+      <c r="M367" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-08 15:17
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -14597,7 +14597,7 @@
         <v>26</v>
       </c>
       <c r="C330" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D330" t="n">
         <v>0</v>
@@ -14606,7 +14606,7 @@
         <v>0</v>
       </c>
       <c r="F330" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G330" t="n">
         <v>5</v>
@@ -14627,7 +14627,7 @@
         <v>0</v>
       </c>
       <c r="M330" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="331">
@@ -16185,31 +16185,31 @@
         </is>
       </c>
       <c r="B367" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="C367" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="D367" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E367" t="n">
         <v>0</v>
       </c>
       <c r="F367" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G367" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H367" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I367" t="n">
         <v>0</v>
       </c>
       <c r="J367" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K367" t="n">
         <v>0</v>
@@ -16218,7 +16218,7 @@
         <v>0</v>
       </c>
       <c r="M367" t="n">
-        <v>1</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-09 13:17
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M367"/>
+  <dimension ref="A1:M368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15930,7 +15930,7 @@
         <v>15</v>
       </c>
       <c r="C361" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D361" t="n">
         <v>12</v>
@@ -15960,7 +15960,7 @@
         <v>0</v>
       </c>
       <c r="M361" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="362">
@@ -16219,6 +16219,49 @@
       </c>
       <c r="M367" t="n">
         <v>105</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B368" t="n">
+        <v>11</v>
+      </c>
+      <c r="C368" t="n">
+        <v>37</v>
+      </c>
+      <c r="D368" t="n">
+        <v>33</v>
+      </c>
+      <c r="E368" t="n">
+        <v>0</v>
+      </c>
+      <c r="F368" t="n">
+        <v>28</v>
+      </c>
+      <c r="G368" t="n">
+        <v>43</v>
+      </c>
+      <c r="H368" t="n">
+        <v>0</v>
+      </c>
+      <c r="I368" t="n">
+        <v>0</v>
+      </c>
+      <c r="J368" t="n">
+        <v>0</v>
+      </c>
+      <c r="K368" t="n">
+        <v>0</v>
+      </c>
+      <c r="L368" t="n">
+        <v>1</v>
+      </c>
+      <c r="M368" t="n">
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-13 13:19
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M368"/>
+  <dimension ref="A1:M372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,12 +459,12 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Ashwagandha</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Other</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -5628,10 +5628,10 @@
         <v>0</v>
       </c>
       <c r="I121" t="n">
+        <v>0</v>
+      </c>
+      <c r="J121" t="n">
         <v>2</v>
-      </c>
-      <c r="J121" t="n">
-        <v>0</v>
       </c>
       <c r="K121" t="n">
         <v>0</v>
@@ -5671,10 +5671,10 @@
         <v>0</v>
       </c>
       <c r="I122" t="n">
+        <v>0</v>
+      </c>
+      <c r="J122" t="n">
         <v>2</v>
-      </c>
-      <c r="J122" t="n">
-        <v>0</v>
       </c>
       <c r="K122" t="n">
         <v>0</v>
@@ -6101,10 +6101,10 @@
         <v>0</v>
       </c>
       <c r="I132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K132" t="n">
         <v>0</v>
@@ -6961,10 +6961,10 @@
         <v>0</v>
       </c>
       <c r="I152" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J152" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K152" t="n">
         <v>0</v>
@@ -7133,10 +7133,10 @@
         <v>0</v>
       </c>
       <c r="I156" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" t="n">
         <v>3</v>
-      </c>
-      <c r="J156" t="n">
-        <v>0</v>
       </c>
       <c r="K156" t="n">
         <v>0</v>
@@ -7219,10 +7219,10 @@
         <v>0</v>
       </c>
       <c r="I158" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" t="n">
         <v>4</v>
-      </c>
-      <c r="J158" t="n">
-        <v>0</v>
       </c>
       <c r="K158" t="n">
         <v>0</v>
@@ -7262,10 +7262,10 @@
         <v>0</v>
       </c>
       <c r="I159" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" t="n">
         <v>11</v>
-      </c>
-      <c r="J159" t="n">
-        <v>0</v>
       </c>
       <c r="K159" t="n">
         <v>0</v>
@@ -7305,10 +7305,10 @@
         <v>0</v>
       </c>
       <c r="I160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
         <v>3</v>
-      </c>
-      <c r="J160" t="n">
-        <v>0</v>
       </c>
       <c r="K160" t="n">
         <v>0</v>
@@ -7348,10 +7348,10 @@
         <v>0</v>
       </c>
       <c r="I161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
         <v>6</v>
-      </c>
-      <c r="J161" t="n">
-        <v>0</v>
       </c>
       <c r="K161" t="n">
         <v>0</v>
@@ -7391,10 +7391,10 @@
         <v>0</v>
       </c>
       <c r="I162" t="n">
+        <v>0</v>
+      </c>
+      <c r="J162" t="n">
         <v>4</v>
-      </c>
-      <c r="J162" t="n">
-        <v>0</v>
       </c>
       <c r="K162" t="n">
         <v>0</v>
@@ -7434,10 +7434,10 @@
         <v>0</v>
       </c>
       <c r="I163" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" t="n">
         <v>2</v>
-      </c>
-      <c r="J163" t="n">
-        <v>0</v>
       </c>
       <c r="K163" t="n">
         <v>0</v>
@@ -7477,10 +7477,10 @@
         <v>0</v>
       </c>
       <c r="I164" t="n">
+        <v>0</v>
+      </c>
+      <c r="J164" t="n">
         <v>2</v>
-      </c>
-      <c r="J164" t="n">
-        <v>0</v>
       </c>
       <c r="K164" t="n">
         <v>0</v>
@@ -7563,10 +7563,10 @@
         <v>0</v>
       </c>
       <c r="I166" t="n">
+        <v>0</v>
+      </c>
+      <c r="J166" t="n">
         <v>6</v>
-      </c>
-      <c r="J166" t="n">
-        <v>0</v>
       </c>
       <c r="K166" t="n">
         <v>0</v>
@@ -7606,10 +7606,10 @@
         <v>0</v>
       </c>
       <c r="I167" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K167" t="n">
         <v>0</v>
@@ -7649,10 +7649,10 @@
         <v>0</v>
       </c>
       <c r="I168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K168" t="n">
         <v>0</v>
@@ -7692,10 +7692,10 @@
         <v>0</v>
       </c>
       <c r="I169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K169" t="n">
         <v>0</v>
@@ -7735,10 +7735,10 @@
         <v>0</v>
       </c>
       <c r="I170" t="n">
+        <v>0</v>
+      </c>
+      <c r="J170" t="n">
         <v>2</v>
-      </c>
-      <c r="J170" t="n">
-        <v>0</v>
       </c>
       <c r="K170" t="n">
         <v>0</v>
@@ -7778,10 +7778,10 @@
         <v>0</v>
       </c>
       <c r="I171" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" t="n">
         <v>2</v>
-      </c>
-      <c r="J171" t="n">
-        <v>0</v>
       </c>
       <c r="K171" t="n">
         <v>0</v>
@@ -7864,10 +7864,10 @@
         <v>0</v>
       </c>
       <c r="I173" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" t="n">
         <v>2</v>
-      </c>
-      <c r="J173" t="n">
-        <v>0</v>
       </c>
       <c r="K173" t="n">
         <v>0</v>
@@ -7907,10 +7907,10 @@
         <v>0</v>
       </c>
       <c r="I174" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" t="n">
         <v>2</v>
-      </c>
-      <c r="J174" t="n">
-        <v>0</v>
       </c>
       <c r="K174" t="n">
         <v>0</v>
@@ -7993,10 +7993,10 @@
         <v>0</v>
       </c>
       <c r="I176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J176" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K176" t="n">
         <v>0</v>
@@ -8122,10 +8122,10 @@
         <v>0</v>
       </c>
       <c r="I179" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J179" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K179" t="n">
         <v>0</v>
@@ -8337,10 +8337,10 @@
         <v>0</v>
       </c>
       <c r="I184" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J184" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K184" t="n">
         <v>0</v>
@@ -8423,10 +8423,10 @@
         <v>0</v>
       </c>
       <c r="I186" t="n">
+        <v>0</v>
+      </c>
+      <c r="J186" t="n">
         <v>2</v>
-      </c>
-      <c r="J186" t="n">
-        <v>0</v>
       </c>
       <c r="K186" t="n">
         <v>0</v>
@@ -8466,10 +8466,10 @@
         <v>0</v>
       </c>
       <c r="I187" t="n">
+        <v>0</v>
+      </c>
+      <c r="J187" t="n">
         <v>3</v>
-      </c>
-      <c r="J187" t="n">
-        <v>0</v>
       </c>
       <c r="K187" t="n">
         <v>0</v>
@@ -8509,10 +8509,10 @@
         <v>0</v>
       </c>
       <c r="I188" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K188" t="n">
         <v>0</v>
@@ -8638,10 +8638,10 @@
         <v>0</v>
       </c>
       <c r="I191" t="n">
+        <v>0</v>
+      </c>
+      <c r="J191" t="n">
         <v>3</v>
-      </c>
-      <c r="J191" t="n">
-        <v>0</v>
       </c>
       <c r="K191" t="n">
         <v>0</v>
@@ -8724,10 +8724,10 @@
         <v>0</v>
       </c>
       <c r="I193" t="n">
+        <v>0</v>
+      </c>
+      <c r="J193" t="n">
         <v>2</v>
-      </c>
-      <c r="J193" t="n">
-        <v>0</v>
       </c>
       <c r="K193" t="n">
         <v>0</v>
@@ -9154,10 +9154,10 @@
         <v>0</v>
       </c>
       <c r="I203" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J203" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K203" t="n">
         <v>0</v>
@@ -9240,10 +9240,10 @@
         <v>0</v>
       </c>
       <c r="I205" t="n">
+        <v>0</v>
+      </c>
+      <c r="J205" t="n">
         <v>2</v>
-      </c>
-      <c r="J205" t="n">
-        <v>0</v>
       </c>
       <c r="K205" t="n">
         <v>0</v>
@@ -9283,10 +9283,10 @@
         <v>0</v>
       </c>
       <c r="I206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J206" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K206" t="n">
         <v>0</v>
@@ -9541,10 +9541,10 @@
         <v>0</v>
       </c>
       <c r="I212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K212" t="n">
         <v>0</v>
@@ -9756,10 +9756,10 @@
         <v>0</v>
       </c>
       <c r="I217" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K217" t="n">
         <v>0</v>
@@ -10272,10 +10272,10 @@
         <v>0</v>
       </c>
       <c r="I229" t="n">
+        <v>0</v>
+      </c>
+      <c r="J229" t="n">
         <v>2</v>
-      </c>
-      <c r="J229" t="n">
-        <v>0</v>
       </c>
       <c r="K229" t="n">
         <v>0</v>
@@ -10358,10 +10358,10 @@
         <v>0</v>
       </c>
       <c r="I231" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" t="n">
         <v>2</v>
-      </c>
-      <c r="J231" t="n">
-        <v>0</v>
       </c>
       <c r="K231" t="n">
         <v>0</v>
@@ -11003,10 +11003,10 @@
         <v>0</v>
       </c>
       <c r="I246" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K246" t="n">
         <v>0</v>
@@ -11046,10 +11046,10 @@
         <v>0</v>
       </c>
       <c r="I247" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K247" t="n">
         <v>0</v>
@@ -12551,10 +12551,10 @@
         <v>1</v>
       </c>
       <c r="I282" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J282" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K282" t="n">
         <v>2</v>
@@ -14615,10 +14615,10 @@
         <v>2</v>
       </c>
       <c r="I330" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J330" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K330" t="n">
         <v>0</v>
@@ -14658,10 +14658,10 @@
         <v>2</v>
       </c>
       <c r="I331" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J331" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K331" t="n">
         <v>0</v>
@@ -14959,10 +14959,10 @@
         <v>2</v>
       </c>
       <c r="I338" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J338" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K338" t="n">
         <v>0</v>
@@ -15088,10 +15088,10 @@
         <v>0</v>
       </c>
       <c r="I341" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K341" t="n">
         <v>0</v>
@@ -15217,10 +15217,10 @@
         <v>2</v>
       </c>
       <c r="I344" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J344" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K344" t="n">
         <v>0</v>
@@ -15260,10 +15260,10 @@
         <v>9</v>
       </c>
       <c r="I345" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J345" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K345" t="n">
         <v>0</v>
@@ -15303,10 +15303,10 @@
         <v>3</v>
       </c>
       <c r="I346" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J346" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K346" t="n">
         <v>0</v>
@@ -15346,10 +15346,10 @@
         <v>1</v>
       </c>
       <c r="I347" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J347" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K347" t="n">
         <v>0</v>
@@ -15389,10 +15389,10 @@
         <v>1</v>
       </c>
       <c r="I348" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J348" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K348" t="n">
         <v>0</v>
@@ -15432,10 +15432,10 @@
         <v>0</v>
       </c>
       <c r="I349" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J349" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K349" t="n">
         <v>0</v>
@@ -15475,10 +15475,10 @@
         <v>1</v>
       </c>
       <c r="I350" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J350" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K350" t="n">
         <v>0</v>
@@ -15518,10 +15518,10 @@
         <v>8</v>
       </c>
       <c r="I351" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J351" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K351" t="n">
         <v>0</v>
@@ -15604,10 +15604,10 @@
         <v>5</v>
       </c>
       <c r="I353" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J353" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K353" t="n">
         <v>0</v>
@@ -15647,10 +15647,10 @@
         <v>4</v>
       </c>
       <c r="I354" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J354" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K354" t="n">
         <v>0</v>
@@ -15733,10 +15733,10 @@
         <v>2</v>
       </c>
       <c r="I356" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J356" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K356" t="n">
         <v>0</v>
@@ -15819,10 +15819,10 @@
         <v>6</v>
       </c>
       <c r="I358" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J358" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K358" t="n">
         <v>0</v>
@@ -15862,10 +15862,10 @@
         <v>1</v>
       </c>
       <c r="I359" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J359" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K359" t="n">
         <v>0</v>
@@ -15905,10 +15905,10 @@
         <v>0</v>
       </c>
       <c r="I360" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J360" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K360" t="n">
         <v>0</v>
@@ -15948,10 +15948,10 @@
         <v>0</v>
       </c>
       <c r="I361" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J361" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K361" t="n">
         <v>0</v>
@@ -15991,10 +15991,10 @@
         <v>0</v>
       </c>
       <c r="I362" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J362" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K362" t="n">
         <v>0</v>
@@ -16034,10 +16034,10 @@
         <v>0</v>
       </c>
       <c r="I363" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J363" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K363" t="n">
         <v>0</v>
@@ -16077,10 +16077,10 @@
         <v>0</v>
       </c>
       <c r="I364" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J364" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K364" t="n">
         <v>0</v>
@@ -16120,10 +16120,10 @@
         <v>0</v>
       </c>
       <c r="I365" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J365" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K365" t="n">
         <v>0</v>
@@ -16163,10 +16163,10 @@
         <v>0</v>
       </c>
       <c r="I366" t="n">
+        <v>4</v>
+      </c>
+      <c r="J366" t="n">
         <v>5</v>
-      </c>
-      <c r="J366" t="n">
-        <v>4</v>
       </c>
       <c r="K366" t="n">
         <v>0</v>
@@ -16206,10 +16206,10 @@
         <v>1</v>
       </c>
       <c r="I367" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J367" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K367" t="n">
         <v>0</v>
@@ -16261,6 +16261,178 @@
         <v>1</v>
       </c>
       <c r="M368" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B369" t="n">
+        <v>26</v>
+      </c>
+      <c r="C369" t="n">
+        <v>37</v>
+      </c>
+      <c r="D369" t="n">
+        <v>27</v>
+      </c>
+      <c r="E369" t="n">
+        <v>0</v>
+      </c>
+      <c r="F369" t="n">
+        <v>34</v>
+      </c>
+      <c r="G369" t="n">
+        <v>43</v>
+      </c>
+      <c r="H369" t="n">
+        <v>0</v>
+      </c>
+      <c r="I369" t="n">
+        <v>36</v>
+      </c>
+      <c r="J369" t="n">
+        <v>0</v>
+      </c>
+      <c r="K369" t="n">
+        <v>0</v>
+      </c>
+      <c r="L369" t="n">
+        <v>1</v>
+      </c>
+      <c r="M369" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B370" t="n">
+        <v>6</v>
+      </c>
+      <c r="C370" t="n">
+        <v>4</v>
+      </c>
+      <c r="D370" t="n">
+        <v>1</v>
+      </c>
+      <c r="E370" t="n">
+        <v>0</v>
+      </c>
+      <c r="F370" t="n">
+        <v>1</v>
+      </c>
+      <c r="G370" t="n">
+        <v>3</v>
+      </c>
+      <c r="H370" t="n">
+        <v>0</v>
+      </c>
+      <c r="I370" t="n">
+        <v>2</v>
+      </c>
+      <c r="J370" t="n">
+        <v>1</v>
+      </c>
+      <c r="K370" t="n">
+        <v>0</v>
+      </c>
+      <c r="L370" t="n">
+        <v>0</v>
+      </c>
+      <c r="M370" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B371" t="n">
+        <v>64</v>
+      </c>
+      <c r="C371" t="n">
+        <v>15</v>
+      </c>
+      <c r="D371" t="n">
+        <v>11</v>
+      </c>
+      <c r="E371" t="n">
+        <v>0</v>
+      </c>
+      <c r="F371" t="n">
+        <v>17</v>
+      </c>
+      <c r="G371" t="n">
+        <v>25</v>
+      </c>
+      <c r="H371" t="n">
+        <v>0</v>
+      </c>
+      <c r="I371" t="n">
+        <v>47</v>
+      </c>
+      <c r="J371" t="n">
+        <v>0</v>
+      </c>
+      <c r="K371" t="n">
+        <v>0</v>
+      </c>
+      <c r="L371" t="n">
+        <v>0</v>
+      </c>
+      <c r="M371" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B372" t="n">
+        <v>30</v>
+      </c>
+      <c r="C372" t="n">
+        <v>13</v>
+      </c>
+      <c r="D372" t="n">
+        <v>13</v>
+      </c>
+      <c r="E372" t="n">
+        <v>0</v>
+      </c>
+      <c r="F372" t="n">
+        <v>8</v>
+      </c>
+      <c r="G372" t="n">
+        <v>16</v>
+      </c>
+      <c r="H372" t="n">
+        <v>0</v>
+      </c>
+      <c r="I372" t="n">
+        <v>73</v>
+      </c>
+      <c r="J372" t="n">
+        <v>0</v>
+      </c>
+      <c r="K372" t="n">
+        <v>0</v>
+      </c>
+      <c r="L372" t="n">
+        <v>0</v>
+      </c>
+      <c r="M372" t="n">
         <v>153</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-15 13:03
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M373"/>
+  <dimension ref="A1:M374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,12 +454,12 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Spearmint</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Other</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -12204,10 +12204,10 @@
         <v>0</v>
       </c>
       <c r="H274" t="n">
+        <v>0</v>
+      </c>
+      <c r="I274" t="n">
         <v>2</v>
-      </c>
-      <c r="I274" t="n">
-        <v>0</v>
       </c>
       <c r="J274" t="n">
         <v>0</v>
@@ -12247,10 +12247,10 @@
         <v>5</v>
       </c>
       <c r="H275" t="n">
+        <v>0</v>
+      </c>
+      <c r="I275" t="n">
         <v>3</v>
-      </c>
-      <c r="I275" t="n">
-        <v>0</v>
       </c>
       <c r="J275" t="n">
         <v>0</v>
@@ -12333,10 +12333,10 @@
         <v>2</v>
       </c>
       <c r="H277" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I277" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J277" t="n">
         <v>0</v>
@@ -12376,10 +12376,10 @@
         <v>0</v>
       </c>
       <c r="H278" t="n">
+        <v>0</v>
+      </c>
+      <c r="I278" t="n">
         <v>2</v>
-      </c>
-      <c r="I278" t="n">
-        <v>0</v>
       </c>
       <c r="J278" t="n">
         <v>0</v>
@@ -12419,10 +12419,10 @@
         <v>1</v>
       </c>
       <c r="H279" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J279" t="n">
         <v>0</v>
@@ -12548,10 +12548,10 @@
         <v>3</v>
       </c>
       <c r="H282" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I282" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J282" t="n">
         <v>1</v>
@@ -12591,10 +12591,10 @@
         <v>1</v>
       </c>
       <c r="H283" t="n">
+        <v>0</v>
+      </c>
+      <c r="I283" t="n">
         <v>2</v>
-      </c>
-      <c r="I283" t="n">
-        <v>0</v>
       </c>
       <c r="J283" t="n">
         <v>0</v>
@@ -12634,10 +12634,10 @@
         <v>7</v>
       </c>
       <c r="H284" t="n">
+        <v>0</v>
+      </c>
+      <c r="I284" t="n">
         <v>6</v>
-      </c>
-      <c r="I284" t="n">
-        <v>0</v>
       </c>
       <c r="J284" t="n">
         <v>0</v>
@@ -12677,10 +12677,10 @@
         <v>4</v>
       </c>
       <c r="H285" t="n">
+        <v>0</v>
+      </c>
+      <c r="I285" t="n">
         <v>4</v>
-      </c>
-      <c r="I285" t="n">
-        <v>0</v>
       </c>
       <c r="J285" t="n">
         <v>0</v>
@@ -12720,10 +12720,10 @@
         <v>1</v>
       </c>
       <c r="H286" t="n">
+        <v>0</v>
+      </c>
+      <c r="I286" t="n">
         <v>3</v>
-      </c>
-      <c r="I286" t="n">
-        <v>0</v>
       </c>
       <c r="J286" t="n">
         <v>0</v>
@@ -12763,10 +12763,10 @@
         <v>1</v>
       </c>
       <c r="H287" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I287" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J287" t="n">
         <v>0</v>
@@ -12806,10 +12806,10 @@
         <v>1</v>
       </c>
       <c r="H288" t="n">
+        <v>0</v>
+      </c>
+      <c r="I288" t="n">
         <v>2</v>
-      </c>
-      <c r="I288" t="n">
-        <v>0</v>
       </c>
       <c r="J288" t="n">
         <v>0</v>
@@ -12849,10 +12849,10 @@
         <v>7</v>
       </c>
       <c r="H289" t="n">
+        <v>0</v>
+      </c>
+      <c r="I289" t="n">
         <v>5</v>
-      </c>
-      <c r="I289" t="n">
-        <v>0</v>
       </c>
       <c r="J289" t="n">
         <v>0</v>
@@ -12892,10 +12892,10 @@
         <v>6</v>
       </c>
       <c r="H290" t="n">
+        <v>0</v>
+      </c>
+      <c r="I290" t="n">
         <v>3</v>
-      </c>
-      <c r="I290" t="n">
-        <v>0</v>
       </c>
       <c r="J290" t="n">
         <v>0</v>
@@ -12935,10 +12935,10 @@
         <v>1</v>
       </c>
       <c r="H291" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I291" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J291" t="n">
         <v>0</v>
@@ -12978,10 +12978,10 @@
         <v>3</v>
       </c>
       <c r="H292" t="n">
+        <v>0</v>
+      </c>
+      <c r="I292" t="n">
         <v>2</v>
-      </c>
-      <c r="I292" t="n">
-        <v>0</v>
       </c>
       <c r="J292" t="n">
         <v>0</v>
@@ -13021,10 +13021,10 @@
         <v>1</v>
       </c>
       <c r="H293" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I293" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J293" t="n">
         <v>0</v>
@@ -13107,10 +13107,10 @@
         <v>10</v>
       </c>
       <c r="H295" t="n">
+        <v>0</v>
+      </c>
+      <c r="I295" t="n">
         <v>6</v>
-      </c>
-      <c r="I295" t="n">
-        <v>0</v>
       </c>
       <c r="J295" t="n">
         <v>0</v>
@@ -13150,10 +13150,10 @@
         <v>8</v>
       </c>
       <c r="H296" t="n">
+        <v>0</v>
+      </c>
+      <c r="I296" t="n">
         <v>9</v>
-      </c>
-      <c r="I296" t="n">
-        <v>0</v>
       </c>
       <c r="J296" t="n">
         <v>0</v>
@@ -13193,10 +13193,10 @@
         <v>2</v>
       </c>
       <c r="H297" t="n">
+        <v>0</v>
+      </c>
+      <c r="I297" t="n">
         <v>3</v>
-      </c>
-      <c r="I297" t="n">
-        <v>0</v>
       </c>
       <c r="J297" t="n">
         <v>0</v>
@@ -13236,10 +13236,10 @@
         <v>2</v>
       </c>
       <c r="H298" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I298" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J298" t="n">
         <v>0</v>
@@ -13279,10 +13279,10 @@
         <v>2</v>
       </c>
       <c r="H299" t="n">
+        <v>0</v>
+      </c>
+      <c r="I299" t="n">
         <v>3</v>
-      </c>
-      <c r="I299" t="n">
-        <v>0</v>
       </c>
       <c r="J299" t="n">
         <v>0</v>
@@ -13408,10 +13408,10 @@
         <v>2</v>
       </c>
       <c r="H302" t="n">
+        <v>0</v>
+      </c>
+      <c r="I302" t="n">
         <v>2</v>
-      </c>
-      <c r="I302" t="n">
-        <v>0</v>
       </c>
       <c r="J302" t="n">
         <v>0</v>
@@ -13451,10 +13451,10 @@
         <v>41</v>
       </c>
       <c r="H303" t="n">
+        <v>0</v>
+      </c>
+      <c r="I303" t="n">
         <v>17</v>
-      </c>
-      <c r="I303" t="n">
-        <v>0</v>
       </c>
       <c r="J303" t="n">
         <v>0</v>
@@ -13494,10 +13494,10 @@
         <v>1</v>
       </c>
       <c r="H304" t="n">
+        <v>0</v>
+      </c>
+      <c r="I304" t="n">
         <v>2</v>
-      </c>
-      <c r="I304" t="n">
-        <v>0</v>
       </c>
       <c r="J304" t="n">
         <v>0</v>
@@ -13537,10 +13537,10 @@
         <v>4</v>
       </c>
       <c r="H305" t="n">
+        <v>0</v>
+      </c>
+      <c r="I305" t="n">
         <v>2</v>
-      </c>
-      <c r="I305" t="n">
-        <v>0</v>
       </c>
       <c r="J305" t="n">
         <v>0</v>
@@ -13580,10 +13580,10 @@
         <v>3</v>
       </c>
       <c r="H306" t="n">
+        <v>0</v>
+      </c>
+      <c r="I306" t="n">
         <v>16</v>
-      </c>
-      <c r="I306" t="n">
-        <v>0</v>
       </c>
       <c r="J306" t="n">
         <v>0</v>
@@ -13623,10 +13623,10 @@
         <v>0</v>
       </c>
       <c r="H307" t="n">
+        <v>0</v>
+      </c>
+      <c r="I307" t="n">
         <v>4</v>
-      </c>
-      <c r="I307" t="n">
-        <v>0</v>
       </c>
       <c r="J307" t="n">
         <v>0</v>
@@ -13666,10 +13666,10 @@
         <v>0</v>
       </c>
       <c r="H308" t="n">
+        <v>0</v>
+      </c>
+      <c r="I308" t="n">
         <v>3</v>
-      </c>
-      <c r="I308" t="n">
-        <v>0</v>
       </c>
       <c r="J308" t="n">
         <v>0</v>
@@ -13709,10 +13709,10 @@
         <v>15</v>
       </c>
       <c r="H309" t="n">
+        <v>0</v>
+      </c>
+      <c r="I309" t="n">
         <v>18</v>
-      </c>
-      <c r="I309" t="n">
-        <v>0</v>
       </c>
       <c r="J309" t="n">
         <v>0</v>
@@ -13752,10 +13752,10 @@
         <v>30</v>
       </c>
       <c r="H310" t="n">
+        <v>0</v>
+      </c>
+      <c r="I310" t="n">
         <v>18</v>
-      </c>
-      <c r="I310" t="n">
-        <v>0</v>
       </c>
       <c r="J310" t="n">
         <v>0</v>
@@ -13795,10 +13795,10 @@
         <v>2</v>
       </c>
       <c r="H311" t="n">
+        <v>0</v>
+      </c>
+      <c r="I311" t="n">
         <v>2</v>
-      </c>
-      <c r="I311" t="n">
-        <v>0</v>
       </c>
       <c r="J311" t="n">
         <v>0</v>
@@ -13838,10 +13838,10 @@
         <v>4</v>
       </c>
       <c r="H312" t="n">
+        <v>0</v>
+      </c>
+      <c r="I312" t="n">
         <v>14</v>
-      </c>
-      <c r="I312" t="n">
-        <v>0</v>
       </c>
       <c r="J312" t="n">
         <v>0</v>
@@ -13881,10 +13881,10 @@
         <v>4</v>
       </c>
       <c r="H313" t="n">
+        <v>0</v>
+      </c>
+      <c r="I313" t="n">
         <v>16</v>
-      </c>
-      <c r="I313" t="n">
-        <v>0</v>
       </c>
       <c r="J313" t="n">
         <v>0</v>
@@ -13924,10 +13924,10 @@
         <v>0</v>
       </c>
       <c r="H314" t="n">
+        <v>0</v>
+      </c>
+      <c r="I314" t="n">
         <v>7</v>
-      </c>
-      <c r="I314" t="n">
-        <v>0</v>
       </c>
       <c r="J314" t="n">
         <v>0</v>
@@ -13967,10 +13967,10 @@
         <v>0</v>
       </c>
       <c r="H315" t="n">
+        <v>0</v>
+      </c>
+      <c r="I315" t="n">
         <v>3</v>
-      </c>
-      <c r="I315" t="n">
-        <v>0</v>
       </c>
       <c r="J315" t="n">
         <v>0</v>
@@ -14010,10 +14010,10 @@
         <v>1</v>
       </c>
       <c r="H316" t="n">
+        <v>0</v>
+      </c>
+      <c r="I316" t="n">
         <v>5</v>
-      </c>
-      <c r="I316" t="n">
-        <v>0</v>
       </c>
       <c r="J316" t="n">
         <v>0</v>
@@ -14053,10 +14053,10 @@
         <v>3</v>
       </c>
       <c r="H317" t="n">
+        <v>0</v>
+      </c>
+      <c r="I317" t="n">
         <v>2</v>
-      </c>
-      <c r="I317" t="n">
-        <v>0</v>
       </c>
       <c r="J317" t="n">
         <v>0</v>
@@ -14139,10 +14139,10 @@
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I319" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J319" t="n">
         <v>0</v>
@@ -14182,10 +14182,10 @@
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I320" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J320" t="n">
         <v>0</v>
@@ -14225,10 +14225,10 @@
         <v>1</v>
       </c>
       <c r="H321" t="n">
+        <v>0</v>
+      </c>
+      <c r="I321" t="n">
         <v>2</v>
-      </c>
-      <c r="I321" t="n">
-        <v>0</v>
       </c>
       <c r="J321" t="n">
         <v>0</v>
@@ -14268,10 +14268,10 @@
         <v>0</v>
       </c>
       <c r="H322" t="n">
+        <v>0</v>
+      </c>
+      <c r="I322" t="n">
         <v>2</v>
-      </c>
-      <c r="I322" t="n">
-        <v>0</v>
       </c>
       <c r="J322" t="n">
         <v>0</v>
@@ -14354,10 +14354,10 @@
         <v>1</v>
       </c>
       <c r="H324" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I324" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J324" t="n">
         <v>0</v>
@@ -14397,10 +14397,10 @@
         <v>1</v>
       </c>
       <c r="H325" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J325" t="n">
         <v>0</v>
@@ -14483,10 +14483,10 @@
         <v>0</v>
       </c>
       <c r="H327" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J327" t="n">
         <v>0</v>
@@ -14526,10 +14526,10 @@
         <v>1</v>
       </c>
       <c r="H328" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I328" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J328" t="n">
         <v>0</v>
@@ -14612,10 +14612,10 @@
         <v>5</v>
       </c>
       <c r="H330" t="n">
+        <v>3</v>
+      </c>
+      <c r="I330" t="n">
         <v>2</v>
-      </c>
-      <c r="I330" t="n">
-        <v>3</v>
       </c>
       <c r="J330" t="n">
         <v>0</v>
@@ -14655,10 +14655,10 @@
         <v>1</v>
       </c>
       <c r="H331" t="n">
+        <v>5</v>
+      </c>
+      <c r="I331" t="n">
         <v>2</v>
-      </c>
-      <c r="I331" t="n">
-        <v>5</v>
       </c>
       <c r="J331" t="n">
         <v>0</v>
@@ -14698,10 +14698,10 @@
         <v>0</v>
       </c>
       <c r="H332" t="n">
+        <v>0</v>
+      </c>
+      <c r="I332" t="n">
         <v>2</v>
-      </c>
-      <c r="I332" t="n">
-        <v>0</v>
       </c>
       <c r="J332" t="n">
         <v>0</v>
@@ -14741,10 +14741,10 @@
         <v>0</v>
       </c>
       <c r="H333" t="n">
+        <v>0</v>
+      </c>
+      <c r="I333" t="n">
         <v>3</v>
-      </c>
-      <c r="I333" t="n">
-        <v>0</v>
       </c>
       <c r="J333" t="n">
         <v>0</v>
@@ -14784,10 +14784,10 @@
         <v>0</v>
       </c>
       <c r="H334" t="n">
+        <v>0</v>
+      </c>
+      <c r="I334" t="n">
         <v>5</v>
-      </c>
-      <c r="I334" t="n">
-        <v>0</v>
       </c>
       <c r="J334" t="n">
         <v>0</v>
@@ -14913,10 +14913,10 @@
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I337" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J337" t="n">
         <v>0</v>
@@ -14956,10 +14956,10 @@
         <v>0</v>
       </c>
       <c r="H338" t="n">
+        <v>1</v>
+      </c>
+      <c r="I338" t="n">
         <v>2</v>
-      </c>
-      <c r="I338" t="n">
-        <v>1</v>
       </c>
       <c r="J338" t="n">
         <v>0</v>
@@ -14999,10 +14999,10 @@
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I339" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J339" t="n">
         <v>0</v>
@@ -15085,10 +15085,10 @@
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J341" t="n">
         <v>0</v>
@@ -15171,10 +15171,10 @@
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I343" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J343" t="n">
         <v>0</v>
@@ -15257,10 +15257,10 @@
         <v>0</v>
       </c>
       <c r="H345" t="n">
+        <v>3</v>
+      </c>
+      <c r="I345" t="n">
         <v>9</v>
-      </c>
-      <c r="I345" t="n">
-        <v>3</v>
       </c>
       <c r="J345" t="n">
         <v>0</v>
@@ -15300,10 +15300,10 @@
         <v>0</v>
       </c>
       <c r="H346" t="n">
+        <v>2</v>
+      </c>
+      <c r="I346" t="n">
         <v>3</v>
-      </c>
-      <c r="I346" t="n">
-        <v>2</v>
       </c>
       <c r="J346" t="n">
         <v>0</v>
@@ -15343,10 +15343,10 @@
         <v>1</v>
       </c>
       <c r="H347" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I347" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J347" t="n">
         <v>0</v>
@@ -15386,10 +15386,10 @@
         <v>5</v>
       </c>
       <c r="H348" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I348" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J348" t="n">
         <v>0</v>
@@ -15429,10 +15429,10 @@
         <v>2</v>
       </c>
       <c r="H349" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I349" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J349" t="n">
         <v>0</v>
@@ -15472,10 +15472,10 @@
         <v>3</v>
       </c>
       <c r="H350" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I350" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
@@ -15515,10 +15515,10 @@
         <v>5</v>
       </c>
       <c r="H351" t="n">
+        <v>2</v>
+      </c>
+      <c r="I351" t="n">
         <v>8</v>
-      </c>
-      <c r="I351" t="n">
-        <v>2</v>
       </c>
       <c r="J351" t="n">
         <v>0</v>
@@ -15558,10 +15558,10 @@
         <v>5</v>
       </c>
       <c r="H352" t="n">
+        <v>0</v>
+      </c>
+      <c r="I352" t="n">
         <v>12</v>
-      </c>
-      <c r="I352" t="n">
-        <v>0</v>
       </c>
       <c r="J352" t="n">
         <v>0</v>
@@ -15601,10 +15601,10 @@
         <v>8</v>
       </c>
       <c r="H353" t="n">
+        <v>3</v>
+      </c>
+      <c r="I353" t="n">
         <v>5</v>
-      </c>
-      <c r="I353" t="n">
-        <v>3</v>
       </c>
       <c r="J353" t="n">
         <v>0</v>
@@ -15644,10 +15644,10 @@
         <v>4</v>
       </c>
       <c r="H354" t="n">
+        <v>3</v>
+      </c>
+      <c r="I354" t="n">
         <v>4</v>
-      </c>
-      <c r="I354" t="n">
-        <v>3</v>
       </c>
       <c r="J354" t="n">
         <v>0</v>
@@ -15687,10 +15687,10 @@
         <v>4</v>
       </c>
       <c r="H355" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I355" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J355" t="n">
         <v>0</v>
@@ -15730,10 +15730,10 @@
         <v>12</v>
       </c>
       <c r="H356" t="n">
+        <v>3</v>
+      </c>
+      <c r="I356" t="n">
         <v>2</v>
-      </c>
-      <c r="I356" t="n">
-        <v>3</v>
       </c>
       <c r="J356" t="n">
         <v>0</v>
@@ -15816,10 +15816,10 @@
         <v>52</v>
       </c>
       <c r="H358" t="n">
+        <v>2</v>
+      </c>
+      <c r="I358" t="n">
         <v>6</v>
-      </c>
-      <c r="I358" t="n">
-        <v>2</v>
       </c>
       <c r="J358" t="n">
         <v>0</v>
@@ -15902,10 +15902,10 @@
         <v>19</v>
       </c>
       <c r="H360" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I360" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J360" t="n">
         <v>0</v>
@@ -15945,10 +15945,10 @@
         <v>26</v>
       </c>
       <c r="H361" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I361" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J361" t="n">
         <v>0</v>
@@ -15988,10 +15988,10 @@
         <v>0</v>
       </c>
       <c r="H362" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I362" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J362" t="n">
         <v>0</v>
@@ -16031,10 +16031,10 @@
         <v>0</v>
       </c>
       <c r="H363" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I363" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J363" t="n">
         <v>0</v>
@@ -16074,10 +16074,10 @@
         <v>10</v>
       </c>
       <c r="H364" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I364" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J364" t="n">
         <v>0</v>
@@ -16117,10 +16117,10 @@
         <v>2</v>
       </c>
       <c r="H365" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I365" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J365" t="n">
         <v>0</v>
@@ -16160,10 +16160,10 @@
         <v>15</v>
       </c>
       <c r="H366" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I366" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J366" t="n">
         <v>5</v>
@@ -16203,10 +16203,10 @@
         <v>19</v>
       </c>
       <c r="H367" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I367" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J367" t="n">
         <v>0</v>
@@ -16289,10 +16289,10 @@
         <v>43</v>
       </c>
       <c r="H369" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I369" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="J369" t="n">
         <v>0</v>
@@ -16332,10 +16332,10 @@
         <v>3</v>
       </c>
       <c r="H370" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I370" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J370" t="n">
         <v>1</v>
@@ -16375,10 +16375,10 @@
         <v>25</v>
       </c>
       <c r="H371" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="I371" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="J371" t="n">
         <v>0</v>
@@ -16418,10 +16418,10 @@
         <v>16</v>
       </c>
       <c r="H372" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="I372" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="J372" t="n">
         <v>0</v>
@@ -16461,10 +16461,10 @@
         <v>7</v>
       </c>
       <c r="H373" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="I373" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="J373" t="n">
         <v>0</v>
@@ -16477,6 +16477,49 @@
       </c>
       <c r="M373" t="n">
         <v>71</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B374" t="n">
+        <v>59</v>
+      </c>
+      <c r="C374" t="n">
+        <v>41</v>
+      </c>
+      <c r="D374" t="n">
+        <v>27</v>
+      </c>
+      <c r="E374" t="n">
+        <v>0</v>
+      </c>
+      <c r="F374" t="n">
+        <v>25</v>
+      </c>
+      <c r="G374" t="n">
+        <v>58</v>
+      </c>
+      <c r="H374" t="n">
+        <v>29</v>
+      </c>
+      <c r="I374" t="n">
+        <v>6</v>
+      </c>
+      <c r="J374" t="n">
+        <v>2</v>
+      </c>
+      <c r="K374" t="n">
+        <v>0</v>
+      </c>
+      <c r="L374" t="n">
+        <v>0</v>
+      </c>
+      <c r="M374" t="n">
+        <v>247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-16 13:02
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M374"/>
+  <dimension ref="A1:M375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,12 +439,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Psyllium Fiber</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Lemon Ginger</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Psyllium Fiber</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -12109,10 +12109,10 @@
         <v>0</v>
       </c>
       <c r="E272" t="n">
+        <v>0</v>
+      </c>
+      <c r="F272" t="n">
         <v>24</v>
-      </c>
-      <c r="F272" t="n">
-        <v>0</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
@@ -12152,10 +12152,10 @@
         <v>0</v>
       </c>
       <c r="E273" t="n">
+        <v>0</v>
+      </c>
+      <c r="F273" t="n">
         <v>30</v>
-      </c>
-      <c r="F273" t="n">
-        <v>0</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -12195,10 +12195,10 @@
         <v>9</v>
       </c>
       <c r="E274" t="n">
+        <v>0</v>
+      </c>
+      <c r="F274" t="n">
         <v>41</v>
-      </c>
-      <c r="F274" t="n">
-        <v>0</v>
       </c>
       <c r="G274" t="n">
         <v>0</v>
@@ -12238,10 +12238,10 @@
         <v>1</v>
       </c>
       <c r="E275" t="n">
+        <v>0</v>
+      </c>
+      <c r="F275" t="n">
         <v>18</v>
-      </c>
-      <c r="F275" t="n">
-        <v>0</v>
       </c>
       <c r="G275" t="n">
         <v>5</v>
@@ -12281,10 +12281,10 @@
         <v>0</v>
       </c>
       <c r="E276" t="n">
+        <v>0</v>
+      </c>
+      <c r="F276" t="n">
         <v>24</v>
-      </c>
-      <c r="F276" t="n">
-        <v>0</v>
       </c>
       <c r="G276" t="n">
         <v>0</v>
@@ -12324,10 +12324,10 @@
         <v>0</v>
       </c>
       <c r="E277" t="n">
+        <v>0</v>
+      </c>
+      <c r="F277" t="n">
         <v>27</v>
-      </c>
-      <c r="F277" t="n">
-        <v>0</v>
       </c>
       <c r="G277" t="n">
         <v>2</v>
@@ -12367,10 +12367,10 @@
         <v>0</v>
       </c>
       <c r="E278" t="n">
+        <v>0</v>
+      </c>
+      <c r="F278" t="n">
         <v>36</v>
-      </c>
-      <c r="F278" t="n">
-        <v>0</v>
       </c>
       <c r="G278" t="n">
         <v>0</v>
@@ -12453,10 +12453,10 @@
         <v>8</v>
       </c>
       <c r="E280" t="n">
+        <v>0</v>
+      </c>
+      <c r="F280" t="n">
         <v>9</v>
-      </c>
-      <c r="F280" t="n">
-        <v>0</v>
       </c>
       <c r="G280" t="n">
         <v>0</v>
@@ -12496,10 +12496,10 @@
         <v>0</v>
       </c>
       <c r="E281" t="n">
+        <v>0</v>
+      </c>
+      <c r="F281" t="n">
         <v>30</v>
-      </c>
-      <c r="F281" t="n">
-        <v>0</v>
       </c>
       <c r="G281" t="n">
         <v>1</v>
@@ -12539,10 +12539,10 @@
         <v>7</v>
       </c>
       <c r="E282" t="n">
+        <v>0</v>
+      </c>
+      <c r="F282" t="n">
         <v>29</v>
-      </c>
-      <c r="F282" t="n">
-        <v>0</v>
       </c>
       <c r="G282" t="n">
         <v>3</v>
@@ -12582,10 +12582,10 @@
         <v>0</v>
       </c>
       <c r="E283" t="n">
+        <v>0</v>
+      </c>
+      <c r="F283" t="n">
         <v>11</v>
-      </c>
-      <c r="F283" t="n">
-        <v>0</v>
       </c>
       <c r="G283" t="n">
         <v>1</v>
@@ -12625,10 +12625,10 @@
         <v>6</v>
       </c>
       <c r="E284" t="n">
+        <v>0</v>
+      </c>
+      <c r="F284" t="n">
         <v>15</v>
-      </c>
-      <c r="F284" t="n">
-        <v>0</v>
       </c>
       <c r="G284" t="n">
         <v>7</v>
@@ -12668,10 +12668,10 @@
         <v>8</v>
       </c>
       <c r="E285" t="n">
+        <v>0</v>
+      </c>
+      <c r="F285" t="n">
         <v>18</v>
-      </c>
-      <c r="F285" t="n">
-        <v>0</v>
       </c>
       <c r="G285" t="n">
         <v>4</v>
@@ -12711,10 +12711,10 @@
         <v>6</v>
       </c>
       <c r="E286" t="n">
+        <v>0</v>
+      </c>
+      <c r="F286" t="n">
         <v>19</v>
-      </c>
-      <c r="F286" t="n">
-        <v>0</v>
       </c>
       <c r="G286" t="n">
         <v>1</v>
@@ -12754,10 +12754,10 @@
         <v>2</v>
       </c>
       <c r="E287" t="n">
+        <v>0</v>
+      </c>
+      <c r="F287" t="n">
         <v>19</v>
-      </c>
-      <c r="F287" t="n">
-        <v>0</v>
       </c>
       <c r="G287" t="n">
         <v>1</v>
@@ -12797,10 +12797,10 @@
         <v>5</v>
       </c>
       <c r="E288" t="n">
+        <v>0</v>
+      </c>
+      <c r="F288" t="n">
         <v>15</v>
-      </c>
-      <c r="F288" t="n">
-        <v>0</v>
       </c>
       <c r="G288" t="n">
         <v>1</v>
@@ -12840,10 +12840,10 @@
         <v>4</v>
       </c>
       <c r="E289" t="n">
+        <v>0</v>
+      </c>
+      <c r="F289" t="n">
         <v>13</v>
-      </c>
-      <c r="F289" t="n">
-        <v>0</v>
       </c>
       <c r="G289" t="n">
         <v>7</v>
@@ -12883,10 +12883,10 @@
         <v>0</v>
       </c>
       <c r="E290" t="n">
+        <v>0</v>
+      </c>
+      <c r="F290" t="n">
         <v>19</v>
-      </c>
-      <c r="F290" t="n">
-        <v>0</v>
       </c>
       <c r="G290" t="n">
         <v>6</v>
@@ -12926,10 +12926,10 @@
         <v>2</v>
       </c>
       <c r="E291" t="n">
+        <v>0</v>
+      </c>
+      <c r="F291" t="n">
         <v>20</v>
-      </c>
-      <c r="F291" t="n">
-        <v>0</v>
       </c>
       <c r="G291" t="n">
         <v>1</v>
@@ -12969,10 +12969,10 @@
         <v>2</v>
       </c>
       <c r="E292" t="n">
+        <v>0</v>
+      </c>
+      <c r="F292" t="n">
         <v>17</v>
-      </c>
-      <c r="F292" t="n">
-        <v>0</v>
       </c>
       <c r="G292" t="n">
         <v>3</v>
@@ -13012,10 +13012,10 @@
         <v>0</v>
       </c>
       <c r="E293" t="n">
+        <v>0</v>
+      </c>
+      <c r="F293" t="n">
         <v>20</v>
-      </c>
-      <c r="F293" t="n">
-        <v>0</v>
       </c>
       <c r="G293" t="n">
         <v>1</v>
@@ -13055,10 +13055,10 @@
         <v>0</v>
       </c>
       <c r="E294" t="n">
+        <v>0</v>
+      </c>
+      <c r="F294" t="n">
         <v>12</v>
-      </c>
-      <c r="F294" t="n">
-        <v>0</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -13098,10 +13098,10 @@
         <v>13</v>
       </c>
       <c r="E295" t="n">
+        <v>0</v>
+      </c>
+      <c r="F295" t="n">
         <v>26</v>
-      </c>
-      <c r="F295" t="n">
-        <v>0</v>
       </c>
       <c r="G295" t="n">
         <v>10</v>
@@ -13141,10 +13141,10 @@
         <v>4</v>
       </c>
       <c r="E296" t="n">
+        <v>0</v>
+      </c>
+      <c r="F296" t="n">
         <v>23</v>
-      </c>
-      <c r="F296" t="n">
-        <v>0</v>
       </c>
       <c r="G296" t="n">
         <v>8</v>
@@ -13184,10 +13184,10 @@
         <v>2</v>
       </c>
       <c r="E297" t="n">
+        <v>0</v>
+      </c>
+      <c r="F297" t="n">
         <v>24</v>
-      </c>
-      <c r="F297" t="n">
-        <v>0</v>
       </c>
       <c r="G297" t="n">
         <v>2</v>
@@ -13227,10 +13227,10 @@
         <v>0</v>
       </c>
       <c r="E298" t="n">
+        <v>0</v>
+      </c>
+      <c r="F298" t="n">
         <v>17</v>
-      </c>
-      <c r="F298" t="n">
-        <v>0</v>
       </c>
       <c r="G298" t="n">
         <v>2</v>
@@ -13270,10 +13270,10 @@
         <v>0</v>
       </c>
       <c r="E299" t="n">
+        <v>0</v>
+      </c>
+      <c r="F299" t="n">
         <v>38</v>
-      </c>
-      <c r="F299" t="n">
-        <v>0</v>
       </c>
       <c r="G299" t="n">
         <v>2</v>
@@ -13313,10 +13313,10 @@
         <v>0</v>
       </c>
       <c r="E300" t="n">
+        <v>0</v>
+      </c>
+      <c r="F300" t="n">
         <v>17</v>
-      </c>
-      <c r="F300" t="n">
-        <v>0</v>
       </c>
       <c r="G300" t="n">
         <v>0</v>
@@ -13356,10 +13356,10 @@
         <v>0</v>
       </c>
       <c r="E301" t="n">
+        <v>0</v>
+      </c>
+      <c r="F301" t="n">
         <v>26</v>
-      </c>
-      <c r="F301" t="n">
-        <v>0</v>
       </c>
       <c r="G301" t="n">
         <v>0</v>
@@ -13399,10 +13399,10 @@
         <v>0</v>
       </c>
       <c r="E302" t="n">
+        <v>0</v>
+      </c>
+      <c r="F302" t="n">
         <v>22</v>
-      </c>
-      <c r="F302" t="n">
-        <v>0</v>
       </c>
       <c r="G302" t="n">
         <v>2</v>
@@ -13442,10 +13442,10 @@
         <v>20</v>
       </c>
       <c r="E303" t="n">
+        <v>0</v>
+      </c>
+      <c r="F303" t="n">
         <v>15</v>
-      </c>
-      <c r="F303" t="n">
-        <v>0</v>
       </c>
       <c r="G303" t="n">
         <v>41</v>
@@ -13485,10 +13485,10 @@
         <v>1</v>
       </c>
       <c r="E304" t="n">
+        <v>0</v>
+      </c>
+      <c r="F304" t="n">
         <v>21</v>
-      </c>
-      <c r="F304" t="n">
-        <v>0</v>
       </c>
       <c r="G304" t="n">
         <v>1</v>
@@ -13528,10 +13528,10 @@
         <v>2</v>
       </c>
       <c r="E305" t="n">
+        <v>1</v>
+      </c>
+      <c r="F305" t="n">
         <v>22</v>
-      </c>
-      <c r="F305" t="n">
-        <v>1</v>
       </c>
       <c r="G305" t="n">
         <v>4</v>
@@ -13614,10 +13614,10 @@
         <v>0</v>
       </c>
       <c r="E307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F307" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G307" t="n">
         <v>0</v>
@@ -13700,10 +13700,10 @@
         <v>0</v>
       </c>
       <c r="E309" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F309" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G309" t="n">
         <v>15</v>
@@ -13743,10 +13743,10 @@
         <v>5</v>
       </c>
       <c r="E310" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F310" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G310" t="n">
         <v>30</v>
@@ -13786,10 +13786,10 @@
         <v>0</v>
       </c>
       <c r="E311" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F311" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G311" t="n">
         <v>2</v>
@@ -13829,10 +13829,10 @@
         <v>0</v>
       </c>
       <c r="E312" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="F312" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="G312" t="n">
         <v>4</v>
@@ -13872,10 +13872,10 @@
         <v>0</v>
       </c>
       <c r="E313" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="F313" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="G313" t="n">
         <v>4</v>
@@ -13915,10 +13915,10 @@
         <v>0</v>
       </c>
       <c r="E314" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="F314" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -13958,10 +13958,10 @@
         <v>0</v>
       </c>
       <c r="E315" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F315" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -14001,10 +14001,10 @@
         <v>1</v>
       </c>
       <c r="E316" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F316" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G316" t="n">
         <v>1</v>
@@ -14044,10 +14044,10 @@
         <v>0</v>
       </c>
       <c r="E317" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F317" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G317" t="n">
         <v>3</v>
@@ -14087,10 +14087,10 @@
         <v>0</v>
       </c>
       <c r="E318" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F318" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="G318" t="n">
         <v>5</v>
@@ -14130,10 +14130,10 @@
         <v>0</v>
       </c>
       <c r="E319" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F319" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
@@ -14173,10 +14173,10 @@
         <v>1</v>
       </c>
       <c r="E320" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F320" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
@@ -14216,10 +14216,10 @@
         <v>0</v>
       </c>
       <c r="E321" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F321" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G321" t="n">
         <v>1</v>
@@ -14259,10 +14259,10 @@
         <v>0</v>
       </c>
       <c r="E322" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F322" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G322" t="n">
         <v>0</v>
@@ -14302,10 +14302,10 @@
         <v>0</v>
       </c>
       <c r="E323" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F323" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G323" t="n">
         <v>0</v>
@@ -14345,10 +14345,10 @@
         <v>1</v>
       </c>
       <c r="E324" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F324" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G324" t="n">
         <v>1</v>
@@ -14388,10 +14388,10 @@
         <v>1</v>
       </c>
       <c r="E325" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F325" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G325" t="n">
         <v>1</v>
@@ -14431,10 +14431,10 @@
         <v>1</v>
       </c>
       <c r="E326" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F326" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G326" t="n">
         <v>3</v>
@@ -14474,10 +14474,10 @@
         <v>0</v>
       </c>
       <c r="E327" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F327" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G327" t="n">
         <v>0</v>
@@ -14517,10 +14517,10 @@
         <v>0</v>
       </c>
       <c r="E328" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F328" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G328" t="n">
         <v>1</v>
@@ -14560,10 +14560,10 @@
         <v>0</v>
       </c>
       <c r="E329" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F329" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G329" t="n">
         <v>0</v>
@@ -14603,10 +14603,10 @@
         <v>0</v>
       </c>
       <c r="E330" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F330" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G330" t="n">
         <v>5</v>
@@ -14646,10 +14646,10 @@
         <v>0</v>
       </c>
       <c r="E331" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G331" t="n">
         <v>1</v>
@@ -14689,10 +14689,10 @@
         <v>0</v>
       </c>
       <c r="E332" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F332" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G332" t="n">
         <v>0</v>
@@ -15850,10 +15850,10 @@
         <v>16</v>
       </c>
       <c r="E359" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F359" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G359" t="n">
         <v>37</v>
@@ -15893,10 +15893,10 @@
         <v>12</v>
       </c>
       <c r="E360" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F360" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G360" t="n">
         <v>19</v>
@@ -15936,10 +15936,10 @@
         <v>12</v>
       </c>
       <c r="E361" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F361" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G361" t="n">
         <v>26</v>
@@ -15979,10 +15979,10 @@
         <v>0</v>
       </c>
       <c r="E362" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F362" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -16022,10 +16022,10 @@
         <v>0</v>
       </c>
       <c r="E363" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F363" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -16065,10 +16065,10 @@
         <v>4</v>
       </c>
       <c r="E364" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F364" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G364" t="n">
         <v>10</v>
@@ -16102,16 +16102,16 @@
         <v>3</v>
       </c>
       <c r="C365" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D365" t="n">
         <v>0</v>
       </c>
       <c r="E365" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F365" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G365" t="n">
         <v>2</v>
@@ -16132,7 +16132,7 @@
         <v>2</v>
       </c>
       <c r="M365" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="366">
@@ -16151,10 +16151,10 @@
         <v>13</v>
       </c>
       <c r="E366" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F366" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G366" t="n">
         <v>15</v>
@@ -16188,16 +16188,16 @@
         <v>21</v>
       </c>
       <c r="C367" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D367" t="n">
         <v>19</v>
       </c>
       <c r="E367" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F367" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G367" t="n">
         <v>19</v>
@@ -16218,7 +16218,7 @@
         <v>0</v>
       </c>
       <c r="M367" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="368">
@@ -16231,16 +16231,16 @@
         <v>11</v>
       </c>
       <c r="C368" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D368" t="n">
         <v>33</v>
       </c>
       <c r="E368" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F368" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="G368" t="n">
         <v>43</v>
@@ -16261,7 +16261,7 @@
         <v>1</v>
       </c>
       <c r="M368" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="369">
@@ -16280,10 +16280,10 @@
         <v>27</v>
       </c>
       <c r="E369" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F369" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="G369" t="n">
         <v>43</v>
@@ -16323,10 +16323,10 @@
         <v>1</v>
       </c>
       <c r="E370" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F370" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G370" t="n">
         <v>3</v>
@@ -16366,10 +16366,10 @@
         <v>11</v>
       </c>
       <c r="E371" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F371" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="G371" t="n">
         <v>25</v>
@@ -16409,10 +16409,10 @@
         <v>13</v>
       </c>
       <c r="E372" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F372" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G372" t="n">
         <v>16</v>
@@ -16452,10 +16452,10 @@
         <v>2</v>
       </c>
       <c r="E373" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F373" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G373" t="n">
         <v>7</v>
@@ -16495,10 +16495,10 @@
         <v>27</v>
       </c>
       <c r="E374" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F374" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G374" t="n">
         <v>58</v>
@@ -16520,6 +16520,49 @@
       </c>
       <c r="M374" t="n">
         <v>247</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B375" t="n">
+        <v>48</v>
+      </c>
+      <c r="C375" t="n">
+        <v>30</v>
+      </c>
+      <c r="D375" t="n">
+        <v>15</v>
+      </c>
+      <c r="E375" t="n">
+        <v>52</v>
+      </c>
+      <c r="F375" t="n">
+        <v>0</v>
+      </c>
+      <c r="G375" t="n">
+        <v>74</v>
+      </c>
+      <c r="H375" t="n">
+        <v>9</v>
+      </c>
+      <c r="I375" t="n">
+        <v>2</v>
+      </c>
+      <c r="J375" t="n">
+        <v>0</v>
+      </c>
+      <c r="K375" t="n">
+        <v>0</v>
+      </c>
+      <c r="L375" t="n">
+        <v>0</v>
+      </c>
+      <c r="M375" t="n">
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-19 13:02
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M375"/>
+  <dimension ref="A1:M378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,12 +444,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Hibiscus</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Lemon Ginger</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Hibiscus</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -12112,10 +12112,10 @@
         <v>0</v>
       </c>
       <c r="F272" t="n">
+        <v>0</v>
+      </c>
+      <c r="G272" t="n">
         <v>24</v>
-      </c>
-      <c r="G272" t="n">
-        <v>0</v>
       </c>
       <c r="H272" t="n">
         <v>0</v>
@@ -12155,10 +12155,10 @@
         <v>0</v>
       </c>
       <c r="F273" t="n">
+        <v>0</v>
+      </c>
+      <c r="G273" t="n">
         <v>30</v>
-      </c>
-      <c r="G273" t="n">
-        <v>0</v>
       </c>
       <c r="H273" t="n">
         <v>0</v>
@@ -12198,10 +12198,10 @@
         <v>0</v>
       </c>
       <c r="F274" t="n">
+        <v>0</v>
+      </c>
+      <c r="G274" t="n">
         <v>41</v>
-      </c>
-      <c r="G274" t="n">
-        <v>0</v>
       </c>
       <c r="H274" t="n">
         <v>0</v>
@@ -12241,10 +12241,10 @@
         <v>0</v>
       </c>
       <c r="F275" t="n">
+        <v>5</v>
+      </c>
+      <c r="G275" t="n">
         <v>18</v>
-      </c>
-      <c r="G275" t="n">
-        <v>5</v>
       </c>
       <c r="H275" t="n">
         <v>0</v>
@@ -12284,10 +12284,10 @@
         <v>0</v>
       </c>
       <c r="F276" t="n">
+        <v>0</v>
+      </c>
+      <c r="G276" t="n">
         <v>24</v>
-      </c>
-      <c r="G276" t="n">
-        <v>0</v>
       </c>
       <c r="H276" t="n">
         <v>0</v>
@@ -12327,10 +12327,10 @@
         <v>0</v>
       </c>
       <c r="F277" t="n">
+        <v>2</v>
+      </c>
+      <c r="G277" t="n">
         <v>27</v>
-      </c>
-      <c r="G277" t="n">
-        <v>2</v>
       </c>
       <c r="H277" t="n">
         <v>0</v>
@@ -12370,10 +12370,10 @@
         <v>0</v>
       </c>
       <c r="F278" t="n">
+        <v>0</v>
+      </c>
+      <c r="G278" t="n">
         <v>36</v>
-      </c>
-      <c r="G278" t="n">
-        <v>0</v>
       </c>
       <c r="H278" t="n">
         <v>0</v>
@@ -12413,10 +12413,10 @@
         <v>0</v>
       </c>
       <c r="F279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G279" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H279" t="n">
         <v>0</v>
@@ -12456,10 +12456,10 @@
         <v>0</v>
       </c>
       <c r="F280" t="n">
+        <v>0</v>
+      </c>
+      <c r="G280" t="n">
         <v>9</v>
-      </c>
-      <c r="G280" t="n">
-        <v>0</v>
       </c>
       <c r="H280" t="n">
         <v>0</v>
@@ -12499,10 +12499,10 @@
         <v>0</v>
       </c>
       <c r="F281" t="n">
+        <v>1</v>
+      </c>
+      <c r="G281" t="n">
         <v>30</v>
-      </c>
-      <c r="G281" t="n">
-        <v>1</v>
       </c>
       <c r="H281" t="n">
         <v>0</v>
@@ -12542,10 +12542,10 @@
         <v>0</v>
       </c>
       <c r="F282" t="n">
+        <v>3</v>
+      </c>
+      <c r="G282" t="n">
         <v>29</v>
-      </c>
-      <c r="G282" t="n">
-        <v>3</v>
       </c>
       <c r="H282" t="n">
         <v>0</v>
@@ -12585,10 +12585,10 @@
         <v>0</v>
       </c>
       <c r="F283" t="n">
+        <v>1</v>
+      </c>
+      <c r="G283" t="n">
         <v>11</v>
-      </c>
-      <c r="G283" t="n">
-        <v>1</v>
       </c>
       <c r="H283" t="n">
         <v>0</v>
@@ -12628,10 +12628,10 @@
         <v>0</v>
       </c>
       <c r="F284" t="n">
+        <v>7</v>
+      </c>
+      <c r="G284" t="n">
         <v>15</v>
-      </c>
-      <c r="G284" t="n">
-        <v>7</v>
       </c>
       <c r="H284" t="n">
         <v>0</v>
@@ -12671,10 +12671,10 @@
         <v>0</v>
       </c>
       <c r="F285" t="n">
+        <v>4</v>
+      </c>
+      <c r="G285" t="n">
         <v>18</v>
-      </c>
-      <c r="G285" t="n">
-        <v>4</v>
       </c>
       <c r="H285" t="n">
         <v>0</v>
@@ -12714,10 +12714,10 @@
         <v>0</v>
       </c>
       <c r="F286" t="n">
+        <v>1</v>
+      </c>
+      <c r="G286" t="n">
         <v>19</v>
-      </c>
-      <c r="G286" t="n">
-        <v>1</v>
       </c>
       <c r="H286" t="n">
         <v>0</v>
@@ -12757,10 +12757,10 @@
         <v>0</v>
       </c>
       <c r="F287" t="n">
+        <v>1</v>
+      </c>
+      <c r="G287" t="n">
         <v>19</v>
-      </c>
-      <c r="G287" t="n">
-        <v>1</v>
       </c>
       <c r="H287" t="n">
         <v>0</v>
@@ -12800,10 +12800,10 @@
         <v>0</v>
       </c>
       <c r="F288" t="n">
+        <v>1</v>
+      </c>
+      <c r="G288" t="n">
         <v>15</v>
-      </c>
-      <c r="G288" t="n">
-        <v>1</v>
       </c>
       <c r="H288" t="n">
         <v>0</v>
@@ -12843,10 +12843,10 @@
         <v>0</v>
       </c>
       <c r="F289" t="n">
+        <v>7</v>
+      </c>
+      <c r="G289" t="n">
         <v>13</v>
-      </c>
-      <c r="G289" t="n">
-        <v>7</v>
       </c>
       <c r="H289" t="n">
         <v>0</v>
@@ -12886,10 +12886,10 @@
         <v>0</v>
       </c>
       <c r="F290" t="n">
+        <v>6</v>
+      </c>
+      <c r="G290" t="n">
         <v>19</v>
-      </c>
-      <c r="G290" t="n">
-        <v>6</v>
       </c>
       <c r="H290" t="n">
         <v>0</v>
@@ -12929,10 +12929,10 @@
         <v>0</v>
       </c>
       <c r="F291" t="n">
+        <v>1</v>
+      </c>
+      <c r="G291" t="n">
         <v>20</v>
-      </c>
-      <c r="G291" t="n">
-        <v>1</v>
       </c>
       <c r="H291" t="n">
         <v>0</v>
@@ -12972,10 +12972,10 @@
         <v>0</v>
       </c>
       <c r="F292" t="n">
+        <v>3</v>
+      </c>
+      <c r="G292" t="n">
         <v>17</v>
-      </c>
-      <c r="G292" t="n">
-        <v>3</v>
       </c>
       <c r="H292" t="n">
         <v>0</v>
@@ -13015,10 +13015,10 @@
         <v>0</v>
       </c>
       <c r="F293" t="n">
+        <v>1</v>
+      </c>
+      <c r="G293" t="n">
         <v>20</v>
-      </c>
-      <c r="G293" t="n">
-        <v>1</v>
       </c>
       <c r="H293" t="n">
         <v>0</v>
@@ -13058,10 +13058,10 @@
         <v>0</v>
       </c>
       <c r="F294" t="n">
+        <v>0</v>
+      </c>
+      <c r="G294" t="n">
         <v>12</v>
-      </c>
-      <c r="G294" t="n">
-        <v>0</v>
       </c>
       <c r="H294" t="n">
         <v>0</v>
@@ -13101,10 +13101,10 @@
         <v>0</v>
       </c>
       <c r="F295" t="n">
+        <v>10</v>
+      </c>
+      <c r="G295" t="n">
         <v>26</v>
-      </c>
-      <c r="G295" t="n">
-        <v>10</v>
       </c>
       <c r="H295" t="n">
         <v>0</v>
@@ -13144,10 +13144,10 @@
         <v>0</v>
       </c>
       <c r="F296" t="n">
+        <v>8</v>
+      </c>
+      <c r="G296" t="n">
         <v>23</v>
-      </c>
-      <c r="G296" t="n">
-        <v>8</v>
       </c>
       <c r="H296" t="n">
         <v>0</v>
@@ -13187,10 +13187,10 @@
         <v>0</v>
       </c>
       <c r="F297" t="n">
+        <v>2</v>
+      </c>
+      <c r="G297" t="n">
         <v>24</v>
-      </c>
-      <c r="G297" t="n">
-        <v>2</v>
       </c>
       <c r="H297" t="n">
         <v>0</v>
@@ -13230,10 +13230,10 @@
         <v>0</v>
       </c>
       <c r="F298" t="n">
+        <v>2</v>
+      </c>
+      <c r="G298" t="n">
         <v>17</v>
-      </c>
-      <c r="G298" t="n">
-        <v>2</v>
       </c>
       <c r="H298" t="n">
         <v>0</v>
@@ -13273,10 +13273,10 @@
         <v>0</v>
       </c>
       <c r="F299" t="n">
+        <v>2</v>
+      </c>
+      <c r="G299" t="n">
         <v>38</v>
-      </c>
-      <c r="G299" t="n">
-        <v>2</v>
       </c>
       <c r="H299" t="n">
         <v>0</v>
@@ -13316,10 +13316,10 @@
         <v>0</v>
       </c>
       <c r="F300" t="n">
+        <v>0</v>
+      </c>
+      <c r="G300" t="n">
         <v>17</v>
-      </c>
-      <c r="G300" t="n">
-        <v>0</v>
       </c>
       <c r="H300" t="n">
         <v>0</v>
@@ -13359,10 +13359,10 @@
         <v>0</v>
       </c>
       <c r="F301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" t="n">
         <v>26</v>
-      </c>
-      <c r="G301" t="n">
-        <v>0</v>
       </c>
       <c r="H301" t="n">
         <v>0</v>
@@ -13402,10 +13402,10 @@
         <v>0</v>
       </c>
       <c r="F302" t="n">
+        <v>2</v>
+      </c>
+      <c r="G302" t="n">
         <v>22</v>
-      </c>
-      <c r="G302" t="n">
-        <v>2</v>
       </c>
       <c r="H302" t="n">
         <v>0</v>
@@ -13445,10 +13445,10 @@
         <v>0</v>
       </c>
       <c r="F303" t="n">
+        <v>41</v>
+      </c>
+      <c r="G303" t="n">
         <v>15</v>
-      </c>
-      <c r="G303" t="n">
-        <v>41</v>
       </c>
       <c r="H303" t="n">
         <v>0</v>
@@ -13488,10 +13488,10 @@
         <v>0</v>
       </c>
       <c r="F304" t="n">
+        <v>1</v>
+      </c>
+      <c r="G304" t="n">
         <v>21</v>
-      </c>
-      <c r="G304" t="n">
-        <v>1</v>
       </c>
       <c r="H304" t="n">
         <v>0</v>
@@ -13531,10 +13531,10 @@
         <v>1</v>
       </c>
       <c r="F305" t="n">
+        <v>4</v>
+      </c>
+      <c r="G305" t="n">
         <v>22</v>
-      </c>
-      <c r="G305" t="n">
-        <v>4</v>
       </c>
       <c r="H305" t="n">
         <v>0</v>
@@ -13574,10 +13574,10 @@
         <v>6</v>
       </c>
       <c r="F306" t="n">
+        <v>3</v>
+      </c>
+      <c r="G306" t="n">
         <v>6</v>
-      </c>
-      <c r="G306" t="n">
-        <v>3</v>
       </c>
       <c r="H306" t="n">
         <v>0</v>
@@ -13703,10 +13703,10 @@
         <v>25</v>
       </c>
       <c r="F309" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G309" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H309" t="n">
         <v>0</v>
@@ -13746,10 +13746,10 @@
         <v>13</v>
       </c>
       <c r="F310" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G310" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H310" t="n">
         <v>0</v>
@@ -13789,10 +13789,10 @@
         <v>3</v>
       </c>
       <c r="F311" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G311" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H311" t="n">
         <v>0</v>
@@ -13832,10 +13832,10 @@
         <v>83</v>
       </c>
       <c r="F312" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G312" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H312" t="n">
         <v>0</v>
@@ -13875,10 +13875,10 @@
         <v>97</v>
       </c>
       <c r="F313" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G313" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H313" t="n">
         <v>0</v>
@@ -14004,10 +14004,10 @@
         <v>25</v>
       </c>
       <c r="F316" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G316" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H316" t="n">
         <v>0</v>
@@ -14047,10 +14047,10 @@
         <v>21</v>
       </c>
       <c r="F317" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G317" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H317" t="n">
         <v>0</v>
@@ -14090,10 +14090,10 @@
         <v>17</v>
       </c>
       <c r="F318" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G318" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H318" t="n">
         <v>0</v>
@@ -14219,10 +14219,10 @@
         <v>10</v>
       </c>
       <c r="F321" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G321" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H321" t="n">
         <v>0</v>
@@ -14348,10 +14348,10 @@
         <v>4</v>
       </c>
       <c r="F324" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G324" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -14391,10 +14391,10 @@
         <v>7</v>
       </c>
       <c r="F325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G325" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H325" t="n">
         <v>0</v>
@@ -14434,10 +14434,10 @@
         <v>10</v>
       </c>
       <c r="F326" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G326" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H326" t="n">
         <v>0</v>
@@ -14520,10 +14520,10 @@
         <v>3</v>
       </c>
       <c r="F328" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G328" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -14606,10 +14606,10 @@
         <v>6</v>
       </c>
       <c r="F330" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G330" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H330" t="n">
         <v>3</v>
@@ -14649,10 +14649,10 @@
         <v>1</v>
       </c>
       <c r="F331" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H331" t="n">
         <v>5</v>
@@ -15337,10 +15337,10 @@
         <v>0</v>
       </c>
       <c r="F347" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G347" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H347" t="n">
         <v>4</v>
@@ -15380,10 +15380,10 @@
         <v>0</v>
       </c>
       <c r="F348" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G348" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H348" t="n">
         <v>6</v>
@@ -15423,10 +15423,10 @@
         <v>0</v>
       </c>
       <c r="F349" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G349" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H349" t="n">
         <v>1</v>
@@ -15466,10 +15466,10 @@
         <v>0</v>
       </c>
       <c r="F350" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G350" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H350" t="n">
         <v>2</v>
@@ -15509,10 +15509,10 @@
         <v>0</v>
       </c>
       <c r="F351" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G351" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H351" t="n">
         <v>2</v>
@@ -15552,10 +15552,10 @@
         <v>0</v>
       </c>
       <c r="F352" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G352" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H352" t="n">
         <v>0</v>
@@ -15595,10 +15595,10 @@
         <v>0</v>
       </c>
       <c r="F353" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G353" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H353" t="n">
         <v>3</v>
@@ -15638,10 +15638,10 @@
         <v>0</v>
       </c>
       <c r="F354" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G354" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H354" t="n">
         <v>3</v>
@@ -15681,10 +15681,10 @@
         <v>0</v>
       </c>
       <c r="F355" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G355" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H355" t="n">
         <v>0</v>
@@ -15724,10 +15724,10 @@
         <v>0</v>
       </c>
       <c r="F356" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G356" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H356" t="n">
         <v>3</v>
@@ -15767,10 +15767,10 @@
         <v>0</v>
       </c>
       <c r="F357" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G357" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H357" t="n">
         <v>0</v>
@@ -15810,10 +15810,10 @@
         <v>0</v>
       </c>
       <c r="F358" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G358" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="H358" t="n">
         <v>2</v>
@@ -15853,10 +15853,10 @@
         <v>4</v>
       </c>
       <c r="F359" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="G359" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H359" t="n">
         <v>1</v>
@@ -15896,10 +15896,10 @@
         <v>10</v>
       </c>
       <c r="F360" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G360" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="H360" t="n">
         <v>2</v>
@@ -15939,10 +15939,10 @@
         <v>13</v>
       </c>
       <c r="F361" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="G361" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H361" t="n">
         <v>3</v>
@@ -16068,10 +16068,10 @@
         <v>4</v>
       </c>
       <c r="F364" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G364" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H364" t="n">
         <v>3</v>
@@ -16111,10 +16111,10 @@
         <v>2</v>
       </c>
       <c r="F365" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G365" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H365" t="n">
         <v>4</v>
@@ -16154,10 +16154,10 @@
         <v>13</v>
       </c>
       <c r="F366" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G366" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H366" t="n">
         <v>4</v>
@@ -16197,10 +16197,10 @@
         <v>20</v>
       </c>
       <c r="F367" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G367" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="H367" t="n">
         <v>2</v>
@@ -16240,10 +16240,10 @@
         <v>28</v>
       </c>
       <c r="F368" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="G368" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="H368" t="n">
         <v>0</v>
@@ -16283,10 +16283,10 @@
         <v>34</v>
       </c>
       <c r="F369" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="G369" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="H369" t="n">
         <v>36</v>
@@ -16326,10 +16326,10 @@
         <v>1</v>
       </c>
       <c r="F370" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G370" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H370" t="n">
         <v>2</v>
@@ -16369,10 +16369,10 @@
         <v>17</v>
       </c>
       <c r="F371" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G371" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H371" t="n">
         <v>47</v>
@@ -16412,10 +16412,10 @@
         <v>8</v>
       </c>
       <c r="F372" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G372" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H372" t="n">
         <v>73</v>
@@ -16455,10 +16455,10 @@
         <v>3</v>
       </c>
       <c r="F373" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G373" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H373" t="n">
         <v>38</v>
@@ -16498,10 +16498,10 @@
         <v>25</v>
       </c>
       <c r="F374" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="G374" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="H374" t="n">
         <v>29</v>
@@ -16541,10 +16541,10 @@
         <v>52</v>
       </c>
       <c r="F375" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="G375" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="H375" t="n">
         <v>9</v>
@@ -16563,6 +16563,135 @@
       </c>
       <c r="M375" t="n">
         <v>230</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B376" t="n">
+        <v>81</v>
+      </c>
+      <c r="C376" t="n">
+        <v>23</v>
+      </c>
+      <c r="D376" t="n">
+        <v>14</v>
+      </c>
+      <c r="E376" t="n">
+        <v>24</v>
+      </c>
+      <c r="F376" t="n">
+        <v>28</v>
+      </c>
+      <c r="G376" t="n">
+        <v>0</v>
+      </c>
+      <c r="H376" t="n">
+        <v>14</v>
+      </c>
+      <c r="I376" t="n">
+        <v>2</v>
+      </c>
+      <c r="J376" t="n">
+        <v>0</v>
+      </c>
+      <c r="K376" t="n">
+        <v>0</v>
+      </c>
+      <c r="L376" t="n">
+        <v>0</v>
+      </c>
+      <c r="M376" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B377" t="n">
+        <v>27</v>
+      </c>
+      <c r="C377" t="n">
+        <v>6</v>
+      </c>
+      <c r="D377" t="n">
+        <v>0</v>
+      </c>
+      <c r="E377" t="n">
+        <v>1</v>
+      </c>
+      <c r="F377" t="n">
+        <v>2</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0</v>
+      </c>
+      <c r="H377" t="n">
+        <v>50</v>
+      </c>
+      <c r="I377" t="n">
+        <v>1</v>
+      </c>
+      <c r="J377" t="n">
+        <v>0</v>
+      </c>
+      <c r="K377" t="n">
+        <v>0</v>
+      </c>
+      <c r="L377" t="n">
+        <v>0</v>
+      </c>
+      <c r="M377" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B378" t="n">
+        <v>89</v>
+      </c>
+      <c r="C378" t="n">
+        <v>27</v>
+      </c>
+      <c r="D378" t="n">
+        <v>16</v>
+      </c>
+      <c r="E378" t="n">
+        <v>16</v>
+      </c>
+      <c r="F378" t="n">
+        <v>28</v>
+      </c>
+      <c r="G378" t="n">
+        <v>0</v>
+      </c>
+      <c r="H378" t="n">
+        <v>130</v>
+      </c>
+      <c r="I378" t="n">
+        <v>4</v>
+      </c>
+      <c r="J378" t="n">
+        <v>1</v>
+      </c>
+      <c r="K378" t="n">
+        <v>0</v>
+      </c>
+      <c r="L378" t="n">
+        <v>0</v>
+      </c>
+      <c r="M378" t="n">
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-19 15:02
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M378"/>
+  <dimension ref="A1:M379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16694,6 +16694,49 @@
         <v>311</v>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B379" t="n">
+        <v>36</v>
+      </c>
+      <c r="C379" t="n">
+        <v>8</v>
+      </c>
+      <c r="D379" t="n">
+        <v>3</v>
+      </c>
+      <c r="E379" t="n">
+        <v>4</v>
+      </c>
+      <c r="F379" t="n">
+        <v>12</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0</v>
+      </c>
+      <c r="H379" t="n">
+        <v>48</v>
+      </c>
+      <c r="I379" t="n">
+        <v>1</v>
+      </c>
+      <c r="J379" t="n">
+        <v>1</v>
+      </c>
+      <c r="K379" t="n">
+        <v>0</v>
+      </c>
+      <c r="L379" t="n">
+        <v>0</v>
+      </c>
+      <c r="M379" t="n">
+        <v>113</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-21 15:03
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M379"/>
+  <dimension ref="A1:M381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16615,7 +16615,7 @@
         </is>
       </c>
       <c r="B377" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C377" t="n">
         <v>6</v>
@@ -16648,7 +16648,7 @@
         <v>0</v>
       </c>
       <c r="M377" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="378">
@@ -16735,6 +16735,92 @@
       </c>
       <c r="M379" t="n">
         <v>281</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>64</v>
+      </c>
+      <c r="C380" t="n">
+        <v>16</v>
+      </c>
+      <c r="D380" t="n">
+        <v>15</v>
+      </c>
+      <c r="E380" t="n">
+        <v>10</v>
+      </c>
+      <c r="F380" t="n">
+        <v>24</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0</v>
+      </c>
+      <c r="H380" t="n">
+        <v>32</v>
+      </c>
+      <c r="I380" t="n">
+        <v>2</v>
+      </c>
+      <c r="J380" t="n">
+        <v>1</v>
+      </c>
+      <c r="K380" t="n">
+        <v>0</v>
+      </c>
+      <c r="L380" t="n">
+        <v>0</v>
+      </c>
+      <c r="M380" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>45</v>
+      </c>
+      <c r="C381" t="n">
+        <v>16</v>
+      </c>
+      <c r="D381" t="n">
+        <v>10</v>
+      </c>
+      <c r="E381" t="n">
+        <v>13</v>
+      </c>
+      <c r="F381" t="n">
+        <v>23</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+      <c r="H381" t="n">
+        <v>13</v>
+      </c>
+      <c r="I381" t="n">
+        <v>5</v>
+      </c>
+      <c r="J381" t="n">
+        <v>2</v>
+      </c>
+      <c r="K381" t="n">
+        <v>0</v>
+      </c>
+      <c r="L381" t="n">
+        <v>0</v>
+      </c>
+      <c r="M381" t="n">
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 12:40
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R377"/>
+  <dimension ref="A1:R381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,12 +444,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Advent Calendar</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Gut Shift</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Advent Calendar</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -16303,10 +16303,10 @@
         <v>0</v>
       </c>
       <c r="F274" t="n">
+        <v>0</v>
+      </c>
+      <c r="G274" t="n">
         <v>3</v>
-      </c>
-      <c r="G274" t="n">
-        <v>0</v>
       </c>
       <c r="H274" t="n">
         <v>0</v>
@@ -16419,10 +16419,10 @@
         <v>1</v>
       </c>
       <c r="F276" t="n">
+        <v>0</v>
+      </c>
+      <c r="G276" t="n">
         <v>2</v>
-      </c>
-      <c r="G276" t="n">
-        <v>0</v>
       </c>
       <c r="H276" t="n">
         <v>0</v>
@@ -16477,10 +16477,10 @@
         <v>8</v>
       </c>
       <c r="F277" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G277" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H277" t="n">
         <v>0</v>
@@ -16593,10 +16593,10 @@
         <v>7</v>
       </c>
       <c r="F279" t="n">
+        <v>0</v>
+      </c>
+      <c r="G279" t="n">
         <v>2</v>
-      </c>
-      <c r="G279" t="n">
-        <v>0</v>
       </c>
       <c r="H279" t="n">
         <v>0</v>
@@ -16651,10 +16651,10 @@
         <v>0</v>
       </c>
       <c r="F280" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H280" t="n">
         <v>0</v>
@@ -16709,10 +16709,10 @@
         <v>6</v>
       </c>
       <c r="F281" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H281" t="n">
         <v>0</v>
@@ -16767,10 +16767,10 @@
         <v>8</v>
       </c>
       <c r="F282" t="n">
+        <v>0</v>
+      </c>
+      <c r="G282" t="n">
         <v>5</v>
-      </c>
-      <c r="G282" t="n">
-        <v>0</v>
       </c>
       <c r="H282" t="n">
         <v>0</v>
@@ -16825,10 +16825,10 @@
         <v>6</v>
       </c>
       <c r="F283" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H283" t="n">
         <v>0</v>
@@ -16883,10 +16883,10 @@
         <v>2</v>
       </c>
       <c r="F284" t="n">
+        <v>0</v>
+      </c>
+      <c r="G284" t="n">
         <v>3</v>
-      </c>
-      <c r="G284" t="n">
-        <v>0</v>
       </c>
       <c r="H284" t="n">
         <v>0</v>
@@ -16941,10 +16941,10 @@
         <v>5</v>
       </c>
       <c r="F285" t="n">
+        <v>0</v>
+      </c>
+      <c r="G285" t="n">
         <v>2</v>
-      </c>
-      <c r="G285" t="n">
-        <v>0</v>
       </c>
       <c r="H285" t="n">
         <v>0</v>
@@ -16999,10 +16999,10 @@
         <v>4</v>
       </c>
       <c r="F286" t="n">
+        <v>0</v>
+      </c>
+      <c r="G286" t="n">
         <v>3</v>
-      </c>
-      <c r="G286" t="n">
-        <v>0</v>
       </c>
       <c r="H286" t="n">
         <v>0</v>
@@ -17057,10 +17057,10 @@
         <v>0</v>
       </c>
       <c r="F287" t="n">
+        <v>0</v>
+      </c>
+      <c r="G287" t="n">
         <v>2</v>
-      </c>
-      <c r="G287" t="n">
-        <v>0</v>
       </c>
       <c r="H287" t="n">
         <v>0</v>
@@ -17115,10 +17115,10 @@
         <v>2</v>
       </c>
       <c r="F288" t="n">
+        <v>0</v>
+      </c>
+      <c r="G288" t="n">
         <v>3</v>
-      </c>
-      <c r="G288" t="n">
-        <v>0</v>
       </c>
       <c r="H288" t="n">
         <v>0</v>
@@ -17173,10 +17173,10 @@
         <v>2</v>
       </c>
       <c r="F289" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G289" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H289" t="n">
         <v>0</v>
@@ -17811,10 +17811,10 @@
         <v>2</v>
       </c>
       <c r="F300" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G300" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H300" t="n">
         <v>0</v>
@@ -17869,10 +17869,10 @@
         <v>3</v>
       </c>
       <c r="F301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" t="n">
         <v>6</v>
-      </c>
-      <c r="G301" t="n">
-        <v>0</v>
       </c>
       <c r="H301" t="n">
         <v>0</v>
@@ -17927,10 +17927,10 @@
         <v>0</v>
       </c>
       <c r="F302" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G302" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H302" t="n">
         <v>0</v>
@@ -18043,10 +18043,10 @@
         <v>0</v>
       </c>
       <c r="F304" t="n">
+        <v>0</v>
+      </c>
+      <c r="G304" t="n">
         <v>25</v>
-      </c>
-      <c r="G304" t="n">
-        <v>0</v>
       </c>
       <c r="H304" t="n">
         <v>0</v>
@@ -18101,10 +18101,10 @@
         <v>5</v>
       </c>
       <c r="F305" t="n">
+        <v>0</v>
+      </c>
+      <c r="G305" t="n">
         <v>13</v>
-      </c>
-      <c r="G305" t="n">
-        <v>0</v>
       </c>
       <c r="H305" t="n">
         <v>0</v>
@@ -18159,10 +18159,10 @@
         <v>0</v>
       </c>
       <c r="F306" t="n">
+        <v>0</v>
+      </c>
+      <c r="G306" t="n">
         <v>3</v>
-      </c>
-      <c r="G306" t="n">
-        <v>0</v>
       </c>
       <c r="H306" t="n">
         <v>0</v>
@@ -18217,10 +18217,10 @@
         <v>0</v>
       </c>
       <c r="F307" t="n">
+        <v>0</v>
+      </c>
+      <c r="G307" t="n">
         <v>83</v>
-      </c>
-      <c r="G307" t="n">
-        <v>0</v>
       </c>
       <c r="H307" t="n">
         <v>0</v>
@@ -18275,10 +18275,10 @@
         <v>0</v>
       </c>
       <c r="F308" t="n">
+        <v>0</v>
+      </c>
+      <c r="G308" t="n">
         <v>97</v>
-      </c>
-      <c r="G308" t="n">
-        <v>0</v>
       </c>
       <c r="H308" t="n">
         <v>0</v>
@@ -18333,10 +18333,10 @@
         <v>0</v>
       </c>
       <c r="F309" t="n">
+        <v>0</v>
+      </c>
+      <c r="G309" t="n">
         <v>102</v>
-      </c>
-      <c r="G309" t="n">
-        <v>0</v>
       </c>
       <c r="H309" t="n">
         <v>0</v>
@@ -18391,10 +18391,10 @@
         <v>0</v>
       </c>
       <c r="F310" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" t="n">
         <v>60</v>
-      </c>
-      <c r="G310" t="n">
-        <v>0</v>
       </c>
       <c r="H310" t="n">
         <v>0</v>
@@ -18449,10 +18449,10 @@
         <v>1</v>
       </c>
       <c r="F311" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" t="n">
         <v>25</v>
-      </c>
-      <c r="G311" t="n">
-        <v>0</v>
       </c>
       <c r="H311" t="n">
         <v>0</v>
@@ -18507,10 +18507,10 @@
         <v>0</v>
       </c>
       <c r="F312" t="n">
+        <v>0</v>
+      </c>
+      <c r="G312" t="n">
         <v>21</v>
-      </c>
-      <c r="G312" t="n">
-        <v>0</v>
       </c>
       <c r="H312" t="n">
         <v>0</v>
@@ -18565,10 +18565,10 @@
         <v>0</v>
       </c>
       <c r="F313" t="n">
+        <v>0</v>
+      </c>
+      <c r="G313" t="n">
         <v>17</v>
-      </c>
-      <c r="G313" t="n">
-        <v>0</v>
       </c>
       <c r="H313" t="n">
         <v>0</v>
@@ -18623,10 +18623,10 @@
         <v>0</v>
       </c>
       <c r="F314" t="n">
+        <v>0</v>
+      </c>
+      <c r="G314" t="n">
         <v>8</v>
-      </c>
-      <c r="G314" t="n">
-        <v>0</v>
       </c>
       <c r="H314" t="n">
         <v>0</v>
@@ -18681,10 +18681,10 @@
         <v>1</v>
       </c>
       <c r="F315" t="n">
+        <v>0</v>
+      </c>
+      <c r="G315" t="n">
         <v>4</v>
-      </c>
-      <c r="G315" t="n">
-        <v>0</v>
       </c>
       <c r="H315" t="n">
         <v>0</v>
@@ -18739,10 +18739,10 @@
         <v>0</v>
       </c>
       <c r="F316" t="n">
+        <v>0</v>
+      </c>
+      <c r="G316" t="n">
         <v>10</v>
-      </c>
-      <c r="G316" t="n">
-        <v>0</v>
       </c>
       <c r="H316" t="n">
         <v>0</v>
@@ -18797,10 +18797,10 @@
         <v>0</v>
       </c>
       <c r="F317" t="n">
+        <v>0</v>
+      </c>
+      <c r="G317" t="n">
         <v>5</v>
-      </c>
-      <c r="G317" t="n">
-        <v>0</v>
       </c>
       <c r="H317" t="n">
         <v>0</v>
@@ -18855,10 +18855,10 @@
         <v>0</v>
       </c>
       <c r="F318" t="n">
+        <v>0</v>
+      </c>
+      <c r="G318" t="n">
         <v>3</v>
-      </c>
-      <c r="G318" t="n">
-        <v>0</v>
       </c>
       <c r="H318" t="n">
         <v>0</v>
@@ -18913,10 +18913,10 @@
         <v>1</v>
       </c>
       <c r="F319" t="n">
+        <v>0</v>
+      </c>
+      <c r="G319" t="n">
         <v>4</v>
-      </c>
-      <c r="G319" t="n">
-        <v>0</v>
       </c>
       <c r="H319" t="n">
         <v>0</v>
@@ -18971,10 +18971,10 @@
         <v>1</v>
       </c>
       <c r="F320" t="n">
+        <v>0</v>
+      </c>
+      <c r="G320" t="n">
         <v>7</v>
-      </c>
-      <c r="G320" t="n">
-        <v>0</v>
       </c>
       <c r="H320" t="n">
         <v>0</v>
@@ -19029,10 +19029,10 @@
         <v>1</v>
       </c>
       <c r="F321" t="n">
+        <v>0</v>
+      </c>
+      <c r="G321" t="n">
         <v>10</v>
-      </c>
-      <c r="G321" t="n">
-        <v>0</v>
       </c>
       <c r="H321" t="n">
         <v>0</v>
@@ -19087,10 +19087,10 @@
         <v>0</v>
       </c>
       <c r="F322" t="n">
+        <v>0</v>
+      </c>
+      <c r="G322" t="n">
         <v>2</v>
-      </c>
-      <c r="G322" t="n">
-        <v>0</v>
       </c>
       <c r="H322" t="n">
         <v>0</v>
@@ -19145,10 +19145,10 @@
         <v>0</v>
       </c>
       <c r="F323" t="n">
+        <v>0</v>
+      </c>
+      <c r="G323" t="n">
         <v>3</v>
-      </c>
-      <c r="G323" t="n">
-        <v>0</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>
@@ -19203,10 +19203,10 @@
         <v>0</v>
       </c>
       <c r="F324" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G324" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -19261,10 +19261,10 @@
         <v>0</v>
       </c>
       <c r="F325" t="n">
+        <v>0</v>
+      </c>
+      <c r="G325" t="n">
         <v>6</v>
-      </c>
-      <c r="G325" t="n">
-        <v>0</v>
       </c>
       <c r="H325" t="n">
         <v>0</v>
@@ -19319,10 +19319,10 @@
         <v>0</v>
       </c>
       <c r="F326" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G326" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H326" t="n">
         <v>0</v>
@@ -19377,10 +19377,10 @@
         <v>0</v>
       </c>
       <c r="F327" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H327" t="n">
         <v>0</v>
@@ -20943,10 +20943,10 @@
         <v>16</v>
       </c>
       <c r="F354" t="n">
+        <v>0</v>
+      </c>
+      <c r="G354" t="n">
         <v>4</v>
-      </c>
-      <c r="G354" t="n">
-        <v>0</v>
       </c>
       <c r="H354" t="n">
         <v>37</v>
@@ -21001,10 +21001,10 @@
         <v>12</v>
       </c>
       <c r="F355" t="n">
+        <v>0</v>
+      </c>
+      <c r="G355" t="n">
         <v>10</v>
-      </c>
-      <c r="G355" t="n">
-        <v>0</v>
       </c>
       <c r="H355" t="n">
         <v>19</v>
@@ -21059,10 +21059,10 @@
         <v>12</v>
       </c>
       <c r="F356" t="n">
+        <v>0</v>
+      </c>
+      <c r="G356" t="n">
         <v>13</v>
-      </c>
-      <c r="G356" t="n">
-        <v>0</v>
       </c>
       <c r="H356" t="n">
         <v>26</v>
@@ -21117,10 +21117,10 @@
         <v>0</v>
       </c>
       <c r="F357" t="n">
+        <v>0</v>
+      </c>
+      <c r="G357" t="n">
         <v>5</v>
-      </c>
-      <c r="G357" t="n">
-        <v>0</v>
       </c>
       <c r="H357" t="n">
         <v>0</v>
@@ -21175,10 +21175,10 @@
         <v>0</v>
       </c>
       <c r="F358" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G358" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H358" t="n">
         <v>0</v>
@@ -21233,10 +21233,10 @@
         <v>4</v>
       </c>
       <c r="F359" t="n">
+        <v>0</v>
+      </c>
+      <c r="G359" t="n">
         <v>4</v>
-      </c>
-      <c r="G359" t="n">
-        <v>0</v>
       </c>
       <c r="H359" t="n">
         <v>10</v>
@@ -21291,10 +21291,10 @@
         <v>0</v>
       </c>
       <c r="F360" t="n">
+        <v>0</v>
+      </c>
+      <c r="G360" t="n">
         <v>2</v>
-      </c>
-      <c r="G360" t="n">
-        <v>0</v>
       </c>
       <c r="H360" t="n">
         <v>2</v>
@@ -21349,10 +21349,10 @@
         <v>13</v>
       </c>
       <c r="F361" t="n">
+        <v>0</v>
+      </c>
+      <c r="G361" t="n">
         <v>13</v>
-      </c>
-      <c r="G361" t="n">
-        <v>0</v>
       </c>
       <c r="H361" t="n">
         <v>14</v>
@@ -21407,10 +21407,10 @@
         <v>19</v>
       </c>
       <c r="F362" t="n">
+        <v>0</v>
+      </c>
+      <c r="G362" t="n">
         <v>20</v>
-      </c>
-      <c r="G362" t="n">
-        <v>0</v>
       </c>
       <c r="H362" t="n">
         <v>18</v>
@@ -21465,10 +21465,10 @@
         <v>33</v>
       </c>
       <c r="F363" t="n">
+        <v>0</v>
+      </c>
+      <c r="G363" t="n">
         <v>28</v>
-      </c>
-      <c r="G363" t="n">
-        <v>0</v>
       </c>
       <c r="H363" t="n">
         <v>39</v>
@@ -21523,10 +21523,10 @@
         <v>26</v>
       </c>
       <c r="F364" t="n">
+        <v>33</v>
+      </c>
+      <c r="G364" t="n">
         <v>34</v>
-      </c>
-      <c r="G364" t="n">
-        <v>33</v>
       </c>
       <c r="H364" t="n">
         <v>38</v>
@@ -21639,10 +21639,10 @@
         <v>11</v>
       </c>
       <c r="F366" t="n">
+        <v>46</v>
+      </c>
+      <c r="G366" t="n">
         <v>17</v>
-      </c>
-      <c r="G366" t="n">
-        <v>46</v>
       </c>
       <c r="H366" t="n">
         <v>22</v>
@@ -21697,10 +21697,10 @@
         <v>13</v>
       </c>
       <c r="F367" t="n">
+        <v>72</v>
+      </c>
+      <c r="G367" t="n">
         <v>8</v>
-      </c>
-      <c r="G367" t="n">
-        <v>72</v>
       </c>
       <c r="H367" t="n">
         <v>15</v>
@@ -21755,10 +21755,10 @@
         <v>2</v>
       </c>
       <c r="F368" t="n">
+        <v>38</v>
+      </c>
+      <c r="G368" t="n">
         <v>3</v>
-      </c>
-      <c r="G368" t="n">
-        <v>38</v>
       </c>
       <c r="H368" t="n">
         <v>5</v>
@@ -21813,10 +21813,10 @@
         <v>26</v>
       </c>
       <c r="F369" t="n">
+        <v>29</v>
+      </c>
+      <c r="G369" t="n">
         <v>25</v>
-      </c>
-      <c r="G369" t="n">
-        <v>29</v>
       </c>
       <c r="H369" t="n">
         <v>56</v>
@@ -21871,10 +21871,10 @@
         <v>15</v>
       </c>
       <c r="F370" t="n">
+        <v>8</v>
+      </c>
+      <c r="G370" t="n">
         <v>52</v>
-      </c>
-      <c r="G370" t="n">
-        <v>8</v>
       </c>
       <c r="H370" t="n">
         <v>72</v>
@@ -21929,10 +21929,10 @@
         <v>14</v>
       </c>
       <c r="F371" t="n">
+        <v>13</v>
+      </c>
+      <c r="G371" t="n">
         <v>24</v>
-      </c>
-      <c r="G371" t="n">
-        <v>13</v>
       </c>
       <c r="H371" t="n">
         <v>26</v>
@@ -21987,10 +21987,10 @@
         <v>0</v>
       </c>
       <c r="F372" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="G372" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="H372" t="n">
         <v>1</v>
@@ -22045,10 +22045,10 @@
         <v>16</v>
       </c>
       <c r="F373" t="n">
+        <v>128</v>
+      </c>
+      <c r="G373" t="n">
         <v>16</v>
-      </c>
-      <c r="G373" t="n">
-        <v>128</v>
       </c>
       <c r="H373" t="n">
         <v>24</v>
@@ -22103,10 +22103,10 @@
         <v>17</v>
       </c>
       <c r="F374" t="n">
+        <v>70</v>
+      </c>
+      <c r="G374" t="n">
         <v>15</v>
-      </c>
-      <c r="G374" t="n">
-        <v>70</v>
       </c>
       <c r="H374" t="n">
         <v>35</v>
@@ -22161,10 +22161,10 @@
         <v>15</v>
       </c>
       <c r="F375" t="n">
+        <v>31</v>
+      </c>
+      <c r="G375" t="n">
         <v>10</v>
-      </c>
-      <c r="G375" t="n">
-        <v>31</v>
       </c>
       <c r="H375" t="n">
         <v>22</v>
@@ -22219,10 +22219,10 @@
         <v>20</v>
       </c>
       <c r="F376" t="n">
+        <v>100</v>
+      </c>
+      <c r="G376" t="n">
         <v>23</v>
-      </c>
-      <c r="G376" t="n">
-        <v>100</v>
       </c>
       <c r="H376" t="n">
         <v>41</v>
@@ -22277,10 +22277,10 @@
         <v>22</v>
       </c>
       <c r="F377" t="n">
+        <v>68</v>
+      </c>
+      <c r="G377" t="n">
         <v>18</v>
-      </c>
-      <c r="G377" t="n">
-        <v>68</v>
       </c>
       <c r="H377" t="n">
         <v>28</v>
@@ -22314,6 +22314,238 @@
       </c>
       <c r="R377" t="n">
         <v>230</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B378" t="n">
+        <v>71</v>
+      </c>
+      <c r="C378" t="n">
+        <v>23</v>
+      </c>
+      <c r="D378" t="n">
+        <v>0</v>
+      </c>
+      <c r="E378" t="n">
+        <v>16</v>
+      </c>
+      <c r="F378" t="n">
+        <v>84</v>
+      </c>
+      <c r="G378" t="n">
+        <v>13</v>
+      </c>
+      <c r="H378" t="n">
+        <v>20</v>
+      </c>
+      <c r="I378" t="n">
+        <v>7</v>
+      </c>
+      <c r="J378" t="n">
+        <v>6</v>
+      </c>
+      <c r="K378" t="n">
+        <v>0</v>
+      </c>
+      <c r="L378" t="n">
+        <v>0</v>
+      </c>
+      <c r="M378" t="n">
+        <v>4</v>
+      </c>
+      <c r="N378" t="n">
+        <v>0</v>
+      </c>
+      <c r="O378" t="n">
+        <v>0</v>
+      </c>
+      <c r="P378" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q378" t="n">
+        <v>0</v>
+      </c>
+      <c r="R378" t="n">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B379" t="n">
+        <v>10</v>
+      </c>
+      <c r="C379" t="n">
+        <v>1</v>
+      </c>
+      <c r="D379" t="n">
+        <v>0</v>
+      </c>
+      <c r="E379" t="n">
+        <v>0</v>
+      </c>
+      <c r="F379" t="n">
+        <v>15</v>
+      </c>
+      <c r="G379" t="n">
+        <v>1</v>
+      </c>
+      <c r="H379" t="n">
+        <v>0</v>
+      </c>
+      <c r="I379" t="n">
+        <v>0</v>
+      </c>
+      <c r="J379" t="n">
+        <v>0</v>
+      </c>
+      <c r="K379" t="n">
+        <v>0</v>
+      </c>
+      <c r="L379" t="n">
+        <v>0</v>
+      </c>
+      <c r="M379" t="n">
+        <v>0</v>
+      </c>
+      <c r="N379" t="n">
+        <v>0</v>
+      </c>
+      <c r="O379" t="n">
+        <v>0</v>
+      </c>
+      <c r="P379" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q379" t="n">
+        <v>0</v>
+      </c>
+      <c r="R379" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>44</v>
+      </c>
+      <c r="C380" t="n">
+        <v>5</v>
+      </c>
+      <c r="D380" t="n">
+        <v>0</v>
+      </c>
+      <c r="E380" t="n">
+        <v>2</v>
+      </c>
+      <c r="F380" t="n">
+        <v>70</v>
+      </c>
+      <c r="G380" t="n">
+        <v>1</v>
+      </c>
+      <c r="H380" t="n">
+        <v>3</v>
+      </c>
+      <c r="I380" t="n">
+        <v>1</v>
+      </c>
+      <c r="J380" t="n">
+        <v>0</v>
+      </c>
+      <c r="K380" t="n">
+        <v>0</v>
+      </c>
+      <c r="L380" t="n">
+        <v>0</v>
+      </c>
+      <c r="M380" t="n">
+        <v>0</v>
+      </c>
+      <c r="N380" t="n">
+        <v>2</v>
+      </c>
+      <c r="O380" t="n">
+        <v>1</v>
+      </c>
+      <c r="P380" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q380" t="n">
+        <v>0</v>
+      </c>
+      <c r="R380" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>0</v>
+      </c>
+      <c r="C381" t="n">
+        <v>0</v>
+      </c>
+      <c r="D381" t="n">
+        <v>0</v>
+      </c>
+      <c r="E381" t="n">
+        <v>0</v>
+      </c>
+      <c r="F381" t="n">
+        <v>0</v>
+      </c>
+      <c r="G381" t="n">
+        <v>1</v>
+      </c>
+      <c r="H381" t="n">
+        <v>0</v>
+      </c>
+      <c r="I381" t="n">
+        <v>0</v>
+      </c>
+      <c r="J381" t="n">
+        <v>0</v>
+      </c>
+      <c r="K381" t="n">
+        <v>0</v>
+      </c>
+      <c r="L381" t="n">
+        <v>0</v>
+      </c>
+      <c r="M381" t="n">
+        <v>0</v>
+      </c>
+      <c r="N381" t="n">
+        <v>0</v>
+      </c>
+      <c r="O381" t="n">
+        <v>0</v>
+      </c>
+      <c r="P381" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q381" t="n">
+        <v>0</v>
+      </c>
+      <c r="R381" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-29 13:54
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="401">
   <si>
     <t>Date</t>
   </si>
@@ -1214,6 +1214,9 @@
   </si>
   <si>
     <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>2026-10-29</t>
   </si>
 </sst>
 </file>
@@ -1571,7 +1574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R383"/>
+  <dimension ref="A1:R384"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -22971,31 +22974,31 @@
         <v>399</v>
       </c>
       <c r="B383">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="C383">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D383">
         <v>0</v>
       </c>
       <c r="E383">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F383">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="G383">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H383">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I383">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J383">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K383">
         <v>0</v>
@@ -23004,7 +23007,7 @@
         <v>0</v>
       </c>
       <c r="M383">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N383">
         <v>0</v>
@@ -23019,7 +23022,63 @@
         <v>0</v>
       </c>
       <c r="R383">
-        <v>6</v>
+        <v>141</v>
+      </c>
+    </row>
+    <row r="384" spans="1:18">
+      <c r="A384" t="s">
+        <v>400</v>
+      </c>
+      <c r="B384">
+        <v>12</v>
+      </c>
+      <c r="C384">
+        <v>0</v>
+      </c>
+      <c r="D384">
+        <v>0</v>
+      </c>
+      <c r="E384">
+        <v>3</v>
+      </c>
+      <c r="F384">
+        <v>86</v>
+      </c>
+      <c r="G384">
+        <v>0</v>
+      </c>
+      <c r="H384">
+        <v>2</v>
+      </c>
+      <c r="I384">
+        <v>4</v>
+      </c>
+      <c r="J384">
+        <v>5</v>
+      </c>
+      <c r="K384">
+        <v>0</v>
+      </c>
+      <c r="L384">
+        <v>1</v>
+      </c>
+      <c r="M384">
+        <v>0</v>
+      </c>
+      <c r="N384">
+        <v>2</v>
+      </c>
+      <c r="O384">
+        <v>0</v>
+      </c>
+      <c r="P384">
+        <v>1</v>
+      </c>
+      <c r="Q384">
+        <v>0</v>
+      </c>
+      <c r="R384">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>